<commit_message>
Simple Flow: spec _4 (V2.6) deliverables regen + state docs — tally 187 (130 Verified / 22 VIU-Pending / 27 Blocked-Env / 5 awaiting-Milos / 3 Deviation / 0 Open-Q)
- Generators: SV map +18=SV-8353, C-R# excluded from bare-R#->Story-16 refs heuristic, assertions 170->187, Story-18 bucket, SUBBUCKET entries for new/reworded/retire-proposed cases
- Regenerated: import CSV/XLSX (187 rows, 0 VIU words, 0 feature-flag words, 4 API sections), Blockers Tracker, TestCases + Results workbooks (id-map 187/187, 0 blanks)
- PROJECT-STATE.md: new §0-BB (V2.6 pass) + WHAT'S-LEFT (retire ruling item 0 + Story-18 re-VIU backlog) + §0 tally table
- CLAUDE.md SF entry: RESUME 2026-07-17 + stale facts fixed (187 in TestRail, SF-QB-09=C29909, Deviations now 3)
- SF-CORE-03 story_ref simplified (refs de-dupe)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_Results.xlsx
+++ b/build/simple-flow/SimpleFlow_Results.xlsx
@@ -166,7 +166,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -176,7 +176,7 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>170</v>
+        <v>187</v>
       </c>
       <c r="C4" s="2" t="n"/>
     </row>
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
@@ -654,7 +654,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
@@ -684,7 +684,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>170</v>
+        <v>187</v>
       </c>
       <c r="C12" s="2" t="n"/>
     </row>
@@ -706,7 +706,7 @@
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>Current headline tally (2026-07-13): VIU-Verified 134 / VIU-Pending 0 / Open-Question 1 / Pending-Retest 0 = 170. Pending-Retest = the V2.4 Δ1-Δ4 cases (expected changed 2026-07-13) awaiting a live re-VIU. DEV-NOT-BUILT is 0.</t>
+          <t>Current headline tally (2026-07-13): VIU-Verified 130 / VIU-Pending 22 / Open-Question 0 / Pending-Retest 0 = 187. Pending-Retest = the V2.4 Δ1-Δ4 cases (expected changed 2026-07-13) awaiting a live re-VIU. DEV-NOT-BUILT is 0.</t>
         </is>
       </c>
       <c r="B14" s="2" t="n"/>
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>169</v>
+        <v>187</v>
       </c>
       <c r="C17" s="2" t="n"/>
     </row>
@@ -743,12 +743,12 @@
           <t>Cases with NO TestRail ID (blank)</t>
         </is>
       </c>
-      <c r="B18" s="9" t="n">
-        <v>1</v>
+      <c r="B18" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Blank: SF-QB-09 — add after the next TestRail sync (IDs not guessed).</t>
+          <t>All authored cases have a TestRail ID (C&lt;id&gt;) + view link.</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
@@ -844,7 +844,7 @@
         </is>
       </c>
       <c r="B26" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="B27" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
@@ -874,7 +874,7 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>170</v>
+        <v>187</v>
       </c>
       <c r="C28" s="2" t="n"/>
     </row>
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="B32" s="6" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
@@ -931,7 +931,7 @@
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="C35" s="2" t="n"/>
     </row>
@@ -1068,7 +1068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I135"/>
+  <dimension ref="A1:I131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="I24" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: surface labels re-confirmed live this run; behavior verified in documented prior VIU drives — optional-invoice wizard actions Cancel / Complete Without Receiving / Receive Parts + 'N parts waiting to receive' (FV-comp13-receivestep.png, 2026-07-10). | Δ core-block caveat added 2026-07-14 (design #4): when a waiting part is a special-order core, Complete Without Receiving is disabled until received (see SF-CORE-03). The base actions Cancel / Complete Without Receiving / Receive Parts for a normal part-bearing WO remain VIU-Verified; the core-waiting disabled state is design-sourced and Blocked-Env (special-order core not seedable).</t>
+          <t>Wording+VIU 2026-07-13: surface labels re-confirmed live this run; behavior verified in documented prior VIU drives — optional-invoice wizard actions Cancel / Complete Without Receiving / Receive Parts + 'N parts waiting to receive' (FV-comp13-receivestep.png, 2026-07-10). | Core caveat RE-ALIGNED 2026-07-17 to spec `_4` (V2.6) Story 18 C-R1/C-R4: the 2026-07-14 design-#4 'disabled until the core is received' caveat is superseded — a Resolve cores screen precedes the choice and only an UNDECIDED core blocks. Base actions remain VIU-Verified; the core leg is spec-sourced and stays Blocked-Env (special-order core not seedable; SV-8353 build likely not deployed).</t>
         </is>
       </c>
     </row>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="I27" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: surface labels re-confirmed live this run; behavior verified in documented prior VIU drives — Complete Without Receiving completes WO, unreceived parts stay waiting, line keeps Receive (2026-07-08/10). | Δ core-block caveat added 2026-07-14 (design #4): Complete Without Receiving is not available while a special-order core is waiting (core must be received first). Base behavior (non-core unreceived parts) remains VIU-Verified.</t>
+          <t>Wording+VIU 2026-07-13: surface labels re-confirmed live this run; behavior verified in documented prior VIU drives — Complete Without Receiving completes WO, unreceived parts stay waiting, line keeps Receive (2026-07-08/10). | Core caveat RE-ALIGNED 2026-07-17 to spec `_4` (V2.6) Story 18 C-R1/C-R4: the 2026-07-14 design-#4 'not available while a core waits' caveat is superseded — only an UNDECIDED core blocks; a decided core completes without receiving. Base behavior (non-core unreceived parts) remains VIU-Verified; the core leg stays Blocked-Env.</t>
         </is>
       </c>
     </row>
@@ -4375,17 +4375,17 @@
     <row r="71">
       <c r="A71" s="12" t="inlineStr">
         <is>
-          <t>C29355</t>
+          <t>C29356</t>
         </is>
       </c>
       <c r="B71" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29355</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29356</t>
         </is>
       </c>
       <c r="C71" s="12" t="inlineStr">
         <is>
-          <t>SF-BULK-06</t>
+          <t>SF-BULK-07</t>
         </is>
       </c>
       <c r="D71" s="12" t="inlineStr">
@@ -4395,7 +4395,7 @@
       </c>
       <c r="E71" s="12" t="inlineStr">
         <is>
-          <t>Verify field editability and locking on Bulk Receive (qty and cost editable; sell locks after WO invoiced/paid)</t>
+          <t>Verify assigning a vendor to a Vendor Missing PO moves it into that vendor's group and entering the missing PN enables receiving</t>
         </is>
       </c>
       <c r="F71" s="12" t="inlineStr">
@@ -4422,17 +4422,17 @@
     <row r="72">
       <c r="A72" s="12" t="inlineStr">
         <is>
-          <t>C29356</t>
+          <t>C29357</t>
         </is>
       </c>
       <c r="B72" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29356</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29357</t>
         </is>
       </c>
       <c r="C72" s="12" t="inlineStr">
         <is>
-          <t>SF-BULK-07</t>
+          <t>SF-BULK-08</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr">
@@ -4442,7 +4442,7 @@
       </c>
       <c r="E72" s="12" t="inlineStr">
         <is>
-          <t>Verify assigning a vendor to a Vendor Missing PO moves it into that vendor's group and entering the missing PN enables receiving</t>
+          <t>Verify Receive All receives everything selected at once and supports partial receive</t>
         </is>
       </c>
       <c r="F72" s="12" t="inlineStr">
@@ -4469,17 +4469,17 @@
     <row r="73">
       <c r="A73" s="12" t="inlineStr">
         <is>
-          <t>C29357</t>
+          <t>C29358</t>
         </is>
       </c>
       <c r="B73" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29357</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29358</t>
         </is>
       </c>
       <c r="C73" s="12" t="inlineStr">
         <is>
-          <t>SF-BULK-08</t>
+          <t>SF-BULK-09</t>
         </is>
       </c>
       <c r="D73" s="12" t="inlineStr">
@@ -4489,7 +4489,7 @@
       </c>
       <c r="E73" s="12" t="inlineStr">
         <is>
-          <t>Verify Receive All receives everything selected at once and supports partial receive</t>
+          <t>Verify Bulk Receive uses the same pipeline as single-PO receive (Delivery → Vendor Bill → QuickBooks)</t>
         </is>
       </c>
       <c r="F73" s="12" t="inlineStr">
@@ -4509,34 +4509,34 @@
       </c>
       <c r="I73" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: receive surfaces re-confirmed live (RCV-po-list.png / RCV-bulk-receive.png) — PO list 'Purchase Orders'+'Receive'; Bulk Receive 'Receive Vendor Parts'/'Back To Purchase Orders'/vendor groups/'Apply to selected POs'/'Invoice Date'/'Tax'/'Receive All'. Behavior per prior VIU (BATCH 7 / 2026-07-10, FV screenshots). (build labels confirmed match; wording corrected where the build differs.)</t>
+          <t>Wording+VIU 2026-07-13: receive surfaces re-confirmed live (RCV-po-list.png / RCV-bulk-receive.png) — PO list 'Purchase Orders'+'Receive'; Bulk Receive 'Receive Vendor Parts'/'Back To Purchase Orders'/vendor groups/'Apply to selected POs'/'Invoice Date'/'Tax'/'Receive All'. Behavior per prior VIU (BATCH 7 / 2026-07-10, FV screenshots). Bulk Receive uses the same pipeline (creates a Delivery + Vendor Bill via receive-requested-parts) - pipeline confirmed prior. FLAG: the QuickBooks-side vendor-bill/AP internals need a human logged into QuickBooks (no QB read API) - QB half not independently verified.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="12" t="inlineStr">
         <is>
-          <t>C29358</t>
+          <t>C29363</t>
         </is>
       </c>
       <c r="B74" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29358</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29363</t>
         </is>
       </c>
       <c r="C74" s="12" t="inlineStr">
         <is>
-          <t>SF-BULK-09</t>
+          <t>SF-PNFIX-01</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
         <is>
-          <t>PO Bulk Receive Page (Story 8)</t>
+          <t>Inline Part-Number Fix (Story 10)</t>
         </is>
       </c>
       <c r="E74" s="12" t="inlineStr">
         <is>
-          <t>Verify Bulk Receive uses the same pipeline as single-PO receive (Delivery → Vendor Bill → QuickBooks)</t>
+          <t>Verify a no-number part shows 'Missing part number' with Edit → enter → save that persists immediately</t>
         </is>
       </c>
       <c r="F74" s="12" t="inlineStr">
@@ -4556,34 +4556,34 @@
       </c>
       <c r="I74" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: receive surfaces re-confirmed live (RCV-po-list.png / RCV-bulk-receive.png) — PO list 'Purchase Orders'+'Receive'; Bulk Receive 'Receive Vendor Parts'/'Back To Purchase Orders'/vendor groups/'Apply to selected POs'/'Invoice Date'/'Tax'/'Receive All'. Behavior per prior VIU (BATCH 7 / 2026-07-10, FV screenshots). Bulk Receive uses the same pipeline (creates a Delivery + Vendor Bill via receive-requested-parts) - pipeline confirmed prior. FLAG: the QuickBooks-side vendor-bill/AP internals need a human logged into QuickBooks (no QB read API) - QB half not independently verified.</t>
+          <t>Wording+VIU 2026-07-13: receive surfaces re-confirmed live (RCV-po-list.png / RCV-bulk-receive.png) — PO list 'Purchase Orders'+'Receive'; Bulk Receive 'Receive Vendor Parts'/'Back To Purchase Orders'/vendor groups/'Apply to selected POs'/'Invoice Date'/'Tax'/'Receive All'. Behavior per prior VIU (BATCH 7 / 2026-07-10, FV screenshots). (build labels confirmed match; wording corrected where the build differs.)</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="12" t="inlineStr">
         <is>
-          <t>C29360</t>
+          <t>C29364</t>
         </is>
       </c>
       <c r="B75" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29360</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29364</t>
         </is>
       </c>
       <c r="C75" s="12" t="inlineStr">
         <is>
-          <t>SF-INV-01</t>
+          <t>SF-PNFIX-02</t>
         </is>
       </c>
       <c r="D75" s="12" t="inlineStr">
         <is>
-          <t>Apply Invoice to Selected POs (Story 9)</t>
+          <t>Inline Part-Number Fix (Story 10)</t>
         </is>
       </c>
       <c r="E75" s="12" t="inlineStr">
         <is>
-          <t>Verify each vendor group has an 'Apply to selected POs' control enabled only with an invoice # and ≥1 PO selected</t>
+          <t>Verify a NEW part number can be entered and saved so the part can be received</t>
         </is>
       </c>
       <c r="F75" s="12" t="inlineStr">
@@ -4603,34 +4603,34 @@
       </c>
       <c r="I75" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: receive surfaces re-confirmed live (RCV-po-list.png / RCV-bulk-receive.png) — PO list 'Purchase Orders'+'Receive'; Bulk Receive 'Receive Vendor Parts'/'Back To Purchase Orders'/vendor groups/'Apply to selected POs'/'Invoice Date'/'Tax'/'Receive All'. Behavior per prior VIU (BATCH 7 / 2026-07-10, FV screenshots). (build labels confirmed match; wording corrected where the build differs.)</t>
+          <t>Rescoped 2026-07-14 for the S10-R2 deprecation (spec _3, 2026-07-14, last-update-wins ruling by QA lead): a part-number add is no longer required to create a first-class inventory/catalog part in v1. Remaining assertions VERIFIED live 2026-07-14: entering a NEW part number persists and the part becomes receivable (POST /api/orders/receive-requested-parts 200 on seeded vendor-missing PO S-15849 after entering a NEW PN + cost + sell + invoice). The previously Blocked-Env downstream inventory/catalog/Part-History creation is no longer a v1 requirement, so it is dropped from the expected result.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="12" t="inlineStr">
         <is>
-          <t>C29361</t>
+          <t>C29365</t>
         </is>
       </c>
       <c r="B76" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29361</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29365</t>
         </is>
       </c>
       <c r="C76" s="12" t="inlineStr">
         <is>
-          <t>SF-INV-02</t>
+          <t>SF-PNFIX-03</t>
         </is>
       </c>
       <c r="D76" s="12" t="inlineStr">
         <is>
-          <t>Apply Invoice to Selected POs (Story 9)</t>
+          <t>Inline Part-Number Fix (Story 10)</t>
         </is>
       </c>
       <c r="E76" s="12" t="inlineStr">
         <is>
-          <t>Verify Apply pre-fills one invoice number into only the selected POs of that vendor, still editable per PO</t>
+          <t>Verify an EXISTING part number can be entered so the part can be received, without overwriting the item's description or category</t>
         </is>
       </c>
       <c r="F76" s="12" t="inlineStr">
@@ -4650,39 +4650,39 @@
       </c>
       <c r="I76" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: receive surfaces re-confirmed live (RCV-po-list.png / RCV-bulk-receive.png) — PO list 'Purchase Orders'+'Receive'; Bulk Receive 'Receive Vendor Parts'/'Back To Purchase Orders'/vendor groups/'Apply to selected POs'/'Invoice Date'/'Tax'/'Receive All'. Behavior per prior VIU (BATCH 7 / 2026-07-10, FV screenshots). (build labels confirmed match; wording corrected where the build differs.)</t>
+          <t>Rescoped 2026-07-14 for the S10-R2 deprecation (spec _3, last-update-wins). Verified live 2026-07-14 that entering a part number persists and the part becomes receivable (receive-requested-parts 200). The 'links to the first-class inventory item + updates stock/cost/history' assertion is deprecated (not a v1 requirement) and removed from the expected; the no-overwrite-of-description/category expectation is retained as a data-safety check.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="12" t="inlineStr">
         <is>
-          <t>C29362</t>
+          <t>C29367</t>
         </is>
       </c>
       <c r="B77" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29362</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29367</t>
         </is>
       </c>
       <c r="C77" s="12" t="inlineStr">
         <is>
-          <t>SF-INV-03</t>
+          <t>SF-PNFIX-05</t>
         </is>
       </c>
       <c r="D77" s="12" t="inlineStr">
         <is>
-          <t>Apply Invoice to Selected POs (Story 9)</t>
+          <t>Inline Part-Number Fix (Story 10)</t>
         </is>
       </c>
       <c r="E77" s="12" t="inlineStr">
         <is>
-          <t>Verify Apply Invoice is scoped per vendor, not offered for the vendorless group, and allows a reused invoice number</t>
+          <t>Verify a part cannot be received without a part number, a vendor (for vendor-missing) and a cost / sell price, even on an invoiced/paid WO</t>
         </is>
       </c>
       <c r="F77" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G77" s="14" t="inlineStr">
@@ -4697,24 +4697,24 @@
       </c>
       <c r="I77" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: receive surfaces re-confirmed live (RCV-po-list.png / RCV-bulk-receive.png) — PO list 'Purchase Orders'+'Receive'; Bulk Receive 'Receive Vendor Parts'/'Back To Purchase Orders'/vendor groups/'Apply to selected POs'/'Invoice Date'/'Tax'/'Receive All'. Behavior per prior VIU (BATCH 7 / 2026-07-10, FV screenshots). (build labels confirmed match; wording corrected where the build differs.)</t>
+          <t>VIU-Verified live 2026-07-14 on the Bulk Receive page (/bulk-receive) with a freshly seeded vendor-missing WO PO (S-15845, order 0ee75c5f, part 'Gear oil' no PN/no vendor/cost=sell=0). Receive gates live-confirmed: a part cannot be received without a part number, without a vendor (for a vendor-missing part), or without a cost/sell price (Receive stayed disabled until all present). The 'even on an invoiced/paid WO' clause is consistent with the field-locking behavior (SF-VAL-09: only the SELL field locks after invoiced/paid; the part-number/cost receive gates remain) — the receive gate itself is unconditional. No error surfaced (gate is a disabled affordance, not a toast).</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="12" t="inlineStr">
         <is>
-          <t>C29363</t>
+          <t>C29368</t>
         </is>
       </c>
       <c r="B78" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29363</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29368</t>
         </is>
       </c>
       <c r="C78" s="12" t="inlineStr">
         <is>
-          <t>SF-PNFIX-01</t>
+          <t>SF-PNFIX-06</t>
         </is>
       </c>
       <c r="D78" s="12" t="inlineStr">
@@ -4724,12 +4724,12 @@
       </c>
       <c r="E78" s="12" t="inlineStr">
         <is>
-          <t>Verify a no-number part shows 'Missing part number' with Edit → enter → save that persists immediately</t>
+          <t>Verify the inline part-number save persists and enables receiving</t>
         </is>
       </c>
       <c r="F78" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G78" s="14" t="inlineStr">
@@ -4744,34 +4744,34 @@
       </c>
       <c r="I78" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: receive surfaces re-confirmed live (RCV-po-list.png / RCV-bulk-receive.png) — PO list 'Purchase Orders'+'Receive'; Bulk Receive 'Receive Vendor Parts'/'Back To Purchase Orders'/vendor groups/'Apply to selected POs'/'Invoice Date'/'Tax'/'Receive All'. Behavior per prior VIU (BATCH 7 / 2026-07-10, FV screenshots). (build labels confirmed match; wording corrected where the build differs.)</t>
+          <t>Rescoped 2026-07-14 for the S10-R2 deprecation (spec _3, last-update-wins). Verified live 2026-07-14 that the inline part-number save persists and the part becomes receivable (receive-requested-parts 200). The technical-guardrail assertion that the inline save must drive catalog creation + an inventory stock Part + Part History is deprecated (not a v1 requirement) and removed from the expected. NOTE: spec _3 leaves the Story-10 Acceptance-Criteria bullets and 'Technical guardrails' paragraph still describing first-class-part creation while R2 itself is struck — an internal inconsistency in the doc; flagged for spec cleanup. Applied the strike per the QA-lead last-update-wins ruling.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="12" t="inlineStr">
         <is>
-          <t>C29364</t>
+          <t>C29369</t>
         </is>
       </c>
       <c r="B79" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29364</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29369</t>
         </is>
       </c>
       <c r="C79" s="12" t="inlineStr">
         <is>
-          <t>SF-PNFIX-02</t>
+          <t>SF-RCV-01</t>
         </is>
       </c>
       <c r="D79" s="12" t="inlineStr">
         <is>
-          <t>Inline Part-Number Fix (Story 10)</t>
+          <t>Receive Button on WO POs (Story 11)</t>
         </is>
       </c>
       <c r="E79" s="12" t="inlineStr">
         <is>
-          <t>Verify a NEW part number can be entered and saved so the part can be received</t>
+          <t>Verify a Receive action appears on WO-originated POs in both the PO list and the PO detail card</t>
         </is>
       </c>
       <c r="F79" s="12" t="inlineStr">
@@ -4791,34 +4791,34 @@
       </c>
       <c r="I79" s="12" t="inlineStr">
         <is>
-          <t>Rescoped 2026-07-14 for the S10-R2 deprecation (spec _3, 2026-07-14, last-update-wins ruling by QA lead): a part-number add is no longer required to create a first-class inventory/catalog part in v1. Remaining assertions VERIFIED live 2026-07-14: entering a NEW part number persists and the part becomes receivable (POST /api/orders/receive-requested-parts 200 on seeded vendor-missing PO S-15849 after entering a NEW PN + cost + sell + invoice). The previously Blocked-Env downstream inventory/catalog/Part-History creation is no longer a v1 requirement, so it is dropped from the expected result.</t>
+          <t>Wording+VIU 2026-07-13: receive surfaces re-confirmed live (RCV-po-list.png / RCV-bulk-receive.png) — PO list 'Purchase Orders'+'Receive'; Bulk Receive 'Receive Vendor Parts'/'Back To Purchase Orders'/vendor groups/'Apply to selected POs'/'Invoice Date'/'Tax'/'Receive All'. Behavior per prior VIU (BATCH 7 / 2026-07-10, FV screenshots). (build labels confirmed match; wording corrected where the build differs.)</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="12" t="inlineStr">
         <is>
-          <t>C29365</t>
+          <t>C29370</t>
         </is>
       </c>
       <c r="B80" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29365</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29370</t>
         </is>
       </c>
       <c r="C80" s="12" t="inlineStr">
         <is>
-          <t>SF-PNFIX-03</t>
+          <t>SF-RCV-02</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
         <is>
-          <t>Inline Part-Number Fix (Story 10)</t>
+          <t>Receive Button on WO POs (Story 11)</t>
         </is>
       </c>
       <c r="E80" s="12" t="inlineStr">
         <is>
-          <t>Verify an EXISTING part number can be entered so the part can be received, without overwriting the item's description or category</t>
+          <t>Verify the Receive action opens the shared Accept Delivery surface</t>
         </is>
       </c>
       <c r="F80" s="12" t="inlineStr">
@@ -4838,39 +4838,39 @@
       </c>
       <c r="I80" s="12" t="inlineStr">
         <is>
-          <t>Rescoped 2026-07-14 for the S10-R2 deprecation (spec _3, last-update-wins). Verified live 2026-07-14 that entering a part number persists and the part becomes receivable (receive-requested-parts 200). The 'links to the first-class inventory item + updates stock/cost/history' assertion is deprecated (not a v1 requirement) and removed from the expected; the no-overwrite-of-description/category expectation is retained as a data-safety check.</t>
+          <t>Wording+VIU 2026-07-13: receive surfaces re-confirmed live (RCV-po-list.png / RCV-bulk-receive.png) — PO list 'Purchase Orders'+'Receive'; Bulk Receive 'Receive Vendor Parts'/'Back To Purchase Orders'/vendor groups/'Apply to selected POs'/'Invoice Date'/'Tax'/'Receive All'. Behavior per prior VIU (BATCH 7 / 2026-07-10, FV screenshots). (build labels confirmed match; wording corrected where the build differs.)</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="12" t="inlineStr">
         <is>
-          <t>C29367</t>
+          <t>C29371</t>
         </is>
       </c>
       <c r="B81" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29367</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29371</t>
         </is>
       </c>
       <c r="C81" s="12" t="inlineStr">
         <is>
-          <t>SF-PNFIX-05</t>
+          <t>SF-RCV-03</t>
         </is>
       </c>
       <c r="D81" s="12" t="inlineStr">
         <is>
-          <t>Inline Part-Number Fix (Story 10)</t>
+          <t>Receive Button on WO POs (Story 11)</t>
         </is>
       </c>
       <c r="E81" s="12" t="inlineStr">
         <is>
-          <t>Verify a part cannot be received without a part number, a vendor (for vendor-missing) and a cost / sell price, even on an invoiced/paid WO</t>
+          <t>Verify the Receive action is hidden for office/readonly users and for fulfilled POs</t>
         </is>
       </c>
       <c r="F81" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G81" s="14" t="inlineStr">
@@ -4885,34 +4885,34 @@
       </c>
       <c r="I81" s="12" t="inlineStr">
         <is>
-          <t>VIU-Verified live 2026-07-14 on the Bulk Receive page (/bulk-receive) with a freshly seeded vendor-missing WO PO (S-15845, order 0ee75c5f, part 'Gear oil' no PN/no vendor/cost=sell=0). Receive gates live-confirmed: a part cannot be received without a part number, without a vendor (for a vendor-missing part), or without a cost/sell price (Receive stayed disabled until all present). The 'even on an invoiced/paid WO' clause is consistent with the field-locking behavior (SF-VAL-09: only the SELL field locks after invoiced/paid; the part-number/cost receive gates remain) — the receive gate itself is unconditional. No error surfaced (gate is a disabled affordance, not a toast).</t>
+          <t>Wording+VIU 2026-07-13: receive surfaces re-confirmed live (RCV-po-list.png / RCV-bulk-receive.png) — PO list 'Purchase Orders'+'Receive'; Bulk Receive 'Receive Vendor Parts'/'Back To Purchase Orders'/vendor groups/'Apply to selected POs'/'Invoice Date'/'Tax'/'Receive All'. Behavior per prior VIU (BATCH 7 / 2026-07-10, FV screenshots). (build labels confirmed match; wording corrected where the build differs.)</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="12" t="inlineStr">
         <is>
-          <t>C29368</t>
+          <t>C29372</t>
         </is>
       </c>
       <c r="B82" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29368</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29372</t>
         </is>
       </c>
       <c r="C82" s="12" t="inlineStr">
         <is>
-          <t>SF-PNFIX-06</t>
+          <t>SF-RCV-04</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
         <is>
-          <t>Inline Part-Number Fix (Story 10)</t>
+          <t>Accept Delivery (Story 12)</t>
         </is>
       </c>
       <c r="E82" s="12" t="inlineStr">
         <is>
-          <t>Verify the inline part-number save persists and enables receiving</t>
+          <t>Verify the existing Accept Delivery screen groups by vendor with per-group invoice #, date, tax, note and Receive</t>
         </is>
       </c>
       <c r="F82" s="12" t="inlineStr">
@@ -4932,34 +4932,34 @@
       </c>
       <c r="I82" s="12" t="inlineStr">
         <is>
-          <t>Rescoped 2026-07-14 for the S10-R2 deprecation (spec _3, last-update-wins). Verified live 2026-07-14 that the inline part-number save persists and the part becomes receivable (receive-requested-parts 200). The technical-guardrail assertion that the inline save must drive catalog creation + an inventory stock Part + Part History is deprecated (not a v1 requirement) and removed from the expected. NOTE: spec _3 leaves the Story-10 Acceptance-Criteria bullets and 'Technical guardrails' paragraph still describing first-class-part creation while R2 itself is struck — an internal inconsistency in the doc; flagged for spec cleanup. Applied the strike per the QA-lead last-update-wins ruling.</t>
+          <t>Wording+VIU 2026-07-13: receive surfaces re-confirmed live (RCV-po-list.png / RCV-bulk-receive.png) — PO list 'Purchase Orders'+'Receive'; Bulk Receive 'Receive Vendor Parts'/'Back To Purchase Orders'/vendor groups/'Apply to selected POs'/'Invoice Date'/'Tax'/'Receive All'. Behavior per prior VIU (BATCH 7 / 2026-07-10, FV screenshots). (build labels confirmed match; wording corrected where the build differs.)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="12" t="inlineStr">
         <is>
-          <t>C29369</t>
+          <t>C29374</t>
         </is>
       </c>
       <c r="B83" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29369</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29374</t>
         </is>
       </c>
       <c r="C83" s="12" t="inlineStr">
         <is>
-          <t>SF-RCV-01</t>
+          <t>SF-RCV-06</t>
         </is>
       </c>
       <c r="D83" s="12" t="inlineStr">
         <is>
-          <t>Receive Button on WO POs (Story 11)</t>
+          <t>Accept Delivery (Story 12)</t>
         </is>
       </c>
       <c r="E83" s="12" t="inlineStr">
         <is>
-          <t>Verify a Receive action appears on WO-originated POs in both the PO list and the PO detail card</t>
+          <t>Verify Accept Delivery receive gates: vendor set, part number entered, cost / sell price entered, vendor invoice # captured</t>
         </is>
       </c>
       <c r="F83" s="12" t="inlineStr">
@@ -4979,39 +4979,39 @@
       </c>
       <c r="I83" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: receive surfaces re-confirmed live (RCV-po-list.png / RCV-bulk-receive.png) — PO list 'Purchase Orders'+'Receive'; Bulk Receive 'Receive Vendor Parts'/'Back To Purchase Orders'/vendor groups/'Apply to selected POs'/'Invoice Date'/'Tax'/'Receive All'. Behavior per prior VIU (BATCH 7 / 2026-07-10, FV screenshots). (build labels confirmed match; wording corrected where the build differs.)</t>
+          <t>VIU-Verified live 2026-07-14 on the Bulk Receive page (/bulk-receive) with a freshly seeded vendor-missing WO PO (S-15845, order 0ee75c5f, part 'Gear oil' no PN/no vendor/cost=sell=0). Receive gates confirmed on the Bulk Receive surface (the WO-PO receive surface; the legacy single-PO Accept Delivery path still 500s for WO POs = BUG-11): no vendor -&gt; Receive disabled; vendor set + no part number -&gt; disabled; part number + cost/sell empty -&gt; disabled; all of vendor + part number + cost/sell present -&gt; receivable. The vendor-invoice-number gate is separately proven (SF-BULK-05 / SF-VAL-05: per-PO Receive disabled until an invoice number is entered).</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="12" t="inlineStr">
         <is>
-          <t>C29370</t>
+          <t>C29377</t>
         </is>
       </c>
       <c r="B84" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29370</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29377</t>
         </is>
       </c>
       <c r="C84" s="12" t="inlineStr">
         <is>
-          <t>SF-RCV-02</t>
+          <t>SF-RCV-09</t>
         </is>
       </c>
       <c r="D84" s="12" t="inlineStr">
         <is>
-          <t>Receive Button on WO POs (Story 11)</t>
+          <t>Accept Delivery (Story 12)</t>
         </is>
       </c>
       <c r="E84" s="12" t="inlineStr">
         <is>
-          <t>Verify the Receive action opens the shared Accept Delivery surface</t>
+          <t>Verify a 'received more than ordered' warning appears when received quantity exceeds ordered quantity</t>
         </is>
       </c>
       <c r="F84" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G84" s="14" t="inlineStr">
@@ -5033,27 +5033,27 @@
     <row r="85">
       <c r="A85" s="12" t="inlineStr">
         <is>
-          <t>C29371</t>
+          <t>C29440</t>
         </is>
       </c>
       <c r="B85" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29371</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29440</t>
         </is>
       </c>
       <c r="C85" s="12" t="inlineStr">
         <is>
-          <t>SF-RCV-03</t>
+          <t>SF-RCV-10</t>
         </is>
       </c>
       <c r="D85" s="12" t="inlineStr">
         <is>
-          <t>Receive Button on WO POs (Story 11)</t>
+          <t>Accept Delivery (Story 12)</t>
         </is>
       </c>
       <c r="E85" s="12" t="inlineStr">
         <is>
-          <t>Verify the Receive action is hidden for office/readonly users and for fulfilled POs</t>
+          <t>Verify cost is editable on the Accept Delivery screen when $0 or missing (parity with Bulk Receive)</t>
         </is>
       </c>
       <c r="F85" s="12" t="inlineStr">
@@ -5080,32 +5080,32 @@
     <row r="86">
       <c r="A86" s="12" t="inlineStr">
         <is>
-          <t>C29372</t>
+          <t>C29378</t>
         </is>
       </c>
       <c r="B86" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29372</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29378</t>
         </is>
       </c>
       <c r="C86" s="12" t="inlineStr">
         <is>
-          <t>SF-RCV-04</t>
+          <t>SF-VEND-01</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr">
         <is>
-          <t>Accept Delivery (Story 12)</t>
+          <t>Assign Vendor + Merge (Story 13)</t>
         </is>
       </c>
       <c r="E86" s="12" t="inlineStr">
         <is>
-          <t>Verify the existing Accept Delivery screen groups by vendor with per-group invoice #, date, tax, note and Receive</t>
+          <t>Verify the vendor-missing group provides a vendor dropdown that assigns a vendor at PO level and saves it</t>
         </is>
       </c>
       <c r="F86" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G86" s="14" t="inlineStr">
@@ -5127,32 +5127,32 @@
     <row r="87">
       <c r="A87" s="12" t="inlineStr">
         <is>
-          <t>C29374</t>
+          <t>C29381</t>
         </is>
       </c>
       <c r="B87" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29374</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29381</t>
         </is>
       </c>
       <c r="C87" s="12" t="inlineStr">
         <is>
-          <t>SF-RCV-06</t>
+          <t>SF-VEND-04</t>
         </is>
       </c>
       <c r="D87" s="12" t="inlineStr">
         <is>
-          <t>Accept Delivery (Story 12)</t>
+          <t>Assign Vendor + Merge (Story 13)</t>
         </is>
       </c>
       <c r="E87" s="12" t="inlineStr">
         <is>
-          <t>Verify Accept Delivery receive gates: vendor set, part number entered, cost / sell price entered, vendor invoice # captured</t>
+          <t>Verify assigning a different vendor with no collision auto-assigns and clears the QB flag, and Receive enables only once the part number and cost / sell price are also present</t>
         </is>
       </c>
       <c r="F87" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G87" s="14" t="inlineStr">
@@ -5167,39 +5167,39 @@
       </c>
       <c r="I87" s="12" t="inlineStr">
         <is>
-          <t>VIU-Verified live 2026-07-14 on the Bulk Receive page (/bulk-receive) with a freshly seeded vendor-missing WO PO (S-15845, order 0ee75c5f, part 'Gear oil' no PN/no vendor/cost=sell=0). Receive gates confirmed on the Bulk Receive surface (the WO-PO receive surface; the legacy single-PO Accept Delivery path still 500s for WO POs = BUG-11): no vendor -&gt; Receive disabled; vendor set + no part number -&gt; disabled; part number + cost/sell empty -&gt; disabled; all of vendor + part number + cost/sell present -&gt; receivable. The vendor-invoice-number gate is separately proven (SF-BULK-05 / SF-VAL-05: per-PO Receive disabled until an invoice number is entered).</t>
+          <t>VIU-Verified live 2026-07-14 on the Bulk Receive page (/bulk-receive) with a freshly seeded vendor-missing WO PO (S-15845, order 0ee75c5f, part 'Gear oil' no PN/no vendor/cost=sell=0). Assigning a brand-new vendor (no collision) via select_assign_vendor -&gt; POST /api/orders/{id}/assign-vendor 200 auto-assigned the vendor with NO Merge/Keep-Separate prompt and cleared the vendor-missing (QuickBooks) flag (PO left the Vendor-Missing group into the vendor's group). Receive then became available only once BOTH the part number AND cost/sell were also supplied (Receive stayed disabled with PN alone / cost=sell=0). Confirms Delta3 S13-R5/R6/R7.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="12" t="inlineStr">
         <is>
-          <t>C29377</t>
+          <t>C29442</t>
         </is>
       </c>
       <c r="B88" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29377</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29442</t>
         </is>
       </c>
       <c r="C88" s="12" t="inlineStr">
         <is>
-          <t>SF-RCV-09</t>
+          <t>SF-VEND-06</t>
         </is>
       </c>
       <c r="D88" s="12" t="inlineStr">
         <is>
-          <t>Accept Delivery (Story 12)</t>
+          <t>Assign Vendor + Merge (Story 13)</t>
         </is>
       </c>
       <c r="E88" s="12" t="inlineStr">
         <is>
-          <t>Verify a 'received more than ordered' warning appears when received quantity exceeds ordered quantity</t>
+          <t>Verify a part cannot be received until a missing cost / sell price is entered</t>
         </is>
       </c>
       <c r="F88" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G88" s="14" t="inlineStr">
@@ -5214,39 +5214,39 @@
       </c>
       <c r="I88" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: receive surfaces re-confirmed live (RCV-po-list.png / RCV-bulk-receive.png) — PO list 'Purchase Orders'+'Receive'; Bulk Receive 'Receive Vendor Parts'/'Back To Purchase Orders'/vendor groups/'Apply to selected POs'/'Invoice Date'/'Tax'/'Receive All'. Behavior per prior VIU (BATCH 7 / 2026-07-10, FV screenshots). (build labels confirmed match; wording corrected where the build differs.)</t>
+          <t>VIU-Verified live 2026-07-14 on the Bulk Receive page (/bulk-receive) with a freshly seeded vendor-missing WO PO (S-15845, order 0ee75c5f, part 'Gear oil' no PN/no vendor/cost=sell=0). On the vendored PO with a part number present but cost=sell=0 the per-PO Receive button stayed DISABLED; entering cost (10) and sell (20) enabled Receive. Confirms a part cannot be received until the missing cost/sell price is entered (Delta3 S13-R7).</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="12" t="inlineStr">
         <is>
-          <t>C29440</t>
+          <t>C29383</t>
         </is>
       </c>
       <c r="B89" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29440</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29383</t>
         </is>
       </c>
       <c r="C89" s="12" t="inlineStr">
         <is>
-          <t>SF-RCV-10</t>
+          <t>SF-WOP-01</t>
         </is>
       </c>
       <c r="D89" s="12" t="inlineStr">
         <is>
-          <t>Accept Delivery (Story 12)</t>
+          <t>Waiting on Parts Column (Story 14)</t>
         </is>
       </c>
       <c r="E89" s="12" t="inlineStr">
         <is>
-          <t>Verify cost is editable on the Accept Delivery screen when $0 or missing (parity with Bulk Receive)</t>
+          <t>Verify an optional 'Waiting on Parts' column can be enabled from the column selector and shows the unreceived-parts count per WO</t>
         </is>
       </c>
       <c r="F89" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G89" s="14" t="inlineStr">
@@ -5261,39 +5261,39 @@
       </c>
       <c r="I89" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: receive surfaces re-confirmed live (RCV-po-list.png / RCV-bulk-receive.png) — PO list 'Purchase Orders'+'Receive'; Bulk Receive 'Receive Vendor Parts'/'Back To Purchase Orders'/vendor groups/'Apply to selected POs'/'Invoice Date'/'Tax'/'Receive All'. Behavior per prior VIU (BATCH 7 / 2026-07-10, FV screenshots). (build labels confirmed match; wording corrected where the build differs.)</t>
+          <t>Wording+VIU 2026-07-13: 'Waiting on Parts' column is off by default (toggle_column_unreceivedPartRequestsCount), enabled from the column selector - Story 14 built, verified prior runs (BATCH 7). Stripped 'EXPECTED PER SPEC' jargon. FLAG: exact column-selector label not re-surfaced this run (width_normal control did not open the selector panel).</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="12" t="inlineStr">
         <is>
-          <t>C29378</t>
+          <t>C29384</t>
         </is>
       </c>
       <c r="B90" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29378</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29384</t>
         </is>
       </c>
       <c r="C90" s="12" t="inlineStr">
         <is>
-          <t>SF-VEND-01</t>
+          <t>SF-WOP-02</t>
         </is>
       </c>
       <c r="D90" s="12" t="inlineStr">
         <is>
-          <t>Assign Vendor + Merge (Story 13)</t>
+          <t>Waiting on Parts Column (Story 14)</t>
         </is>
       </c>
       <c r="E90" s="12" t="inlineStr">
         <is>
-          <t>Verify the vendor-missing group provides a vendor dropdown that assigns a vendor at PO level and saves it</t>
+          <t>Verify clicking the Waiting on Parts count opens Accept Delivery for the WO's first unreceived PO</t>
         </is>
       </c>
       <c r="F90" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G90" s="14" t="inlineStr">
@@ -5308,39 +5308,39 @@
       </c>
       <c r="I90" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: receive surfaces re-confirmed live (RCV-po-list.png / RCV-bulk-receive.png) — PO list 'Purchase Orders'+'Receive'; Bulk Receive 'Receive Vendor Parts'/'Back To Purchase Orders'/vendor groups/'Apply to selected POs'/'Invoice Date'/'Tax'/'Receive All'. Behavior per prior VIU (BATCH 7 / 2026-07-10, FV screenshots). (build labels confirmed match; wording corrected where the build differs.)</t>
+          <t>Wording+VIU 2026-07-13: clicking the Waiting on Parts count opens the Bulk Receive page for the WO's first unreceived PO - verified prior (case 29384 pushed 2026-07-09/10).</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="12" t="inlineStr">
         <is>
-          <t>C29381</t>
+          <t>C29385</t>
         </is>
       </c>
       <c r="B91" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29381</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29385</t>
         </is>
       </c>
       <c r="C91" s="12" t="inlineStr">
         <is>
-          <t>SF-VEND-04</t>
+          <t>SF-WOP-03</t>
         </is>
       </c>
       <c r="D91" s="12" t="inlineStr">
         <is>
-          <t>Assign Vendor + Merge (Story 13)</t>
+          <t>Waiting on Parts Column (Story 14)</t>
         </is>
       </c>
       <c r="E91" s="12" t="inlineStr">
         <is>
-          <t>Verify assigning a different vendor with no collision auto-assigns and clears the QB flag, and Receive enables only once the part number and cost / sell price are also present</t>
+          <t>Verify a work order with nothing to receive shows '—' with no link in the Waiting on Parts column</t>
         </is>
       </c>
       <c r="F91" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G91" s="14" t="inlineStr">
@@ -5355,34 +5355,34 @@
       </c>
       <c r="I91" s="12" t="inlineStr">
         <is>
-          <t>VIU-Verified live 2026-07-14 on the Bulk Receive page (/bulk-receive) with a freshly seeded vendor-missing WO PO (S-15845, order 0ee75c5f, part 'Gear oil' no PN/no vendor/cost=sell=0). Assigning a brand-new vendor (no collision) via select_assign_vendor -&gt; POST /api/orders/{id}/assign-vendor 200 auto-assigned the vendor with NO Merge/Keep-Separate prompt and cleared the vendor-missing (QuickBooks) flag (PO left the Vendor-Missing group into the vendor's group). Receive then became available only once BOTH the part number AND cost/sell were also supplied (Receive stayed disabled with PN alone / cost=sell=0). Confirms Delta3 S13-R5/R6/R7.</t>
+          <t>Wording+VIU 2026-07-13: WO with nothing to receive shows '—' (no link) - verified prior (BATCH 7). Stripped 'EXPECTED PER SPEC' jargon.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="12" t="inlineStr">
         <is>
-          <t>C29442</t>
+          <t>C29386</t>
         </is>
       </c>
       <c r="B92" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29442</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29386</t>
         </is>
       </c>
       <c r="C92" s="12" t="inlineStr">
         <is>
-          <t>SF-VEND-06</t>
+          <t>SF-REV-01</t>
         </is>
       </c>
       <c r="D92" s="12" t="inlineStr">
         <is>
-          <t>Assign Vendor + Merge (Story 13)</t>
+          <t>Review ON (Story 16)</t>
         </is>
       </c>
       <c r="E92" s="12" t="inlineStr">
         <is>
-          <t>Verify a part cannot be received until a missing cost / sell price is entered</t>
+          <t>Verify the Require Review setting drives the review flow when turned on</t>
         </is>
       </c>
       <c r="F92" s="12" t="inlineStr">
@@ -5402,34 +5402,34 @@
       </c>
       <c r="I92" s="12" t="inlineStr">
         <is>
-          <t>VIU-Verified live 2026-07-14 on the Bulk Receive page (/bulk-receive) with a freshly seeded vendor-missing WO PO (S-15845, order 0ee75c5f, part 'Gear oil' no PN/no vendor/cost=sell=0). On the vendored PO with a part number present but cost=sell=0 the per-PO Receive button stayed DISABLED; entering cost (10) and sell (20) enabled Receive. Confirms a part cannot be received until the missing cost/sell price is entered (Delta3 S13-R7).</t>
+          <t>Wording+VIU 2026-07-13 (S2-15823 live, Require Review ON): with Require Review ON, completing routes into the review flow (Send To Review), not a direct complete. | Δ5/R12 sanity clause added 2026-07-14 (review-ON last-line-resolve -&gt; Ready for Review; auto-complete trigger verified in SF-AUTO-05).</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="12" t="inlineStr">
         <is>
-          <t>C29383</t>
+          <t>C29387</t>
         </is>
       </c>
       <c r="B93" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29383</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29387</t>
         </is>
       </c>
       <c r="C93" s="12" t="inlineStr">
         <is>
-          <t>SF-WOP-01</t>
+          <t>SF-REV-02</t>
         </is>
       </c>
       <c r="D93" s="12" t="inlineStr">
         <is>
-          <t>Waiting on Parts Column (Story 14)</t>
+          <t>Review ON (Story 16)</t>
         </is>
       </c>
       <c r="E93" s="12" t="inlineStr">
         <is>
-          <t>Verify an optional 'Waiting on Parts' column can be enabled from the column selector and shows the unreceived-parts count per WO</t>
+          <t>Verify the completion action reads 'Send To Review' when Require Review is on</t>
         </is>
       </c>
       <c r="F93" s="12" t="inlineStr">
@@ -5449,34 +5449,34 @@
       </c>
       <c r="I93" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: 'Waiting on Parts' column is off by default (toggle_column_unreceivedPartRequestsCount), enabled from the column selector - Story 14 built, verified prior runs (BATCH 7). Stripped 'EXPECTED PER SPEC' jargon. FLAG: exact column-selector label not re-surfaced this run (width_normal control did not open the selector panel).</t>
+          <t>Wording+VIU 2026-07-13 + relevance-fix re-VIU 2026-07-13 (S2-15827/S2-15783 live, Require Review ON): the primary action button = 'Send To Review' on BOTH ready and part-bearing WOs (it replaces 'Complete Work Order'). For a part-bearing WO, clicking 'Send To Review' opens a dialog HEADED 'Complete &amp; Send to Review' (body 'N part waiting to receive'; buttons Cancel / Receive Parts / Send To Review). So 'Complete &amp; Send to Review' is the review-dialog HEADER, not the button; the clickable CTA is 'Send To Review'. Title corrected + expected #2 corrected (a part-bearing WO does NOT read 'Complete Work Order'). Evidence: screenshots/relevance-fix-2026-07-13/.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="12" t="inlineStr">
         <is>
-          <t>C29384</t>
+          <t>C29388</t>
         </is>
       </c>
       <c r="B94" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29384</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29388</t>
         </is>
       </c>
       <c r="C94" s="12" t="inlineStr">
         <is>
-          <t>SF-WOP-02</t>
+          <t>SF-REV-03</t>
         </is>
       </c>
       <c r="D94" s="12" t="inlineStr">
         <is>
-          <t>Waiting on Parts Column (Story 14)</t>
+          <t>Review ON (Story 16)</t>
         </is>
       </c>
       <c r="E94" s="12" t="inlineStr">
         <is>
-          <t>Verify clicking the Waiting on Parts count opens Accept Delivery for the WO's first unreceived PO</t>
+          <t>Verify the Details step collects only mileage and engine hours when review is on (VIN captured later by reviewer)</t>
         </is>
       </c>
       <c r="F94" s="12" t="inlineStr">
@@ -5496,39 +5496,39 @@
       </c>
       <c r="I94" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: clicking the Waiting on Parts count opens the Bulk Receive page for the WO's first unreceived PO - verified prior (case 29384 pushed 2026-07-09/10).</t>
+          <t>Wording+VIU 2026-07-13: the completion Details modal shows Mileage + Engine Hours and no VIN field (confirmed live on the review-off modal S2-15827; review-on captures VIN in Mark Reviewed per SF-REV-06). Upgraded from Pending - the field set is now confirmed.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="12" t="inlineStr">
         <is>
-          <t>C29385</t>
+          <t>C29389</t>
         </is>
       </c>
       <c r="B95" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29385</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29389</t>
         </is>
       </c>
       <c r="C95" s="12" t="inlineStr">
         <is>
-          <t>SF-WOP-03</t>
+          <t>SF-REV-04</t>
         </is>
       </c>
       <c r="D95" s="12" t="inlineStr">
         <is>
-          <t>Waiting on Parts Column (Story 14)</t>
+          <t>Review ON (Story 16)</t>
         </is>
       </c>
       <c r="E95" s="12" t="inlineStr">
         <is>
-          <t>Verify a work order with nothing to receive shows '—' with no link in the Waiting on Parts column</t>
+          <t>Verify 'Receive Parts' routes to the shared receive page (no inline modal) in the review flow</t>
         </is>
       </c>
       <c r="F95" s="12" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G95" s="14" t="inlineStr">
@@ -5543,24 +5543,24 @@
       </c>
       <c r="I95" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: WO with nothing to receive shows '—' (no link) - verified prior (BATCH 7). Stripped 'EXPECTED PER SPEC' jargon.</t>
+          <t>Wording+VIU 2026-07-13: 'Receive Parts' opens the shared receive page (not an inline modal) in the review flow — verified prior drive (FV-rev04-receivestep/afterreceive.png, 2026-07-10); review flow re-confirmed live this run.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="12" t="inlineStr">
         <is>
-          <t>C29386</t>
+          <t>C29390</t>
         </is>
       </c>
       <c r="B96" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29386</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29390</t>
         </is>
       </c>
       <c r="C96" s="12" t="inlineStr">
         <is>
-          <t>SF-REV-01</t>
+          <t>SF-REV-05</t>
         </is>
       </c>
       <c r="D96" s="12" t="inlineStr">
@@ -5570,12 +5570,12 @@
       </c>
       <c r="E96" s="12" t="inlineStr">
         <is>
-          <t>Verify the Require Review setting drives the review flow when turned on</t>
+          <t>Verify Send to Review moves the WO to Review (amber) with a 'Ready for Review' banner and locks lines to Complete</t>
         </is>
       </c>
       <c r="F96" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G96" s="14" t="inlineStr">
@@ -5590,24 +5590,24 @@
       </c>
       <c r="I96" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13 (S2-15823 live, Require Review ON): with Require Review ON, completing routes into the review flow (Send To Review), not a direct complete. | Δ5/R12 sanity clause added 2026-07-14 (review-ON last-line-resolve -&gt; Ready for Review; auto-complete trigger verified in SF-AUTO-05).</t>
+          <t>Wording+VIU 2026-07-13 + relevance-fix re-VIU 2026-07-13 (S2-15823/S2-15827 live, Require Review ON): the confirm button is 'Send To Review' (NOT 'Complete &amp; Send to Review' - that is the dialog HEADER for a part-bearing WO). Send To Review -&gt; status 'Review' + 'Ready for Review' indicator; lines lock to Complete. (amber colour per design; status text 'Review' confirmed.) Step 1 label corrected. Evidence: screenshots/relevance-fix-2026-07-13/. | Δ5/R12 sanity clause added 2026-07-14 (review-ON last-line-resolve -&gt; Ready for Review; auto-complete trigger verified in SF-AUTO-05).</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="12" t="inlineStr">
         <is>
-          <t>C29387</t>
+          <t>C29391</t>
         </is>
       </c>
       <c r="B97" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29387</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29391</t>
         </is>
       </c>
       <c r="C97" s="12" t="inlineStr">
         <is>
-          <t>SF-REV-02</t>
+          <t>SF-REV-06</t>
         </is>
       </c>
       <c r="D97" s="12" t="inlineStr">
@@ -5617,12 +5617,12 @@
       </c>
       <c r="E97" s="12" t="inlineStr">
         <is>
-          <t>Verify the completion action reads 'Send To Review' when Require Review is on</t>
+          <t>Verify the Mark Reviewed dialog captures VIN (required) and disables Confirm until VIN is entered</t>
         </is>
       </c>
       <c r="F97" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G97" s="14" t="inlineStr">
@@ -5637,24 +5637,24 @@
       </c>
       <c r="I97" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13 + relevance-fix re-VIU 2026-07-13 (S2-15827/S2-15783 live, Require Review ON): the primary action button = 'Send To Review' on BOTH ready and part-bearing WOs (it replaces 'Complete Work Order'). For a part-bearing WO, clicking 'Send To Review' opens a dialog HEADED 'Complete &amp; Send to Review' (body 'N part waiting to receive'; buttons Cancel / Receive Parts / Send To Review). So 'Complete &amp; Send to Review' is the review-dialog HEADER, not the button; the clickable CTA is 'Send To Review'. Title corrected + expected #2 corrected (a part-bearing WO does NOT read 'Complete Work Order'). Evidence: screenshots/relevance-fix-2026-07-13/.</t>
+          <t>Wording+VIU 2026-07-13: Mark Reviewed action confirmed live (S2-15823). The VIN-required dialog surfaces only when the WO lacks a valid VIN; every test WO this run had a VIN (so Mark Reviewed completed directly - see SF-REV-08). VIN-required dialog verified prior run 2026-07-06 (S16-04-review-wizard.png). Stripped dev test-id 'input_review_vin' from tester wording.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="12" t="inlineStr">
         <is>
-          <t>C29388</t>
+          <t>C29392</t>
         </is>
       </c>
       <c r="B98" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29388</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29392</t>
         </is>
       </c>
       <c r="C98" s="12" t="inlineStr">
         <is>
-          <t>SF-REV-03</t>
+          <t>SF-REV-07</t>
         </is>
       </c>
       <c r="D98" s="12" t="inlineStr">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="E98" s="12" t="inlineStr">
         <is>
-          <t>Verify the Details step collects only mileage and engine hours when review is on (VIN captured later by reviewer)</t>
+          <t>Verify on Send to Review lines lock to Complete and inventory is auto-picked</t>
         </is>
       </c>
       <c r="F98" s="12" t="inlineStr">
@@ -5684,24 +5684,24 @@
       </c>
       <c r="I98" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: the completion Details modal shows Mileage + Engine Hours and no VIN field (confirmed live on the review-off modal S2-15827; review-on captures VIN in Mark Reviewed per SF-REV-06). Upgraded from Pending - the field set is now confirmed.</t>
+          <t>Wording+VIU 2026-07-13 (S2-15823 live, Require Review ON): on Send To Review the lines lock to Complete and inventory is auto-picked (design; review state confirmed live).</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="12" t="inlineStr">
         <is>
-          <t>C29389</t>
+          <t>C29393</t>
         </is>
       </c>
       <c r="B99" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29389</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29393</t>
         </is>
       </c>
       <c r="C99" s="12" t="inlineStr">
         <is>
-          <t>SF-REV-04</t>
+          <t>SF-REV-08</t>
         </is>
       </c>
       <c r="D99" s="12" t="inlineStr">
@@ -5711,12 +5711,12 @@
       </c>
       <c r="E99" s="12" t="inlineStr">
         <is>
-          <t>Verify 'Receive Parts' routes to the shared receive page (no inline modal) in the review flow</t>
+          <t>Verify Confirm Review signs off and completes the work order directly (no distinct Reviewed holding state)</t>
         </is>
       </c>
       <c r="F99" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G99" s="14" t="inlineStr">
@@ -5726,29 +5726,29 @@
       </c>
       <c r="H99" s="12" t="inlineStr">
         <is>
-          <t>READY (VIU-Verified)</t>
+          <t>BLOCKED — MILOS ANSWER · Milos answers Open Question Q8, Q4 — Distinct 'Reviewed' state before final Complete — expected or single-step?</t>
         </is>
       </c>
       <c r="I99" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: 'Receive Parts' opens the shared receive page (not an inline modal) in the review flow — verified prior drive (FV-rev04-receivestep/afterreceive.png, 2026-07-10); review flow re-confirmed live this run.</t>
+          <t>Wording+VIU 2026-07-13 (S2-15823 live, Require Review ON): Mark Reviewed (VIN present) signs off and moves the WO directly Review -&gt; Complete; no distinct 'Reviewed' holding state and no separate final Complete click (S2-15823 went Review-&gt;Complete). | Δ5/R12 sanity clause added 2026-07-14 (review-ON last-line-resolve -&gt; Ready for Review; auto-complete trigger verified in SF-AUTO-05).</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="12" t="inlineStr">
         <is>
-          <t>C29390</t>
+          <t>C29394</t>
         </is>
       </c>
       <c r="B100" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29390</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29394</t>
         </is>
       </c>
       <c r="C100" s="12" t="inlineStr">
         <is>
-          <t>SF-REV-05</t>
+          <t>SF-REV-09</t>
         </is>
       </c>
       <c r="D100" s="12" t="inlineStr">
@@ -5758,12 +5758,12 @@
       </c>
       <c r="E100" s="12" t="inlineStr">
         <is>
-          <t>Verify Send to Review moves the WO to Review (amber) with a 'Ready for Review' banner and locks lines to Complete</t>
+          <t>Verify Mark Reviewed is gated by the Review Work Orders permission and disabled for a role without it</t>
         </is>
       </c>
       <c r="F100" s="12" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G100" s="14" t="inlineStr">
@@ -5778,24 +5778,24 @@
       </c>
       <c r="I100" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13 + relevance-fix re-VIU 2026-07-13 (S2-15823/S2-15827 live, Require Review ON): the confirm button is 'Send To Review' (NOT 'Complete &amp; Send to Review' - that is the dialog HEADER for a part-bearing WO). Send To Review -&gt; status 'Review' + 'Ready for Review' indicator; lines lock to Complete. (amber colour per design; status text 'Review' confirmed.) Step 1 label corrected. Evidence: screenshots/relevance-fix-2026-07-13/. | Δ5/R12 sanity clause added 2026-07-14 (review-ON last-line-resolve -&gt; Ready for Review; auto-complete trigger verified in SF-AUTO-05).</t>
+          <t>Wording+VIU 2026-07-13: Mark Reviewed gated by Review Work Orders (woReviewWorkOrders) per fresh roles matrix (roles-matrix-2026-07-13.md); role without it sees Mark Reviewed disabled + 'Awaiting review'; self-review allowed when the role holds the permission (Milos ruling). Review flow re-confirmed live.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="12" t="inlineStr">
         <is>
-          <t>C29391</t>
+          <t>C29395</t>
         </is>
       </c>
       <c r="B101" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29391</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29395</t>
         </is>
       </c>
       <c r="C101" s="12" t="inlineStr">
         <is>
-          <t>SF-REV-06</t>
+          <t>SF-REV-10</t>
         </is>
       </c>
       <c r="D101" s="12" t="inlineStr">
@@ -5805,12 +5805,12 @@
       </c>
       <c r="E101" s="12" t="inlineStr">
         <is>
-          <t>Verify the Mark Reviewed dialog captures VIN (required) and disables Confirm until VIN is entered</t>
+          <t>Verify the Mark Reviewed dialog includes VIN / Serial # (required) with no review note field</t>
         </is>
       </c>
       <c r="F101" s="12" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G101" s="14" t="inlineStr">
@@ -5820,29 +5820,29 @@
       </c>
       <c r="H101" s="12" t="inlineStr">
         <is>
-          <t>READY (VIU-Verified)</t>
+          <t>BLOCKED — MILOS ANSWER · Milos answers Open Question Q7 — Optional review-note field absent — descope or bug?</t>
         </is>
       </c>
       <c r="I101" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: Mark Reviewed action confirmed live (S2-15823). The VIN-required dialog surfaces only when the WO lacks a valid VIN; every test WO this run had a VIN (so Mark Reviewed completed directly - see SF-REV-08). VIN-required dialog verified prior run 2026-07-06 (S16-04-review-wizard.png). Stripped dev test-id 'input_review_vin' from tester wording.</t>
+          <t>Wording+VIU 2026-07-13: Mark Reviewed uses VIN / Serial # only, no review note field (V2.4 Δ4 confirmed; SF-REV-06/10 were already note-free). Dialog surfaces when VIN missing (verified prior 2026-07-06); Mark Reviewed action re-confirmed live this run.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="12" t="inlineStr">
         <is>
-          <t>C29392</t>
+          <t>C29397</t>
         </is>
       </c>
       <c r="B102" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29392</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29397</t>
         </is>
       </c>
       <c r="C102" s="12" t="inlineStr">
         <is>
-          <t>SF-REV-07</t>
+          <t>SF-REV-12</t>
         </is>
       </c>
       <c r="D102" s="12" t="inlineStr">
@@ -5852,7 +5852,7 @@
       </c>
       <c r="E102" s="12" t="inlineStr">
         <is>
-          <t>Verify on Send to Review lines lock to Complete and inventory is auto-picked</t>
+          <t>Verify a 'Ready for Review' list filter/column surfaces the reviewer queue</t>
         </is>
       </c>
       <c r="F102" s="12" t="inlineStr">
@@ -5872,24 +5872,24 @@
       </c>
       <c r="I102" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13 (S2-15823 live, Require Review ON): on Send To Review the lines lock to Complete and inventory is auto-picked (design; review state confirmed live).</t>
+          <t>Wording+VIU 2026-07-13: 'Ready for Review' indicator confirmed on a WO in Review (S2-15823). Reviewer-queue surfacing on the WO list per design; the 'Ready for Review' label is build-accurate.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="12" t="inlineStr">
         <is>
-          <t>C29393</t>
+          <t>C29398</t>
         </is>
       </c>
       <c r="B103" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29393</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29398</t>
         </is>
       </c>
       <c r="C103" s="12" t="inlineStr">
         <is>
-          <t>SF-REV-08</t>
+          <t>SF-REV-13</t>
         </is>
       </c>
       <c r="D103" s="12" t="inlineStr">
@@ -5899,12 +5899,12 @@
       </c>
       <c r="E103" s="12" t="inlineStr">
         <is>
-          <t>Verify Confirm Review signs off and completes the work order directly (no distinct Reviewed holding state)</t>
+          <t>Verify all lines must be approved before Send To Review (the 'Send To Review' action is disabled until every line is approved)</t>
         </is>
       </c>
       <c r="F103" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G103" s="14" t="inlineStr">
@@ -5914,44 +5914,44 @@
       </c>
       <c r="H103" s="12" t="inlineStr">
         <is>
-          <t>BLOCKED — MILOS ANSWER · Milos answers Open Question Q8, Q4 — Distinct 'Reviewed' state before final Complete — expected or single-step?</t>
+          <t>READY (VIU-Verified)</t>
         </is>
       </c>
       <c r="I103" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13 (S2-15823 live, Require Review ON): Mark Reviewed (VIN present) signs off and moves the WO directly Review -&gt; Complete; no distinct 'Reviewed' holding state and no separate final Complete click (S2-15823 went Review-&gt;Complete). | Δ5/R12 sanity clause added 2026-07-14 (review-ON last-line-resolve -&gt; Ready for Review; auto-complete trigger verified in SF-AUTO-05).</t>
+          <t>Wording+VIU 2026-07-13 + relevance-fix re-VIU 2026-07-13 (S2-15783 live, Require Review ON, one unapproved line): the 'Send To Review' button is DISABLED (isDisabled=true) while a line is unapproved; it becomes usable only after every line is approved. Step label corrected ('Complete &amp; Send to Review' -&gt; 'Send To Review'; the clickable action is 'Send To Review') and expected made build-accurate (the button is disabled rather than showing an error message). Evidence: screenshots/relevance-fix-2026-07-13/neg-5b653a02-sendtoreview-blocked.png.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="12" t="inlineStr">
         <is>
-          <t>C29394</t>
+          <t>C29401</t>
         </is>
       </c>
       <c r="B104" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29394</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29401</t>
         </is>
       </c>
       <c r="C104" s="12" t="inlineStr">
         <is>
-          <t>SF-REV-09</t>
+          <t>SF-UX-01</t>
         </is>
       </c>
       <c r="D104" s="12" t="inlineStr">
         <is>
-          <t>Review ON (Story 16)</t>
+          <t>UX Refinements (Story 15)</t>
         </is>
       </c>
       <c r="E104" s="12" t="inlineStr">
         <is>
-          <t>Verify Mark Reviewed is gated by the Review Work Orders permission and disabled for a role without it</t>
+          <t>Verify the work order primary button reads 'Create Work Order'</t>
         </is>
       </c>
       <c r="F104" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G104" s="14" t="inlineStr">
@@ -5966,34 +5966,34 @@
       </c>
       <c r="I104" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: Mark Reviewed gated by Review Work Orders (woReviewWorkOrders) per fresh roles matrix (roles-matrix-2026-07-13.md); role without it sees Mark Reviewed disabled + 'Awaiting review'; self-review allowed when the role holds the permission (Milos ruling). Review flow re-confirmed live.</t>
+          <t>Wording+VIU 2026-07-13 (UX-workorders-list.png): the Work Orders create form's primary button reads 'Create Work Order' (confirmed on /workorders list Create Work Order button).</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="12" t="inlineStr">
         <is>
-          <t>C29395</t>
+          <t>C29402</t>
         </is>
       </c>
       <c r="B105" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29395</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29402</t>
         </is>
       </c>
       <c r="C105" s="12" t="inlineStr">
         <is>
-          <t>SF-REV-10</t>
+          <t>SF-UX-02</t>
         </is>
       </c>
       <c r="D105" s="12" t="inlineStr">
         <is>
-          <t>Review ON (Story 16)</t>
+          <t>UX Refinements (Story 15)</t>
         </is>
       </c>
       <c r="E105" s="12" t="inlineStr">
         <is>
-          <t>Verify the Mark Reviewed dialog includes VIN / Serial # (required) with no review note field</t>
+          <t>Verify required fields at completion appear in a centralized center modal and the tech story is NOT in that modal</t>
         </is>
       </c>
       <c r="F105" s="12" t="inlineStr">
@@ -6008,39 +6008,39 @@
       </c>
       <c r="H105" s="12" t="inlineStr">
         <is>
-          <t>BLOCKED — MILOS ANSWER · Milos answers Open Question Q7 — Optional review-note field absent — descope or bug?</t>
+          <t>READY (VIU-Verified)</t>
         </is>
       </c>
       <c r="I105" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: Mark Reviewed uses VIN / Serial # only, no review note field (V2.4 Δ4 confirmed; SF-REV-06/10 were already note-free). Dialog surfaces when VIN missing (verified prior 2026-07-06); Mark Reviewed action re-confirmed live this run.</t>
+          <t>Wording+VIU 2026-07-13: required fields collected in the centralized 'Complete Work Order' modal (Mileage + Engine Hours; no VIN field in the modal - see SF-COMP-16/SF-VAL-02 build finding); tech story handled separately.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="12" t="inlineStr">
         <is>
-          <t>C29397</t>
+          <t>C29403</t>
         </is>
       </c>
       <c r="B106" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29397</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29403</t>
         </is>
       </c>
       <c r="C106" s="12" t="inlineStr">
         <is>
-          <t>SF-REV-12</t>
+          <t>SF-UX-03</t>
         </is>
       </c>
       <c r="D106" s="12" t="inlineStr">
         <is>
-          <t>Review ON (Story 16)</t>
+          <t>UX Refinements (Story 15)</t>
         </is>
       </c>
       <c r="E106" s="12" t="inlineStr">
         <is>
-          <t>Verify a 'Ready for Review' list filter/column surfaces the reviewer queue</t>
+          <t>Verify the success screen shows WO number and total with Done and Go to Invoice, and the invoice number is on the Finance step</t>
         </is>
       </c>
       <c r="F106" s="12" t="inlineStr">
@@ -6060,39 +6060,39 @@
       </c>
       <c r="I106" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: 'Ready for Review' indicator confirmed on a WO in Review (S2-15823). Reviewer-queue surfacing on the WO list per design; the 'Ready for Review' label is build-accurate.</t>
+          <t>Wording+VIU 2026-07-13: success screen shows WO number + total with 'Done' and 'Go To Invoice'; invoice number appears on the Finance step (confirmed live via SF-COMP drives S2-15825 'Invoice total $434.95').</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="12" t="inlineStr">
         <is>
-          <t>C29398</t>
+          <t>C29405</t>
         </is>
       </c>
       <c r="B107" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29398</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29405</t>
         </is>
       </c>
       <c r="C107" s="12" t="inlineStr">
         <is>
-          <t>SF-REV-13</t>
+          <t>SF-PERM-01</t>
         </is>
       </c>
       <c r="D107" s="12" t="inlineStr">
         <is>
-          <t>Review ON (Story 16)</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="E107" s="12" t="inlineStr">
         <is>
-          <t>Verify all lines must be approved before Send To Review (the 'Send To Review' action is disabled until every line is approved)</t>
+          <t>Verify only owner/admin can view and modify Work Order settings (non-admin blocked)</t>
         </is>
       </c>
       <c r="F107" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G107" s="14" t="inlineStr">
@@ -6107,34 +6107,34 @@
       </c>
       <c r="I107" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13 + relevance-fix re-VIU 2026-07-13 (S2-15783 live, Require Review ON, one unapproved line): the 'Send To Review' button is DISABLED (isDisabled=true) while a line is unapproved; it becomes usable only after every line is approved. Step label corrected ('Complete &amp; Send to Review' -&gt; 'Send To Review'; the clickable action is 'Send To Review') and expected made build-accurate (the button is disabled rather than showing an error message). Evidence: screenshots/relevance-fix-2026-07-13/neg-5b653a02-sendtoreview-blocked.png.</t>
+          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Settings gate re-driven live: Technician POST /api/organizations/settings/change = 403, Admin = 200 (App Settings / settingsApp atom, BE-enforced). FE redirects non-admin from the settings route.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="12" t="inlineStr">
         <is>
-          <t>C29401</t>
+          <t>C29406</t>
         </is>
       </c>
       <c r="B108" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29401</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29406</t>
         </is>
       </c>
       <c r="C108" s="12" t="inlineStr">
         <is>
-          <t>SF-UX-01</t>
+          <t>SF-PERM-02</t>
         </is>
       </c>
       <c r="D108" s="12" t="inlineStr">
         <is>
-          <t>UX Refinements (Story 15)</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="E108" s="12" t="inlineStr">
         <is>
-          <t>Verify the work order primary button reads 'Create Work Order'</t>
+          <t>Verify which roles can complete a work order (Simple completion)</t>
         </is>
       </c>
       <c r="F108" s="12" t="inlineStr">
@@ -6154,34 +6154,34 @@
       </c>
       <c r="I108" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13 (UX-workorders-list.png): the Work Orders create form's primary button reads 'Create Work Order' (confirmed on /workorders list Create Work Order button).</t>
+          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Complete-WO gate = workOrdersCreateAndEdit; roles that can complete (Admin, Service Manager, Senior SA, Service Advisor, Foreman, Parts Manager) vs cannot (Technician, Parts Tech, Office, Sales Rep, Time Clock) match the matrix. FE confirmed (Complete Work Order button hidden for Technician, prior TECH-wo-detail.png); BE does not enforce WO completion (documented gap, see SF-PERM-06).</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="12" t="inlineStr">
         <is>
-          <t>C29402</t>
+          <t>C29407</t>
         </is>
       </c>
       <c r="B109" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29402</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29407</t>
         </is>
       </c>
       <c r="C109" s="12" t="inlineStr">
         <is>
-          <t>SF-UX-02</t>
+          <t>SF-PERM-03</t>
         </is>
       </c>
       <c r="D109" s="12" t="inlineStr">
         <is>
-          <t>UX Refinements (Story 15)</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="E109" s="12" t="inlineStr">
         <is>
-          <t>Verify required fields at completion appear in a centralized center modal and the tech story is NOT in that modal</t>
+          <t>Verify which roles can perform Bulk Receive</t>
         </is>
       </c>
       <c r="F109" s="12" t="inlineStr">
@@ -6201,34 +6201,34 @@
       </c>
       <c r="I109" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: required fields collected in the centralized 'Complete Work Order' modal (Mileage + Engine Hours; no VIN field in the modal - see SF-COMP-16/SF-VAL-02 build finding); tech story handled separately.</t>
+          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Bulk Receive gate = vendorOrderManagementCreateAndEdit + seeFinancialData; per-role result (Admin/SM/SrSA/SA/Foreman/Parts Manager/Parts Tech can; Office view-only; Sales Rep &amp; Time Clock cannot) matches the matrix. Stories 7/8 confirmed BUILT.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="12" t="inlineStr">
         <is>
-          <t>C29403</t>
+          <t>C29408</t>
         </is>
       </c>
       <c r="B110" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29403</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29408</t>
         </is>
       </c>
       <c r="C110" s="12" t="inlineStr">
         <is>
-          <t>SF-UX-03</t>
+          <t>SF-PERM-04</t>
         </is>
       </c>
       <c r="D110" s="12" t="inlineStr">
         <is>
-          <t>UX Refinements (Story 15)</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="E110" s="12" t="inlineStr">
         <is>
-          <t>Verify the success screen shows WO number and total with Done and Go to Invoice, and the invoice number is on the Finance step</t>
+          <t>Verify which roles can Mark Reviewed (sign off)</t>
         </is>
       </c>
       <c r="F110" s="12" t="inlineStr">
@@ -6248,24 +6248,24 @@
       </c>
       <c r="I110" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: success screen shows WO number + total with 'Done' and 'Go To Invoice'; invoice number appears on the Finance step (confirmed live via SF-COMP drives S2-15825 'Invoice total $434.95').</t>
+          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Mark Reviewed gate = woReviewWorkOrders (not open-to-all). Self-review allowed when the role holds the permission (Milos ruling 2026-07-10; no reviewer!=completer identity block). Per-role has/lacks matches the matrix.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="12" t="inlineStr">
         <is>
-          <t>C29405</t>
+          <t>C29409</t>
         </is>
       </c>
       <c r="B111" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29405</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29409</t>
         </is>
       </c>
       <c r="C111" s="12" t="inlineStr">
         <is>
-          <t>SF-PERM-01</t>
+          <t>SF-PERM-05</t>
         </is>
       </c>
       <c r="D111" s="12" t="inlineStr">
@@ -6275,12 +6275,12 @@
       </c>
       <c r="E111" s="12" t="inlineStr">
         <is>
-          <t>Verify only owner/admin can view and modify Work Order settings (non-admin blocked)</t>
+          <t>Verify the PO Receive button is hidden for office/readonly users</t>
         </is>
       </c>
       <c r="F111" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G111" s="14" t="inlineStr">
@@ -6295,24 +6295,24 @@
       </c>
       <c r="I111" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Settings gate re-driven live: Technician POST /api/organizations/settings/change = 403, Admin = 200 (App Settings / settingsApp atom, BE-enforced). FE redirects non-admin from the settings route.</t>
+          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). PO Receive gate = woOrderParts (Order Parts); Office lacks it -&gt; no Receive on PO list/detail. FE confirmed (Technician redirected from /parts/orders, prior TECH-po-list.png).</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="12" t="inlineStr">
         <is>
-          <t>C29406</t>
+          <t>C29410</t>
         </is>
       </c>
       <c r="B112" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29406</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29410</t>
         </is>
       </c>
       <c r="C112" s="12" t="inlineStr">
         <is>
-          <t>SF-PERM-02</t>
+          <t>SF-PERM-06</t>
         </is>
       </c>
       <c r="D112" s="12" t="inlineStr">
@@ -6322,7 +6322,7 @@
       </c>
       <c r="E112" s="12" t="inlineStr">
         <is>
-          <t>Verify which roles can complete a work order (Simple completion)</t>
+          <t>Verify permission gating of Simple-Flow settings and work-order actions (UI gating is the v1 pass criterion)</t>
         </is>
       </c>
       <c r="F112" s="12" t="inlineStr">
@@ -6342,24 +6342,24 @@
       </c>
       <c r="I112" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Complete-WO gate = workOrdersCreateAndEdit; roles that can complete (Admin, Service Manager, Senior SA, Service Advisor, Foreman, Parts Manager) vs cannot (Technician, Parts Tech, Office, Sales Rep, Time Clock) match the matrix. FE confirmed (Complete Work Order button hidden for Technician, prior TECH-wo-detail.png); BE does not enforce WO completion (documented gap, see SF-PERM-06).</t>
+          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Live: BE enforces the distinct settings atom (Technician settings save -&gt; 403, Admin -&gt; 200) but does NOT enforce the WO-completion / review atoms (documented 'app blocks / backend allows' gap, draft TICKET 2). v1 pass = app-level restriction (Milos Round-2 ruling). Cleaned tester wording: removed backend enum names and internal 'UI pass/API fail' phrasing.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="12" t="inlineStr">
         <is>
-          <t>C29407</t>
+          <t>C29411</t>
         </is>
       </c>
       <c r="B113" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29407</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29411</t>
         </is>
       </c>
       <c r="C113" s="12" t="inlineStr">
         <is>
-          <t>SF-PERM-03</t>
+          <t>SF-PERM-07</t>
         </is>
       </c>
       <c r="D113" s="12" t="inlineStr">
@@ -6369,12 +6369,12 @@
       </c>
       <c r="E113" s="12" t="inlineStr">
         <is>
-          <t>Verify which roles can perform Bulk Receive</t>
+          <t>Verify review sign-off is governed by the Review Work Orders custom-role permission (not open to all)</t>
         </is>
       </c>
       <c r="F113" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G113" s="14" t="inlineStr">
@@ -6389,24 +6389,24 @@
       </c>
       <c r="I113" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Bulk Receive gate = vendorOrderManagementCreateAndEdit + seeFinancialData; per-role result (Admin/SM/SrSA/SA/Foreman/Parts Manager/Parts Tech can; Office view-only; Sales Rep &amp; Time Clock cannot) matches the matrix. Stories 7/8 confirmed BUILT.</t>
+          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Review sign-off = Review Work Orders (woReviewWorkOrders), custom-role gated, not open-to-all for v1. Self-review allowed when the role holds the permission (Milos ruling 2026-07-10).</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="12" t="inlineStr">
         <is>
-          <t>C29408</t>
+          <t>C29412</t>
         </is>
       </c>
       <c r="B114" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29408</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29412</t>
         </is>
       </c>
       <c r="C114" s="12" t="inlineStr">
         <is>
-          <t>SF-PERM-04</t>
+          <t>SF-PERM-08</t>
         </is>
       </c>
       <c r="D114" s="12" t="inlineStr">
@@ -6416,12 +6416,12 @@
       </c>
       <c r="E114" s="12" t="inlineStr">
         <is>
-          <t>Verify which roles can Mark Reviewed (sign off)</t>
+          <t>Verify a user who holds the Mark Reviewed permission can Mark Reviewed a work order they completed</t>
         </is>
       </c>
       <c r="F114" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G114" s="14" t="inlineStr">
@@ -6436,24 +6436,24 @@
       </c>
       <c r="I114" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Mark Reviewed gate = woReviewWorkOrders (not open-to-all). Self-review allowed when the role holds the permission (Milos ruling 2026-07-10; no reviewer!=completer identity block). Per-role has/lacks matches the matrix.</t>
+          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Positive self-review: a role holding woReviewWorkOrders may Mark Reviewed a WO it completed (permission-gated only, no identity block). A role lacking it cannot. Matches matrix + Milos ruling.</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="12" t="inlineStr">
         <is>
-          <t>C29409</t>
+          <t>C29413</t>
         </is>
       </c>
       <c r="B115" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29409</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29413</t>
         </is>
       </c>
       <c r="C115" s="12" t="inlineStr">
         <is>
-          <t>SF-PERM-05</t>
+          <t>SF-PERM-09</t>
         </is>
       </c>
       <c r="D115" s="12" t="inlineStr">
@@ -6463,12 +6463,12 @@
       </c>
       <c r="E115" s="12" t="inlineStr">
         <is>
-          <t>Verify the PO Receive button is hidden for office/readonly users</t>
+          <t>Verify a Technician cannot add a vendorless / no-part-number part (lacks See Financial Data)</t>
         </is>
       </c>
       <c r="F115" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G115" s="14" t="inlineStr">
@@ -6483,24 +6483,24 @@
       </c>
       <c r="I115" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). PO Receive gate = woOrderParts (Order Parts); Office lacks it -&gt; no Receive on PO list/detail. FE confirmed (Technician redirected from /parts/orders, prior TECH-po-list.png).</t>
+          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Technician lacks seeFinancialData (confirmed live: Tech 6 perms, no seeFinancialData) so cannot add a vendorless / no-part-number part (sell price mandatory, gated by See Financial Data). FE gate holds; BE financial-gate on part-add not re-driven this session.</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="12" t="inlineStr">
         <is>
-          <t>C29410</t>
+          <t>C29414</t>
         </is>
       </c>
       <c r="B116" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29410</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29414</t>
         </is>
       </c>
       <c r="C116" s="12" t="inlineStr">
         <is>
-          <t>SF-PERM-06</t>
+          <t>SF-PERM-10</t>
         </is>
       </c>
       <c r="D116" s="12" t="inlineStr">
@@ -6510,12 +6510,12 @@
       </c>
       <c r="E116" s="12" t="inlineStr">
         <is>
-          <t>Verify permission gating of Simple-Flow settings and work-order actions (UI gating is the v1 pass criterion)</t>
+          <t>Verify the Complete Work Order action follows the per-role completion permission matrix</t>
         </is>
       </c>
       <c r="F116" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G116" s="14" t="inlineStr">
@@ -6530,39 +6530,39 @@
       </c>
       <c r="I116" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Live: BE enforces the distinct settings atom (Technician settings save -&gt; 403, Admin -&gt; 200) but does NOT enforce the WO-completion / review atoms (documented 'app blocks / backend allows' gap, draft TICKET 2). v1 pass = app-level restriction (Milos Round-2 ruling). Cleaned tester wording: removed backend enum names and internal 'UI pass/API fail' phrasing.</t>
+          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Per-role completion matrix (Complete gate = workOrdersCreateAndEdit) matches roles-matrix-2026-07-13.md exactly: HAS = Admin, Service Manager, Senior SA, Service Advisor, Foreman, Parts Manager; LACKS = Technician, Parts Tech, Office, Sales Rep, Time Clock.</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="12" t="inlineStr">
         <is>
-          <t>C29411</t>
+          <t>C29415</t>
         </is>
       </c>
       <c r="B117" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29411</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29415</t>
         </is>
       </c>
       <c r="C117" s="12" t="inlineStr">
         <is>
-          <t>SF-PERM-07</t>
+          <t>SF-VAL-01</t>
         </is>
       </c>
       <c r="D117" s="12" t="inlineStr">
         <is>
-          <t>Permissions</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="E117" s="12" t="inlineStr">
         <is>
-          <t>Verify review sign-off is governed by the Review Work Orders custom-role permission (not open to all)</t>
+          <t>Verify completion is blocked when required mileage is missing</t>
         </is>
       </c>
       <c r="F117" s="12" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G117" s="14" t="inlineStr">
@@ -6577,39 +6577,39 @@
       </c>
       <c r="I117" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Review sign-off = Review Work Orders (woReviewWorkOrders), custom-role gated, not open-to-all for v1. Self-review allowed when the role holds the permission (Milos ruling 2026-07-10).</t>
+          <t>Wording+VIU 2026-07-13 (S2-15783 live, Require Mileage ON): the completion Details modal shows a Mileage field; leaving it empty and pressing 'Complete Work Order' shows a 'required field' error and completion does not proceed. Settings restored byte-identical.</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="12" t="inlineStr">
         <is>
-          <t>C29412</t>
+          <t>C29417</t>
         </is>
       </c>
       <c r="B118" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29412</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29417</t>
         </is>
       </c>
       <c r="C118" s="12" t="inlineStr">
         <is>
-          <t>SF-PERM-08</t>
+          <t>SF-VAL-03</t>
         </is>
       </c>
       <c r="D118" s="12" t="inlineStr">
         <is>
-          <t>Permissions</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="E118" s="12" t="inlineStr">
         <is>
-          <t>Verify a user who holds the Mark Reviewed permission can Mark Reviewed a work order they completed</t>
+          <t>Verify completion is blocked when required engine hours are missing</t>
         </is>
       </c>
       <c r="F118" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G118" s="14" t="inlineStr">
@@ -6624,39 +6624,39 @@
       </c>
       <c r="I118" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Positive self-review: a role holding woReviewWorkOrders may Mark Reviewed a WO it completed (permission-gated only, no identity block). A role lacking it cannot. Matches matrix + Milos ruling.</t>
+          <t>Wording+VIU 2026-07-13 (S2-15783 live, Require Engine Hours ON): the completion Details modal shows an Engine Hours field; empty -&gt; 'required field' error, completion blocked. Same modal as SF-VAL-01 (Mileage + Engine Hours).</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="12" t="inlineStr">
         <is>
-          <t>C29413</t>
+          <t>C29418</t>
         </is>
       </c>
       <c r="B119" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29413</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29418</t>
         </is>
       </c>
       <c r="C119" s="12" t="inlineStr">
         <is>
-          <t>SF-PERM-09</t>
+          <t>SF-VAL-04</t>
         </is>
       </c>
       <c r="D119" s="12" t="inlineStr">
         <is>
-          <t>Permissions</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="E119" s="12" t="inlineStr">
         <is>
-          <t>Verify a Technician cannot add a vendorless / no-part-number part (lacks See Financial Data)</t>
+          <t>Verify the tech-story Next/Continue button stays disabled while the story textarea is empty</t>
         </is>
       </c>
       <c r="F119" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G119" s="14" t="inlineStr">
@@ -6671,34 +6671,34 @@
       </c>
       <c r="I119" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Technician lacks seeFinancialData (confirmed live: Tech 6 perms, no seeFinancialData) so cannot add a vendorless / no-part-number part (sell price mandatory, gated by See Financial Data). FE gate holds; BE financial-gate on part-add not re-driven this session.</t>
+          <t>Wording+VIU 2026-07-13: tech-story modal Next/Continue disabled while the story textarea is empty (Require Tech Story gate) - behavior per prior VIU; tech-story requirement is a Work Orders setting toggle (see SF-SET-15).</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="12" t="inlineStr">
         <is>
-          <t>C29414</t>
+          <t>C29419</t>
         </is>
       </c>
       <c r="B120" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29414</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29419</t>
         </is>
       </c>
       <c r="C120" s="12" t="inlineStr">
         <is>
-          <t>SF-PERM-10</t>
+          <t>SF-VAL-05</t>
         </is>
       </c>
       <c r="D120" s="12" t="inlineStr">
         <is>
-          <t>Permissions</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="E120" s="12" t="inlineStr">
         <is>
-          <t>Verify the Complete Work Order action follows the per-role completion permission matrix</t>
+          <t>Verify a required-invoice receive is blocked without a vendor invoice number</t>
         </is>
       </c>
       <c r="F120" s="12" t="inlineStr">
@@ -6718,24 +6718,24 @@
       </c>
       <c r="I120" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Per-role completion matrix (Complete gate = workOrdersCreateAndEdit) matches roles-matrix-2026-07-13.md exactly: HAS = Admin, Service Manager, Senior SA, Service Advisor, Foreman, Parts Manager; LACKS = Technician, Parts Tech, Office, Sales Rep, Time Clock.</t>
+          <t>Wording+VIU 2026-07-13: required-invoice receive blocked without a vendor invoice number - verified prior drive (FV-val05-noinvoice/withinvoice.png, 2026-07-10). Require Vendor Invoice Number gate.</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="12" t="inlineStr">
         <is>
-          <t>C29415</t>
+          <t>C29420</t>
         </is>
       </c>
       <c r="B121" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29415</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29420</t>
         </is>
       </c>
       <c r="C121" s="12" t="inlineStr">
         <is>
-          <t>SF-VAL-01</t>
+          <t>SF-VAL-06</t>
         </is>
       </c>
       <c r="D121" s="12" t="inlineStr">
@@ -6745,7 +6745,7 @@
       </c>
       <c r="E121" s="12" t="inlineStr">
         <is>
-          <t>Verify completion is blocked when required mileage is missing</t>
+          <t>Verify a vendor-missing part cannot be received without a vendor, a part number, and a cost / sell price</t>
         </is>
       </c>
       <c r="F121" s="12" t="inlineStr">
@@ -6765,24 +6765,24 @@
       </c>
       <c r="I121" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13 (S2-15783 live, Require Mileage ON): the completion Details modal shows a Mileage field; leaving it empty and pressing 'Complete Work Order' shows a 'required field' error and completion does not proceed. Settings restored byte-identical.</t>
+          <t>VIU-Verified live 2026-07-14 on the Bulk Receive page (/bulk-receive) with a freshly seeded vendor-missing WO PO (S-15845, order 0ee75c5f, part 'Gear oil' no PN/no vendor/cost=sell=0). Receive-button gate progression confirmed: no vendor -&gt; Receive DISABLED; vendor assigned (POST /api/orders/{id}/assign-vendor 200, auto-assigned with NO merge prompt, vendor-missing flag cleared) but no part number -&gt; DISABLED; part number entered but cost/sell still 0 -&gt; DISABLED; part number + vendor invoice number + cost + sell all present -&gt; Receive ENABLED (receivable). Confirms a vendor-missing part cannot be received without a vendor, a part number, and a cost/sell price.</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="12" t="inlineStr">
         <is>
-          <t>C29417</t>
+          <t>C29421</t>
         </is>
       </c>
       <c r="B122" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29417</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29421</t>
         </is>
       </c>
       <c r="C122" s="12" t="inlineStr">
         <is>
-          <t>SF-VAL-03</t>
+          <t>SF-VAL-07</t>
         </is>
       </c>
       <c r="D122" s="12" t="inlineStr">
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E122" s="12" t="inlineStr">
         <is>
-          <t>Verify completion is blocked when required engine hours are missing</t>
+          <t>Verify Confirm Review is disabled until a VIN is entered in the Mark Reviewed dialog</t>
         </is>
       </c>
       <c r="F122" s="12" t="inlineStr">
@@ -6812,24 +6812,24 @@
       </c>
       <c r="I122" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13 (S2-15783 live, Require Engine Hours ON): the completion Details modal shows an Engine Hours field; empty -&gt; 'required field' error, completion blocked. Same modal as SF-VAL-01 (Mileage + Engine Hours).</t>
+          <t>Wording+VIU 2026-07-13: Confirm Review disabled until VIN entered in the Mark Reviewed dialog (surfaces when the WO lacks a valid VIN) - same gate as SF-REV-06; Mark Reviewed action confirmed live this run, VIN-required dialog per prior 2026-07-06.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="12" t="inlineStr">
         <is>
-          <t>C29418</t>
+          <t>C29422</t>
         </is>
       </c>
       <c r="B123" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29418</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29422</t>
         </is>
       </c>
       <c r="C123" s="12" t="inlineStr">
         <is>
-          <t>SF-VAL-04</t>
+          <t>SF-VAL-08</t>
         </is>
       </c>
       <c r="D123" s="12" t="inlineStr">
@@ -6839,7 +6839,7 @@
       </c>
       <c r="E123" s="12" t="inlineStr">
         <is>
-          <t>Verify the tech-story Next/Continue button stays disabled while the story textarea is empty</t>
+          <t>Verify re-completing after cancelling does not create duplicate POs</t>
         </is>
       </c>
       <c r="F123" s="12" t="inlineStr">
@@ -6859,24 +6859,24 @@
       </c>
       <c r="I123" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: tech-story modal Next/Continue disabled while the story textarea is empty (Require Tech Story gate) - behavior per prior VIU; tech-story requirement is a Work Orders setting toggle (see SF-SET-15).</t>
+          <t>Wording+VIU 2026-07-13: re-completing after cancel creates no duplicate POs (idempotent) - verified prior (2026-07-08); consistent with SF-COMP-15/23.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="12" t="inlineStr">
         <is>
-          <t>C29419</t>
+          <t>C29424</t>
         </is>
       </c>
       <c r="B124" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29419</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29424</t>
         </is>
       </c>
       <c r="C124" s="12" t="inlineStr">
         <is>
-          <t>SF-VAL-05</t>
+          <t>SF-VAL-10</t>
         </is>
       </c>
       <c r="D124" s="12" t="inlineStr">
@@ -6886,12 +6886,12 @@
       </c>
       <c r="E124" s="12" t="inlineStr">
         <is>
-          <t>Verify a required-invoice receive is blocked without a vendor invoice number</t>
+          <t>Verify the same vendor invoice number can be reused across POs (uniqueness relaxed)</t>
         </is>
       </c>
       <c r="F124" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G124" s="14" t="inlineStr">
@@ -6906,24 +6906,24 @@
       </c>
       <c r="I124" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: required-invoice receive blocked without a vendor invoice number - verified prior drive (FV-val05-noinvoice/withinvoice.png, 2026-07-10). Require Vendor Invoice Number gate.</t>
+          <t>Wording+VIU 2026-07-13: the same vendor invoice number can be reused across POs (uniqueness relaxed) - verified prior (2026-07-10, Story 9 apply-invoice).</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="12" t="inlineStr">
         <is>
-          <t>C29420</t>
+          <t>C29425</t>
         </is>
       </c>
       <c r="B125" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29420</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29425</t>
         </is>
       </c>
       <c r="C125" s="12" t="inlineStr">
         <is>
-          <t>SF-VAL-06</t>
+          <t>SF-VAL-11</t>
         </is>
       </c>
       <c r="D125" s="12" t="inlineStr">
@@ -6933,12 +6933,12 @@
       </c>
       <c r="E125" s="12" t="inlineStr">
         <is>
-          <t>Verify a vendor-missing part cannot be received without a vendor, a part number, and a cost / sell price</t>
+          <t>Verify an unapproved line disables the Complete Work Order button with a tooltip (regardless of the Require Vendor Invoice Number setting)</t>
         </is>
       </c>
       <c r="F125" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G125" s="14" t="inlineStr">
@@ -6953,34 +6953,34 @@
       </c>
       <c r="I125" s="12" t="inlineStr">
         <is>
-          <t>VIU-Verified live 2026-07-14 on the Bulk Receive page (/bulk-receive) with a freshly seeded vendor-missing WO PO (S-15845, order 0ee75c5f, part 'Gear oil' no PN/no vendor/cost=sell=0). Receive-button gate progression confirmed: no vendor -&gt; Receive DISABLED; vendor assigned (POST /api/orders/{id}/assign-vendor 200, auto-assigned with NO merge prompt, vendor-missing flag cleared) but no part number -&gt; DISABLED; part number entered but cost/sell still 0 -&gt; DISABLED; part number + vendor invoice number + cost + sell all present -&gt; Receive ENABLED (receivable). Confirms a vendor-missing part cannot be received without a vendor, a part number, and a cost/sell price.</t>
+          <t>VIU-Verified live 2026-07-14 (WO 4448308d). Build behavior: an unapproved (Needs Approval) line disables the 'Complete Work Order' button (aria-disabled) with the GENERIC tooltip 'Every line must be approved or declined in order to complete the work order.' — confirmed identical with Require Vendor Invoice Number ON and OFF. Approving the line (status-&gt;authorized) re-enables the button. BUILD-vs-SPEC observation: the build applies the disabled-button model UNIVERSALLY, not only the Story-4 required-invoice flow (spec Δ2 expected the other flows to keep an active button + 'you need to approve the line' error toast). Not an error/data-corruption (stricter, cleaner gate) — logged as OBS in bugs-log, case ruled Verified against the build. Wording corrected: dropped the 'names the line' claim and the 'button stays active/error toast' branch.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="12" t="inlineStr">
         <is>
-          <t>C29421</t>
+          <t>C29433</t>
         </is>
       </c>
       <c r="B126" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29421</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29433</t>
         </is>
       </c>
       <c r="C126" s="12" t="inlineStr">
         <is>
-          <t>SF-VAL-07</t>
+          <t>SF-QB-08</t>
         </is>
       </c>
       <c r="D126" s="12" t="inlineStr">
         <is>
-          <t>Validation / Edge</t>
+          <t>QuickBooks / Inventory Integrity</t>
         </is>
       </c>
       <c r="E126" s="12" t="inlineStr">
         <is>
-          <t>Verify Confirm Review is disabled until a VIN is entered in the Mark Reviewed dialog</t>
+          <t>Verify Part History is preserved for a part that is genuinely inventory-tracked</t>
         </is>
       </c>
       <c r="F126" s="12" t="inlineStr">
@@ -7000,39 +7000,39 @@
       </c>
       <c r="I126" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: Confirm Review disabled until VIN entered in the Mark Reviewed dialog (surfaces when the WO lacks a valid VIN) - same gate as SF-REV-06; Mark Reviewed action confirmed live this run, VIN-required dialog per prior 2026-07-06.</t>
+          <t>Rescoped 2026-07-14 for the S10-R2 deprecation (spec _3, last-update-wins). Previously Blocked-Env on QuickBooks; the QB dependency is not needed for this assertion. Part History for a genuinely inventory-tracked part is a native in-app feature (Parts &gt; Inventory clock icon) and inventory decrement + Part History on simple completion is verified elsewhere (SF-COMP-07 Passed). Since a plain part-number add no longer makes a part inventory-tracked (S10-R2 struck), the invariant now only claims Part History for parts that ARE inventory-tracked — which holds.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="12" t="inlineStr">
         <is>
-          <t>C29422</t>
+          <t>C29461</t>
         </is>
       </c>
       <c r="B127" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29422</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29461</t>
         </is>
       </c>
       <c r="C127" s="12" t="inlineStr">
         <is>
-          <t>SF-VAL-08</t>
+          <t>SF-AUTO-01</t>
         </is>
       </c>
       <c r="D127" s="12" t="inlineStr">
         <is>
-          <t>Validation / Edge</t>
+          <t>Auto-Complete Trigger (Story 16 R12/R13)</t>
         </is>
       </c>
       <c r="E127" s="12" t="inlineStr">
         <is>
-          <t>Verify re-completing after cancelling does not create duplicate POs</t>
+          <t>Verify resolving the last open line by completing a single line auto-completes the work order when Require Review is off</t>
         </is>
       </c>
       <c r="F127" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G127" s="14" t="inlineStr">
@@ -7047,39 +7047,39 @@
       </c>
       <c r="I127" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: re-completing after cancel creates no duplicate POs (idempotent) - verified prior (2026-07-08); consistent with SF-COMP-15/23.</t>
+          <t>Wording+VIU 2026-07-14 (S-15838 live, Require Review OFF): two authorized lines; completing line 1 left the WO 'Approved'; completing the last line auto-flipped the WO to 'Complete' with no separate Complete Work Order step (WO status read via GET /api/work-orders/view/{id}).</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="12" t="inlineStr">
         <is>
-          <t>C29424</t>
+          <t>C29462</t>
         </is>
       </c>
       <c r="B128" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29424</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29462</t>
         </is>
       </c>
       <c r="C128" s="12" t="inlineStr">
         <is>
-          <t>SF-VAL-10</t>
+          <t>SF-AUTO-02</t>
         </is>
       </c>
       <c r="D128" s="12" t="inlineStr">
         <is>
-          <t>Validation / Edge</t>
+          <t>Auto-Complete Trigger (Story 16 R12/R13)</t>
         </is>
       </c>
       <c r="E128" s="12" t="inlineStr">
         <is>
-          <t>Verify the same vendor invoice number can be reused across POs (uniqueness relaxed)</t>
+          <t>Verify resolving the last open lines in bulk (several at once) auto-completes the work order when Require Review is off</t>
         </is>
       </c>
       <c r="F128" s="12" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G128" s="14" t="inlineStr">
@@ -7094,39 +7094,39 @@
       </c>
       <c r="I128" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: the same vendor invoice number can be reused across POs (uniqueness relaxed) - verified prior (2026-07-10, Story 9 apply-invoice).</t>
+          <t>Wording+VIU 2026-07-14 (S-15824 / 446c1cd6 live, Require Review OFF): 3 authorized labor lines resolved in one bulk call (POST /api/work-orders/lines/change-lines {field:'status',value:'complete',lines:[...]} -&gt; 201); the WO auto-flipped 'Approved' -&gt; 'Complete' with no separate Complete step.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="12" t="inlineStr">
         <is>
-          <t>C29425</t>
+          <t>C29463</t>
         </is>
       </c>
       <c r="B129" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29425</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29463</t>
         </is>
       </c>
       <c r="C129" s="12" t="inlineStr">
         <is>
-          <t>SF-VAL-11</t>
+          <t>SF-AUTO-03</t>
         </is>
       </c>
       <c r="D129" s="12" t="inlineStr">
         <is>
-          <t>Validation / Edge</t>
+          <t>Auto-Complete Trigger (Story 16 R12/R13)</t>
         </is>
       </c>
       <c r="E129" s="12" t="inlineStr">
         <is>
-          <t>Verify an unapproved line disables the Complete Work Order button with a tooltip (regardless of the Require Vendor Invoice Number setting)</t>
+          <t>Verify a split that leaves a work order fully resolved auto-completes that work order when Require Review is off</t>
         </is>
       </c>
       <c r="F129" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G129" s="14" t="inlineStr">
@@ -7141,39 +7141,39 @@
       </c>
       <c r="I129" s="12" t="inlineStr">
         <is>
-          <t>VIU-Verified live 2026-07-14 (WO 4448308d). Build behavior: an unapproved (Needs Approval) line disables the 'Complete Work Order' button (aria-disabled) with the GENERIC tooltip 'Every line must be approved or declined in order to complete the work order.' — confirmed identical with Require Vendor Invoice Number ON and OFF. Approving the line (status-&gt;authorized) re-enables the button. BUILD-vs-SPEC observation: the build applies the disabled-button model UNIVERSALLY, not only the Story-4 required-invoice flow (spec Δ2 expected the other flows to keep an active button + 'you need to approve the line' error toast). Not an error/data-corruption (stricter, cleaner gate) — logged as OBS in bugs-log, case ruled Verified against the build. Wording corrected: dropped the 'names the line' claim and the 'button stays active/error toast' branch.</t>
+          <t>Wording+VIU 2026-07-14 (S-15822 / a8fb8d3f live, Require Review OFF): completed 2 of 3 lines (WO stayed 'Approved'), then split the still-open line to a new WO (POST /api/work-orders/split -&gt; 201, new WO id returned); the original WO, now fully resolved, auto-flipped to 'Complete'. New split WO cleaned up (deleted).</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="12" t="inlineStr">
         <is>
-          <t>C29433</t>
+          <t>C29465</t>
         </is>
       </c>
       <c r="B130" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29433</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29465</t>
         </is>
       </c>
       <c r="C130" s="12" t="inlineStr">
         <is>
-          <t>SF-QB-08</t>
+          <t>SF-AUTO-05</t>
         </is>
       </c>
       <c r="D130" s="12" t="inlineStr">
         <is>
-          <t>QuickBooks / Inventory Integrity</t>
+          <t>Auto-Complete Trigger (Story 16 R12/R13)</t>
         </is>
       </c>
       <c r="E130" s="12" t="inlineStr">
         <is>
-          <t>Verify Part History is preserved for a part that is genuinely inventory-tracked</t>
+          <t>Verify that with Require Review on, resolving the last open line routes the work order to Ready for Review instead of auto-completing</t>
         </is>
       </c>
       <c r="F130" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G130" s="14" t="inlineStr">
@@ -7188,24 +7188,24 @@
       </c>
       <c r="I130" s="12" t="inlineStr">
         <is>
-          <t>Rescoped 2026-07-14 for the S10-R2 deprecation (spec _3, last-update-wins). Previously Blocked-Env on QuickBooks; the QB dependency is not needed for this assertion. Part History for a genuinely inventory-tracked part is a native in-app feature (Parts &gt; Inventory clock icon) and inventory decrement + Part History on simple completion is verified elsewhere (SF-COMP-07 Passed). Since a plain part-number add no longer makes a part inventory-tracked (S10-R2 struck), the invariant now only claims Part History for parts that ARE inventory-tracked — which holds.</t>
+          <t>Wording+VIU 2026-07-14 (S-15813 / 73d150d3 live): flipped Require Review ON (POST /api/organizations/settings/change requireReview:true); completing line 1 left the WO 'Approved'; resolving the last line routed the WO to 'Review' (Ready for Review), NOT 'Complete'. Settings restored byte-identical to baseline afterward.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="12" t="inlineStr">
         <is>
-          <t>C29461</t>
+          <t>C29467</t>
         </is>
       </c>
       <c r="B131" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29461</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29467</t>
         </is>
       </c>
       <c r="C131" s="12" t="inlineStr">
         <is>
-          <t>SF-AUTO-01</t>
+          <t>SF-AUTO-07</t>
         </is>
       </c>
       <c r="D131" s="12" t="inlineStr">
@@ -7215,12 +7215,12 @@
       </c>
       <c r="E131" s="12" t="inlineStr">
         <is>
-          <t>Verify resolving the last open line by completing a single line auto-completes the work order when Require Review is off</t>
+          <t>Verify the work order status transitions on the backend when the last open line is resolved (auto-Complete when review off, Ready for Review when review on)</t>
         </is>
       </c>
       <c r="F131" s="12" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G131" s="14" t="inlineStr">
@@ -7234,194 +7234,6 @@
         </is>
       </c>
       <c r="I131" s="12" t="inlineStr">
-        <is>
-          <t>Wording+VIU 2026-07-14 (S-15838 live, Require Review OFF): two authorized lines; completing line 1 left the WO 'Approved'; completing the last line auto-flipped the WO to 'Complete' with no separate Complete Work Order step (WO status read via GET /api/work-orders/view/{id}).</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="12" t="inlineStr">
-        <is>
-          <t>C29462</t>
-        </is>
-      </c>
-      <c r="B132" s="13" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29462</t>
-        </is>
-      </c>
-      <c r="C132" s="12" t="inlineStr">
-        <is>
-          <t>SF-AUTO-02</t>
-        </is>
-      </c>
-      <c r="D132" s="12" t="inlineStr">
-        <is>
-          <t>Auto-Complete Trigger (Story 16 R12/R13)</t>
-        </is>
-      </c>
-      <c r="E132" s="12" t="inlineStr">
-        <is>
-          <t>Verify resolving the last open lines in bulk (several at once) auto-completes the work order when Require Review is off</t>
-        </is>
-      </c>
-      <c r="F132" s="12" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G132" s="14" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="H132" s="12" t="inlineStr">
-        <is>
-          <t>READY (VIU-Verified)</t>
-        </is>
-      </c>
-      <c r="I132" s="12" t="inlineStr">
-        <is>
-          <t>Wording+VIU 2026-07-14 (S-15824 / 446c1cd6 live, Require Review OFF): 3 authorized labor lines resolved in one bulk call (POST /api/work-orders/lines/change-lines {field:'status',value:'complete',lines:[...]} -&gt; 201); the WO auto-flipped 'Approved' -&gt; 'Complete' with no separate Complete step.</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="12" t="inlineStr">
-        <is>
-          <t>C29463</t>
-        </is>
-      </c>
-      <c r="B133" s="13" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29463</t>
-        </is>
-      </c>
-      <c r="C133" s="12" t="inlineStr">
-        <is>
-          <t>SF-AUTO-03</t>
-        </is>
-      </c>
-      <c r="D133" s="12" t="inlineStr">
-        <is>
-          <t>Auto-Complete Trigger (Story 16 R12/R13)</t>
-        </is>
-      </c>
-      <c r="E133" s="12" t="inlineStr">
-        <is>
-          <t>Verify a split that leaves a work order fully resolved auto-completes that work order when Require Review is off</t>
-        </is>
-      </c>
-      <c r="F133" s="12" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G133" s="14" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="H133" s="12" t="inlineStr">
-        <is>
-          <t>READY (VIU-Verified)</t>
-        </is>
-      </c>
-      <c r="I133" s="12" t="inlineStr">
-        <is>
-          <t>Wording+VIU 2026-07-14 (S-15822 / a8fb8d3f live, Require Review OFF): completed 2 of 3 lines (WO stayed 'Approved'), then split the still-open line to a new WO (POST /api/work-orders/split -&gt; 201, new WO id returned); the original WO, now fully resolved, auto-flipped to 'Complete'. New split WO cleaned up (deleted).</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" s="12" t="inlineStr">
-        <is>
-          <t>C29465</t>
-        </is>
-      </c>
-      <c r="B134" s="13" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29465</t>
-        </is>
-      </c>
-      <c r="C134" s="12" t="inlineStr">
-        <is>
-          <t>SF-AUTO-05</t>
-        </is>
-      </c>
-      <c r="D134" s="12" t="inlineStr">
-        <is>
-          <t>Auto-Complete Trigger (Story 16 R12/R13)</t>
-        </is>
-      </c>
-      <c r="E134" s="12" t="inlineStr">
-        <is>
-          <t>Verify that with Require Review on, resolving the last open line routes the work order to Ready for Review instead of auto-completing</t>
-        </is>
-      </c>
-      <c r="F134" s="12" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G134" s="14" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="H134" s="12" t="inlineStr">
-        <is>
-          <t>READY (VIU-Verified)</t>
-        </is>
-      </c>
-      <c r="I134" s="12" t="inlineStr">
-        <is>
-          <t>Wording+VIU 2026-07-14 (S-15813 / 73d150d3 live): flipped Require Review ON (POST /api/organizations/settings/change requireReview:true); completing line 1 left the WO 'Approved'; resolving the last line routed the WO to 'Review' (Ready for Review), NOT 'Complete'. Settings restored byte-identical to baseline afterward.</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="12" t="inlineStr">
-        <is>
-          <t>C29467</t>
-        </is>
-      </c>
-      <c r="B135" s="13" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29467</t>
-        </is>
-      </c>
-      <c r="C135" s="12" t="inlineStr">
-        <is>
-          <t>SF-AUTO-07</t>
-        </is>
-      </c>
-      <c r="D135" s="12" t="inlineStr">
-        <is>
-          <t>Auto-Complete Trigger (Story 16 R12/R13)</t>
-        </is>
-      </c>
-      <c r="E135" s="12" t="inlineStr">
-        <is>
-          <t>Verify the work order status transitions on the backend when the last open line is resolved (auto-Complete when review off, Ready for Review when review on)</t>
-        </is>
-      </c>
-      <c r="F135" s="12" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G135" s="14" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="H135" s="12" t="inlineStr">
-        <is>
-          <t>READY (VIU-Verified)</t>
-        </is>
-      </c>
-      <c r="I135" s="12" t="inlineStr">
         <is>
           <t>Wording+VIU 2026-07-14: verified the backend status transition directly. Resolve action POST /api/work-orders/lines/change-status {status:'complete'} returns 200; GET /api/work-orders/view/{id} then shows work_order.status = 'Complete' when Require Review was OFF (S-15838/S-15824), and status = 'Review' (Ready for Review) when Require Review was ON (S-15813). Placed in an API-titled section per Standing Rule 4 (asserts a backend status transition).</t>
         </is>
@@ -7559,10 +7371,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B129" r:id="rId128"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B130" r:id="rId129"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B131" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B132" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B133" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B134" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B135" r:id="rId134"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7574,7 +7382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7635,7 +7443,1065 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>C29892</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29892</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>SF-CORE-11</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>Core parts — Pre-Resolve (Story 18)</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>Verify the Resolve cores screen lists every un-received vendor core with part info, core charge and OK / Not OK, plus an invoice-accuracy message</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G2" s="15" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="H2" s="12" t="inlineStr">
+        <is>
+          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: needs-data · who: QA (needs cookies+seed data) · needs: QA VIU: seed a WO with core-charge parts, drive the completion Resolve-Cores modal + invoice-gate round-trip.</t>
+        </is>
+      </c>
+      <c r="I2" s="12" t="inlineStr">
+        <is>
+          <t>NEW 2026-07-17 per spec `_4` (V2.6) Δ8 — Story 18 Core Parts (SV-8353), pre-resolve-before-receive model. Not yet observed — expected Blocked-Env at re-VIU until (a) a special-order vendor-sourced core is seedable (P550848 is_core=0; a vendor-sourced part request drops the core attribute — needs a dev-seeded core) and (b) the SV-8353 pre-resolve build is deployed on sv7301 (probe the completion wizard for the resolve step + the pre-resolve endpoint first). Screen labels from the Resolve Cores Flow design (wizard step 'Resolve cores'; Inventory / Special order groups; OK / Not OK) are design-sourced pending live confirm; the C-R9 state texts are spec-quoted — confirm exact on-screen wording live, never invent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>C29893</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29893</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>SF-CORE-12</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>Core parts — Pre-Resolve (Story 18)</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>Verify marking a core Not OK immediately adds the core charge to the work order total and customer invoice, while OK adds no charge</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G3" s="15" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="H3" s="12" t="inlineStr">
+        <is>
+          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: needs-data · who: QA (needs cookies+seed data) · needs: QA VIU: seed a WO with core-charge parts, drive the completion Resolve-Cores modal + invoice-gate round-trip.</t>
+        </is>
+      </c>
+      <c r="I3" s="12" t="inlineStr">
+        <is>
+          <t>NEW 2026-07-17 per spec `_4` (V2.6) Δ8 — Story 18 Core Parts (SV-8353), pre-resolve-before-receive model. Not yet observed — expected Blocked-Env at re-VIU until (a) a special-order vendor-sourced core is seedable (P550848 is_core=0; a vendor-sourced part request drops the core attribute — needs a dev-seeded core) and (b) the SV-8353 pre-resolve build is deployed on sv7301 (probe the completion wizard for the resolve step + the pre-resolve endpoint first).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>C29894</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29894</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>SF-CORE-13</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Core parts — Pre-Resolve (Story 18)</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>Verify completion and invoice creation are blocked only while a core is undecided — a decided core does not block</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: needs-data · who: QA (needs cookies+seed data) · needs: QA VIU: seed a WO with core-charge parts, drive the completion Resolve-Cores modal + invoice-gate round-trip.</t>
+        </is>
+      </c>
+      <c r="I4" s="12" t="inlineStr">
+        <is>
+          <t>NEW 2026-07-17 per spec `_4` (V2.6) Δ8 — Story 18 Core Parts (SV-8353), pre-resolve-before-receive model. Not yet observed — expected Blocked-Env at re-VIU until (a) a special-order vendor-sourced core is seedable (P550848 is_core=0; a vendor-sourced part request drops the core attribute — needs a dev-seeded core) and (b) the SV-8353 pre-resolve build is deployed on sv7301 (probe the completion wizard for the resolve step + the pre-resolve endpoint first).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>C29895</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29895</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>SF-CORE-14</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Core parts — Pre-Resolve (Story 18)</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>Verify receiving a pre-resolved core auto-applies the saved decision: OK creates exactly one vendor return, Not OK creates none, the invoice never changes, retries create no duplicates</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G5" s="15" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: needs-data · who: QA (needs cookies+seed data) · needs: QA VIU: seed a WO with core-charge parts, drive the completion Resolve-Cores modal + invoice-gate round-trip.</t>
+        </is>
+      </c>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>NEW 2026-07-17 per spec `_4` (V2.6) Δ8 — Story 18 Core Parts (SV-8353), pre-resolve-before-receive model. Not yet observed — expected Blocked-Env at re-VIU until (a) a special-order vendor-sourced core is seedable (P550848 is_core=0; a vendor-sourced part request drops the core attribute — needs a dev-seeded core) and (b) the SV-8353 pre-resolve build is deployed on sv7301 (probe the completion wizard for the resolve step + the pre-resolve endpoint first).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>C29896</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29896</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>SF-CORE-15</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Core parts — Pre-Resolve (Story 18)</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>Verify the receive dialog locks quantity to the full remaining amount once the work order is invoiced/paid, with the core auto-selected and an explanatory tooltip</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: needs-data · who: QA (needs cookies+seed data) · needs: QA VIU: seed a WO with core-charge parts, drive the completion Resolve-Cores modal + invoice-gate round-trip.</t>
+        </is>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>NEW 2026-07-17 per spec `_4` (V2.6) Δ8 — Story 18 Core Parts (SV-8353), pre-resolve-before-receive model. Not yet observed — expected Blocked-Env at re-VIU until (a) a special-order vendor-sourced core is seedable (P550848 is_core=0; a vendor-sourced part request drops the core attribute — needs a dev-seeded core) and (b) the SV-8353 pre-resolve build is deployed on sv7301 (probe the completion wizard for the resolve step + the pre-resolve endpoint first). Tooltip text is spec-quoted (C-R8) — confirm exact on-screen wording live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>C29897</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29897</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>SF-CORE-16</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>Core parts — Pre-Resolve (Story 18)</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>Verify the Lines tab shows the core decision state before and after receive: 'Core decision pending', 'Core OK — return to vendor, no charge', 'Core Not OK — customer charged'</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: needs-data · who: QA (needs cookies+seed data) · needs: QA VIU: seed a WO with core-charge parts, drive the completion Resolve-Cores modal + invoice-gate round-trip.</t>
+        </is>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>NEW 2026-07-17 per spec `_4` (V2.6) Δ8 — Story 18 Core Parts (SV-8353), pre-resolve-before-receive model. Not yet observed — expected Blocked-Env at re-VIU until (a) a special-order vendor-sourced core is seedable (P550848 is_core=0; a vendor-sourced part request drops the core attribute — needs a dev-seeded core) and (b) the SV-8353 pre-resolve build is deployed on sv7301 (probe the completion wizard for the resolve step + the pre-resolve endpoint first). The three state texts are spec-quoted (C-R9) — confirm exact on-screen wording live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>C29898</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29898</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>SF-CORE-17</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>Core parts — Pre-Resolve (Story 18)</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>Verify a core decision cannot be changed once the work order has an active invoice</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: needs-data · who: QA (needs cookies+seed data) · needs: QA VIU: seed a WO with core-charge parts, drive the completion Resolve-Cores modal + invoice-gate round-trip.</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>NEW 2026-07-17 per spec `_4` (V2.6) Δ8 — Story 18 Core Parts (SV-8353), pre-resolve-before-receive model. Not yet observed — expected Blocked-Env at re-VIU until (a) a special-order vendor-sourced core is seedable (P550848 is_core=0; a vendor-sourced part request drops the core attribute — needs a dev-seeded core) and (b) the SV-8353 pre-resolve build is deployed on sv7301 (probe the completion wizard for the resolve step + the pre-resolve endpoint first).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>C29899</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29899</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>SF-CORE-18</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Core Pre-Resolve (Story 18)</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>API: Verify POST /api/work-orders/{id}/pre-resolve-cores persists the core decision on the part request with no side-effect records</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G9" s="15" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: needs-data · who: QA (needs cookies+seed data) · needs: QA VIU: seed a WO with core-charge parts, drive the completion Resolve-Cores modal + invoice-gate round-trip.</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>NEW 2026-07-17 per spec `_4` (V2.6) Δ8 — Story 18 Core Parts (SV-8353), pre-resolve-before-receive model. Not yet observed — expected Blocked-Env at re-VIU until (a) a special-order vendor-sourced core is seedable (P550848 is_core=0; a vendor-sourced part request drops the core attribute — needs a dev-seeded core) and (b) the SV-8353 pre-resolve build is deployed on sv7301 (probe the completion wizard for the resolve step + the pre-resolve endpoint first). Endpoint from the SV-8353 technical plan — existence on sv7301 unconfirmed; probe before re-VIU.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>C29900</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29900</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>SF-CORE-19</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Core Pre-Resolve (Story 18)</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>API: Verify resolving a received core via the existing handle-core endpoints also writes the decision back to the linked core part request</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: needs-data · who: QA (needs cookies+seed data) · needs: QA VIU: seed a WO with core-charge parts, drive the completion Resolve-Cores modal + invoice-gate round-trip.</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>NEW 2026-07-17 per spec `_4` (V2.6) Δ8 — Story 18 Core Parts (SV-8353), pre-resolve-before-receive model. Not yet observed — expected Blocked-Env at re-VIU until (a) a special-order vendor-sourced core is seedable (P550848 is_core=0; a vendor-sourced part request drops the core attribute — needs a dev-seeded core) and (b) the SV-8353 pre-resolve build is deployed on sv7301 (probe the completion wizard for the resolve step + the pre-resolve endpoint first).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>C29906</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29906</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>SF-POSEL-07</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>PO Multi-Select (Story 7)</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>Verify part-sale-originated POs appear in the PO list and are selectable like work-order POs</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: reachable-now · who: QA (needs cookies+seed data) · needs: QA VIU: fresh sv7301 cookies + seeded data to drive this scenario.</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>NEW 2026-07-17 per spec `_4` (V2.6) Δ15 — part-sale POs CONFIRMED in scope for Stories 7/8 (§8 'Part Sales — confirmed (Jul 14)'; new S7 AC bullet). Seeding self-serviceable per Rule 14 (create a Part Sale with a vendor part). Not yet observed — re-VIU at the next live pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>C29355</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29355</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>SF-BULK-06</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>PO Bulk Receive Page (Story 8)</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>Verify Bulk Receive field editability: quantity editable (partial receive), cost editable ONLY when it is $0, sell locks after the WO is invoiced/paid</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="H12" s="12" t="inlineStr">
+        <is>
+          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: reachable-now · who: QA (needs cookies+seed data) · needs: QA VIU: fresh sv7301 cookies + seeded data to drive this scenario.</t>
+        </is>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>REWORDED 2026-07-17 to spec `_4` (V2.6) Δ14 (S8-R7: 'Cost is editable (if the cost is 0, if cost is not 0 cost filed should not be editable)'). The previous VIU-Verified was against the OLD 'qty and cost editable' build behavior (2026-07-13 labels). The $0-only rule has NOT been observed → re-VIU needed; if the build allows editing a non-zero cost on Bulk Receive it is a deviation until dev ships. SPEC INCONSISTENCY flagged for Milos (Rule 15.5): the surviving S8-R7 tail 'after it locks, only cost remains editable' contradicts the new only-if-$0 rule for a non-zero-cost part — cited, not silently resolved (this case asserts the $0-only rule per latest-wins; S10-R3/S12-R5 '$0/missing' parity aligns with it).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>C29907</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29907</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>SF-BULK-11</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>PO Bulk Receive Page (Story 8)</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>Verify a part-sale-originated PO can be received on the Bulk Receive page like a work-order PO</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G13" s="15" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: reachable-now · who: QA (needs cookies+seed data) · needs: QA VIU: fresh sv7301 cookies + seeded data to drive this scenario.</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>NEW 2026-07-17 per spec `_4` (V2.6) Δ15 — part-sale POs receivable on Bulk Receive (new S8 AC bullet). Seeding self-serviceable per Rule 14. Not yet observed — re-VIU at the next live pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>C29360</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29360</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>SF-INV-01</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>Apply Invoice to Selected POs (Story 9)</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>Verify each vendor group has an invoice number field under the vendor name, available only when at least one PO of that vendor is selected (no Apply button)</t>
+        </is>
+      </c>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: reachable-now · who: QA (needs cookies+seed data) · needs: QA VIU: fresh sv7301 cookies + seeded data to drive this scenario.</t>
+        </is>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>REWORDED 2026-07-17 to spec `_4` (V2.6) Δ13 (change-log 2026-07-16: 'Apply button removed from Bulk Invoice — invoice number is typed &amp; remembered, no button'). The previous VIU-Verified was against the OLD build behavior — the live label 'Apply to selected POs' was confirmed present 2026-07-13 (RCV-bulk-receive.png). The new no-button behavior has NOT been observed → re-VIU needed; the current build likely DEVIATES (button still present) until dev ships the removal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>C29361</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29361</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>SF-INV-02</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Apply Invoice to Selected POs (Story 9)</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>Verify a typed invoice number fills only the selected POs of that vendor with no Apply click, still editable per PO</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: reachable-now · who: QA (needs cookies+seed data) · needs: QA VIU: fresh sv7301 cookies + seeded data to drive this scenario.</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>REWORDED 2026-07-17 to spec `_4` (V2.6) Δ13: the fill happens as the number is typed — no Apply click. Previous VIU-Verified was against the OLD Apply-button build (2026-07-13). New behavior NOT observed → re-VIU needed; likely a build deviation until dev removes the button.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>C29362</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29362</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>SF-INV-03</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Apply Invoice to Selected POs (Story 9)</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>Verify the vendor invoice number field is scoped per vendor, absent for the vendorless group, and allows a reused invoice number</t>
+        </is>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="H16" s="12" t="inlineStr">
+        <is>
+          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: reachable-now · who: QA (needs cookies+seed data) · needs: QA VIU: fresh sv7301 cookies + seeded data to drive this scenario.</t>
+        </is>
+      </c>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>REWORDED 2026-07-17 to spec `_4` (V2.6) Δ13: per-vendor scoping retained; the vendorless group now explicitly shows NO invoice-number field (new AC). Previous VIU-Verified was against the OLD Apply-button build (2026-07-13). New behavior NOT observed → re-VIU needed; likely a build deviation until dev ships.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>C29901</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29901</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>SF-RCV-11</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>Receive Button on WO POs (Story 11)</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>Verify returning from receiving lands on the exact work order line the receive started from, not the top of the work order</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G17" s="15" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: reachable-now · who: QA (needs cookies+seed data) · needs: QA VIU: seed deliverable POs, drive the Receive / Accept-Delivery flow.</t>
+        </is>
+      </c>
+      <c r="I17" s="12" t="inlineStr">
+        <is>
+          <t>NEW 2026-07-17 per spec `_4` (V2.6) Δ9 — S11-R4 return-to-originating-line (change-log 2026-07-15 'Jul 14 SU follow-ups'). Self-serviceable per Rule 14 (seed a multi-line WO with an orderable part). Not yet observed — re-VIU at the next live pass; new requirement, may not be built on sv7301 yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>C29902</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29902</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>SF-RCV-12</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>Accept Delivery (Story 12)</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>Verify clicking Receive on a single work order part opens Accept Delivery showing all of that vendor's to-receive parts plus the vendorless group</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G18" s="15" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="H18" s="12" t="inlineStr">
+        <is>
+          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: reachable-now · who: QA (needs cookies+seed data) · needs: QA VIU: seed deliverable POs, drive the Receive / Accept-Delivery flow.</t>
+        </is>
+      </c>
+      <c r="I18" s="12" t="inlineStr">
+        <is>
+          <t>NEW 2026-07-17 per spec `_4` (V2.6) Δ10 — S12-R6 vendorless group surfaced on single-part receive (change-log 2026-07-15). Covers the CONTENT of the single-part receive view; the vendor-missing group POSITION deviation stays with SF-RCV-05/07 (Milos Round-3 ruling — unaffected by S12-R6). Self-serviceable per Rule 14. Not yet observed — re-VIU; may not be built on sv7301 yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>C29903</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29903</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>SF-RCV-13</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>Accept Delivery (Story 12)</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>Verify a vendorless part can be assigned a vendor / merged into the single-part receive on the spot, reusing the same invoice number</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G19" s="15" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="H19" s="12" t="inlineStr">
+        <is>
+          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: reachable-now · who: QA (needs cookies+seed data) · needs: QA VIU: seed deliverable POs, drive the Receive / Accept-Delivery flow.</t>
+        </is>
+      </c>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>NEW 2026-07-17 per spec `_4` (V2.6) Δ10 — the assign/merge-on-the-spot leg of S12-R6 ('reusing the same invoice number... rather than going back'). Self-serviceable per Rule 14. Not yet observed — re-VIU; may not be built on sv7301 yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>C29904</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29904</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>SF-VEND-07</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>Assign Vendor + Merge (Story 13)</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>Verify an assigned vendor stays changeable via the same dropdown until the part is received or the work order is invoiced/paid</t>
+        </is>
+      </c>
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G20" s="15" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="H20" s="12" t="inlineStr">
+        <is>
+          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: reachable-now · who: QA (needs cookies+seed data) · needs: QA VIU: seed vendor-missing POs, drive Assign-Vendor + merge.</t>
+        </is>
+      </c>
+      <c r="I20" s="12" t="inlineStr">
+        <is>
+          <t>NEW 2026-07-17 per spec `_4` (V2.6) Δ11 — S13-R8 (from SV-8343, change-log 2026-07-16: 'Vendor + part number stay changeable until receive'). Prevents receiving against the wrong vendor. Self-serviceable per Rule 14 (the invoiced/paid leg may stay Blocked-Env — invoiced/paid WO not drivable in this env, see §0-ZZ). Not yet observed — re-VIU; may not be built yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>C29905</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29905</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>SF-VEND-08</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>Assign Vendor + Merge (Story 13)</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>Verify the part number stays editable via the edit icon after entry until the part is received or the work order is invoiced/paid</t>
+        </is>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="H21" s="12" t="inlineStr">
+        <is>
+          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: reachable-now · who: QA (needs cookies+seed data) · needs: QA VIU: seed vendor-missing POs, drive Assign-Vendor + merge.</t>
+        </is>
+      </c>
+      <c r="I21" s="12" t="inlineStr">
+        <is>
+          <t>NEW 2026-07-17 per spec `_4` (V2.6) Δ11 — the part-number leg of S13-R8 ('likewise editable (edit icon) after entry, under the same condition'). Self-serviceable per Rule 14 (invoiced/paid leg may stay Blocked-Env). Not yet observed — re-VIU; may not be built yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>C29908</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29908</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>SF-WOP-04</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Waiting on Parts Column (Story 14)</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>Verify part-sale orders behave with the Waiting on Parts column — unreceived count and receive shortcut work without errors</t>
+        </is>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G22" s="15" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="H22" s="12" t="inlineStr">
+        <is>
+          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: reachable-now · who: QA (needs cookies+seed data) · needs: QA VIU: fresh sv7301 cookies + seeded data to drive this scenario.</t>
+        </is>
+      </c>
+      <c r="I22" s="12" t="inlineStr">
+        <is>
+          <t>NEW 2026-07-17 per spec `_4` (V2.6) Δ15 — the spec's remaining check: 'verify part-sale POs behave in Bulk Receive + Waiting-on-Parts'. Whether part sales surface on the list carrying the Waiting on Parts column is NOT specified — VIU-confirm the surface live (expected #1 allows either counted-consistently or cleanly-excluded; only errors/broken links fail). Seeding self-serviceable per Rule 14.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>C29909</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29909</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>SF-QB-09</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>QuickBooks / Inventory Integrity</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>Verify part-sale order status transitions are not regressed by the shared order/status logic (requested to waiting-to-receive to received)</t>
+        </is>
+      </c>
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="H23" s="12" t="inlineStr">
+        <is>
+          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: reachable-now · who: QA (needs cookies+seed data) · needs: QA VIU: complete a WO end-to-end and inspect the QuickBooks / inventory side-effects (Journal Entry, Part History, inventory decrement).</t>
+        </is>
+      </c>
+      <c r="I23" s="12" t="inlineStr">
+        <is>
+          <t>RESCOPED 2026-07-17 per spec `_4` (V2.6) Δ15 — the §8 'Part Sales impact (investigation — BE)' open question is now CONFIRMED in-spec ('Part Sales — confirmed (Jul 14)': adding a part on a Part Sale already creates a PO received via the same PO/receive pipeline; part-sale POs in scope for PO multi-select + Bulk Receive + Accept Delivery). This case now covers the spec's residual check ('the new order/status logic does not regress part-sale status transitions'); the in-scope part-sale PO behaviors are covered by the new cases SF-POSEL-07 (PO list / multi-select), SF-BULK-11 (Bulk Receive) and SF-WOP-04 (Waiting on Parts). Open-Question RESOLVED → VIU-Pending (seedable per Rule 14: create a Part Sale with a vendor part). ADDED TO TESTRAIL 2026-07-17 (was deliberately unmapped while an open question).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId22"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7646,7 +8512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7710,50 +8576,6 @@
       <c r="J1" s="5" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="12" t="inlineStr"/>
-      <c r="B2" s="12" t="inlineStr"/>
-      <c r="C2" s="12" t="inlineStr">
-        <is>
-          <t>SF-QB-09</t>
-        </is>
-      </c>
-      <c r="D2" s="12" t="inlineStr">
-        <is>
-          <t>QuickBooks / Inventory Integrity</t>
-        </is>
-      </c>
-      <c r="E2" s="12" t="inlineStr">
-        <is>
-          <t>Investigate: Part Sales unaffected by the shared order/status logic (requested -&gt; orderable/waiting-to-receive)</t>
-        </is>
-      </c>
-      <c r="F2" s="12" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="G2" s="15" t="inlineStr">
-        <is>
-          <t>Open-Question</t>
-        </is>
-      </c>
-      <c r="H2" s="12" t="inlineStr">
-        <is>
-          <t>BLOCKED — VIU PENDING (QA) · sub-bucket: reachable-now · who: QA (needs cookies+seed data) · needs: QA VIU: complete a WO end-to-end and inspect the QuickBooks / inventory side-effects (Journal Entry, Part History, inventory decrement).</t>
-        </is>
-      </c>
-      <c r="I2" s="12" t="inlineStr">
-        <is>
-          <t>QA VIU: complete a WO end-to-end and inspect the QuickBooks / inventory side-effects (Journal Entry, Part History, inventory decrement).</t>
-        </is>
-      </c>
-      <c r="J2" s="12" t="inlineStr">
-        <is>
-          <t>[No TestRail ID in map — add after next TestRail sync] NEW V2.4 §8 open question (D9). Placeholder only — do NOT fabricate expected. The shared order/status logic (requested -&gt; orderable/waiting-to-receive; PO-on-order without vendor/cost) may touch Part Sales; confirm with dev and report. Excluded from the TestRail XML update batch until scoped. | 2026-07-13: NOT in testrail-id-map.csv (no C-ID) - Open-Question / dev-investigation case, not created in TestRail. Follow-up: assign a C-ID only if/when it is imported after dev confirmation. | 2026-07-14 grind: remains an Open-Question / dev BE-investigation. The claim (Part Sales unaffected by the shared requested-&gt;orderable/waiting-to-receive order-status logic) is a back-end code-path question that is NOT meaningfully UI-observable from the app; confirming it requires dev to trace whether the shared order/status logic touches the Part Sales flow. Still unmapped in testrail-id-map.csv (no C-ID) — assign a C-ID only if imported after dev confirmation. Kept Open-Question.</t>
         </is>
       </c>
     </row>
@@ -8354,7 +9176,7 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Verify a waiting special-order core disables Complete Without Receiving (with a tooltip) and offers Receive Parts</t>
+          <t>Verify a Resolve cores screen appears before the Receive parts / Complete without receiving choice and only an undecided core blocks completing</t>
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr">
@@ -8374,7 +9196,7 @@
       </c>
       <c r="I13" s="12" t="inlineStr">
         <is>
-          <t>FLIPPED 2026-07-14 per design #4: a waiting special-order core now makes Complete Without Receiving UN-available (was 'stays available'). Blocked-Env (reconfirmed live 2026-07-14): a SPECIAL-ORDER (vendor-sourced) core cannot be created in this build — the genuine cored catalog part P550848 (core_charge=1) is stored is_core=0 and a vendor-sourced part request for it drops the core attribute, so a core that must be ORDERED and RECEIVED is not seedable. Needs a hand-seeded (dev/data) special-order core to drive the un-skippable-core completion behavior. Wording updated to the design #4 core-block behavior. design4 tooltip "Receive the core part first — its core charge must be settled before you can complete."; waiting-card "N parts waiting to receive — includes a core charge." + "Receive it to settle the core (OK / Not OK) before completing this work order." (WO Review Flow.html). Copy is per design #4 — not yet live-confirmed because a special-order (vendor-sourced) core is not seedable in this build.</t>
+          <t>REWORDED 2026-07-17 to spec `_4` (V2.6) Story 18 C-R1/C-R4 (SV-8353, pre-resolve-before-receive): replaces the 2026-07-14 design-#4 'Complete Without Receiving DISABLED while a core waits' model — completion is now gated ONLY on undecided (NULL) cores; a DECIDED core does not block Complete Without Receiving. Screen labels from the Resolve Cores Flow design (wizard step 'Resolve cores'; Inventory / Special order groups; 'OK / Not OK'; 'N / M resolved' progress; '+$X to invoice' running total) — design-sourced, pending live confirm; state labels 'Core decision pending' / 'Core OK — return to vendor, no charge' / 'Core Not OK — customer charged' are spec-quoted (C-R9) — confirm exact on-screen text live. Blocked-Env: a special-order (vendor-sourced) core is still not seedable in this build (P550848 is_core=0; a vendor-sourced part request drops the core attribute) — needs a dev-seeded special-order core. ALSO: Story 18 / SV-8353 is a new dev plan, so the pre-resolve build is likely NOT deployed on sv7301 yet — probe the completion wizard for the resolve step + the pre-resolve endpoint before any re-VIU.</t>
         </is>
       </c>
     </row>
@@ -8401,7 +9223,7 @@
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>Verify the invoice shows a 'Cores pending' flag when unresolved special-order cores exist</t>
+          <t>Verify the 'Cores pending' indication reflects only undecided special-order cores (a decided core clears it)</t>
         </is>
       </c>
       <c r="F14" s="12" t="inlineStr">
@@ -8421,7 +9243,7 @@
       </c>
       <c r="I14" s="12" t="inlineStr">
         <is>
-          <t>Blocked-Env (precise, reconfirmed live 2026-07-14): a SPECIAL-ORDER (vendor-sourced) core cannot be created in this build. The genuine cored catalog part P550848 (core_charge=1, catalogue_part_id 4b4753e0) carries its core attribute ONLY when added via the inventory-source catalog path (select_part forces Source=Inventory). A vendor-sourced part request for the SAME part (POST /api/work-orders/part/make-request with part_source_type='vendor' + inventory_part_id of P550848) returns 201 but the resulting part request has is_core=false and core_charge=0 — the core charge is dropped. Because a core that must be ORDERED and RECEIVED (special-order) is not seedable, the invoice-gate / receive-time core-resolution scenarios (Cores-pending flag, Resolve-at-Create-Invoice, receive-round-trip core resolution, PartRequest-only core, part-sale-vs-service auto-resolve, bulk-receive Ok/Not-OK once received, review-flow core resolution) cannot be driven. NOTE: the INVENTORY-core resolution path (line-level Ok/Not-OK, live +$ to invoice, no distinct Resolve-Cores wizard step) IS verified — see SF-CORE-01/02/10. Needs a hand-seeded special-order/vendor core part (dev/data).</t>
+          <t>REWORDED 2026-07-17 to spec `_4` (V2.6) Story 18 C-R4: 'Cores pending' now reflects UNDECIDED (NULL) cores only — the old invoice-gate model (flag while cores unresolved until received) is replaced by the pre-resolve model; a decided-but-unreceived core no longer flags. Blocked-Env: a special-order (vendor-sourced) core is still not seedable in this build (P550848 is_core=0; a vendor-sourced part request drops the core attribute) — needs a dev-seeded special-order core. ALSO: Story 18 / SV-8353 is a new dev plan, so the pre-resolve build is likely NOT deployed on sv7301 yet — probe the completion wizard for the resolve step + the pre-resolve endpoint before any re-VIU.</t>
         </is>
       </c>
     </row>
@@ -8468,7 +9290,7 @@
       </c>
       <c r="I15" s="12" t="inlineStr">
         <is>
-          <t>Aligned 2026-07-14 to design #4 un-skippable core: the cored line must be received first (Complete Without Receiving / Skip is disabled while the core is waiting). Blocked-Env (reconfirmed live 2026-07-14): a SPECIAL-ORDER (vendor-sourced) core cannot be created in this build — the genuine cored catalog part P550848 (core_charge=1) is stored is_core=0 and a vendor-sourced part request for it drops the core attribute, so a core that must be ORDERED and RECEIVED is not seedable. Needs a hand-seeded (dev/data) special-order core to drive the un-skippable-core completion behavior. Wording updated to the design #4 core-block behavior. design4 tooltip "Receive the core part first — its core charge must be settled before you can complete."; waiting-card "N parts waiting to receive — includes a core charge." + "Receive it to settle the core (OK / Not OK) before completing this work order." (WO Review Flow.html). Copy is per design #4 — not yet live-confirmed because a special-order (vendor-sourced) core is not seedable in this build.</t>
+          <t>RETIRE-PROPOSED (spec `_4` Δ8 — invoice-gate core model removed, 2026-07-17): the Create-Invoice-gate resolve module (route-to-receive, core-only partial receive at the gate) no longer exists in spec `_4` — Story 18 pre-resolves before receiving. Kept in TestRail UNTOUCHED pending the user's / QA-lead's explicit keep-vs-retire ruling (per the Δ7 precedent of never silently dropping). | Aligned 2026-07-14 to design #4 un-skippable core: the cored line must be received first (Complete Without Receiving / Skip is disabled while the core is waiting). Blocked-Env (reconfirmed live 2026-07-14): a SPECIAL-ORDER (vendor-sourced) core cannot be created in this build — the genuine cored catalog part P550848 (core_charge=1) is stored is_core=0 and a vendor-sourced part request for it drops the core attribute, so a core that must be ORDERED and RECEIVED is not seedable. Needs a hand-seeded (dev/data) special-order core to drive the un-skippable-core completion behavior. Wording updated to the design #4 core-block behavior. design4 tooltip "Receive the core part first — its core charge must be settled before you can complete."; waiting-card "N parts waiting to receive — includes a core charge." + "Receive it to settle the core (OK / Not OK) before completing this work order." (WO Review Flow.html). Copy is per design #4 — not yet live-confirmed because a special-order (vendor-sourced) core is not seedable in this build.</t>
         </is>
       </c>
     </row>
@@ -8515,7 +9337,7 @@
       </c>
       <c r="I16" s="12" t="inlineStr">
         <is>
-          <t>Aligned 2026-07-14 to design #4 un-skippable core. Blocked-Env (reconfirmed live 2026-07-14): a SPECIAL-ORDER (vendor-sourced) core cannot be created in this build — the genuine cored catalog part P550848 (core_charge=1) is stored is_core=0 and a vendor-sourced part request for it drops the core attribute, so a core that must be ORDERED and RECEIVED is not seedable. Needs a hand-seeded (dev/data) special-order core to drive the un-skippable-core completion behavior. Wording updated to the design #4 core-block behavior. design4 tooltip "Receive the core part first — its core charge must be settled before you can complete."; waiting-card "N parts waiting to receive — includes a core charge." + "Receive it to settle the core (OK / Not OK) before completing this work order." (WO Review Flow.html). Copy is per design #4 — not yet live-confirmed because a special-order (vendor-sourced) core is not seedable in this build.</t>
+          <t>RETIRE-PROPOSED (spec `_4` Δ8 — invoice-gate core model removed, 2026-07-17): the invoice-gate resolve module's cancel path no longer exists in spec `_4` — Story 18 pre-resolves before receiving. Kept in TestRail UNTOUCHED pending the user's / QA-lead's explicit keep-vs-retire ruling (per the Δ7 precedent of never silently dropping). | Aligned 2026-07-14 to design #4 un-skippable core. Blocked-Env (reconfirmed live 2026-07-14): a SPECIAL-ORDER (vendor-sourced) core cannot be created in this build — the genuine cored catalog part P550848 (core_charge=1) is stored is_core=0 and a vendor-sourced part request for it drops the core attribute, so a core that must be ORDERED and RECEIVED is not seedable. Needs a hand-seeded (dev/data) special-order core to drive the un-skippable-core completion behavior. Wording updated to the design #4 core-block behavior. design4 tooltip "Receive the core part first — its core charge must be settled before you can complete."; waiting-card "N parts waiting to receive — includes a core charge." + "Receive it to settle the core (OK / Not OK) before completing this work order." (WO Review Flow.html). Copy is per design #4 — not yet live-confirmed because a special-order (vendor-sourced) core is not seedable in this build.</t>
         </is>
       </c>
     </row>
@@ -8542,7 +9364,7 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Verify special-order cores are resolved after the required-invoice Receive round-trip before Complete</t>
+          <t>Verify the required-invoice flow asks to resolve special-order cores FIRST and then to receive them</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
@@ -8562,7 +9384,7 @@
       </c>
       <c r="I17" s="12" t="inlineStr">
         <is>
-          <t>Aligned 2026-07-14 to design #4 un-skippable core (required-invoice path already receive-first). Blocked-Env (reconfirmed live 2026-07-14): a SPECIAL-ORDER (vendor-sourced) core cannot be created in this build — the genuine cored catalog part P550848 (core_charge=1) is stored is_core=0 and a vendor-sourced part request for it drops the core attribute, so a core that must be ORDERED and RECEIVED is not seedable. Needs a hand-seeded (dev/data) special-order core to drive the un-skippable-core completion behavior. Wording updated to the design #4 core-block behavior. design4 tooltip "Receive the core part first — its core charge must be settled before you can complete."; waiting-card "N parts waiting to receive — includes a core charge." + "Receive it to settle the core (OK / Not OK) before completing this work order." (WO Review Flow.html). Copy is per design #4 — not yet live-confirmed because a special-order (vendor-sourced) core is not seedable in this build.</t>
+          <t>REWORDED 2026-07-17 to spec `_4` (V2.6) Story 18 C-R6: the required-invoice flow FLIPS from resolve-AFTER-the-receive-round-trip (old S4-C2) to resolve-FIRST-then-receive (unified with the optional flow, change-log 2026-07-16). NOTE the Resolve Cores Flow design still codes the required-flow branch as resolve-after-receive — spec (2026-07-16) wins; design flagged for cleanup. Blocked-Env: a special-order (vendor-sourced) core is still not seedable in this build (P550848 is_core=0; a vendor-sourced part request drops the core attribute) — needs a dev-seeded special-order core. ALSO: Story 18 / SV-8353 is a new dev plan, so the pre-resolve build is likely NOT deployed on sv7301 yet — probe the completion wizard for the resolve step + the pre-resolve endpoint before any re-VIU.</t>
         </is>
       </c>
     </row>
@@ -8589,7 +9411,7 @@
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Verify the invoice gate detects an unresolved special-order core that exists only as a PartRequest</t>
+          <t>Verify the completion and invoice gates detect an undecided special-order core that exists only as a requested part</t>
         </is>
       </c>
       <c r="F18" s="12" t="inlineStr">
@@ -8609,7 +9431,7 @@
       </c>
       <c r="I18" s="12" t="inlineStr">
         <is>
-          <t>Blocked-Env (precise, reconfirmed live 2026-07-14): a SPECIAL-ORDER (vendor-sourced) core cannot be created in this build. The genuine cored catalog part P550848 (core_charge=1, catalogue_part_id 4b4753e0) carries its core attribute ONLY when added via the inventory-source catalog path (select_part forces Source=Inventory). A vendor-sourced part request for the SAME part (POST /api/work-orders/part/make-request with part_source_type='vendor' + inventory_part_id of P550848) returns 201 but the resulting part request has is_core=false and core_charge=0 — the core charge is dropped. Because a core that must be ORDERED and RECEIVED (special-order) is not seedable, the invoice-gate / receive-time core-resolution scenarios (Cores-pending flag, Resolve-at-Create-Invoice, receive-round-trip core resolution, PartRequest-only core, part-sale-vs-service auto-resolve, bulk-receive Ok/Not-OK once received, review-flow core resolution) cannot be driven. NOTE: the INVENTORY-core resolution path (line-level Ok/Not-OK, live +$ to invoice, no distinct Resolve-Cores wizard step) IS verified — see SF-CORE-01/02/10. Needs a hand-seeded special-order/vendor core part (dev/data).</t>
+          <t>REWORDED 2026-07-17 to spec `_4` (V2.6) Story 18 C-R2/C-R4: detection now works off the decision saved on the core work_order_part_request (core_resolution = ok | not_ok | NULL; NULL = undecided blocks) instead of the old invoice-gate PartRequest scan — no WorkOrderPart needed. Blocked-Env: a special-order (vendor-sourced) core is still not seedable in this build (P550848 is_core=0; a vendor-sourced part request drops the core attribute) — needs a dev-seeded special-order core. ALSO: Story 18 / SV-8353 is a new dev plan, so the pre-resolve build is likely NOT deployed on sv7301 yet — probe the completion wizard for the resolve step + the pre-resolve endpoint before any re-VIU.</t>
         </is>
       </c>
     </row>
@@ -8656,7 +9478,7 @@
       </c>
       <c r="I19" s="12" t="inlineStr">
         <is>
-          <t>Blocked-Env (precise, reconfirmed live 2026-07-14): a SPECIAL-ORDER (vendor-sourced) core cannot be created in this build. The genuine cored catalog part P550848 (core_charge=1, catalogue_part_id 4b4753e0) carries its core attribute ONLY when added via the inventory-source catalog path (select_part forces Source=Inventory). A vendor-sourced part request for the SAME part (POST /api/work-orders/part/make-request with part_source_type='vendor' + inventory_part_id of P550848) returns 201 but the resulting part request has is_core=false and core_charge=0 — the core charge is dropped. Because a core that must be ORDERED and RECEIVED (special-order) is not seedable, the invoice-gate / receive-time core-resolution scenarios (Cores-pending flag, Resolve-at-Create-Invoice, receive-round-trip core resolution, PartRequest-only core, part-sale-vs-service auto-resolve, bulk-receive Ok/Not-OK once received, review-flow core resolution) cannot be driven. NOTE: the INVENTORY-core resolution path (line-level Ok/Not-OK, live +$ to invoice, no distinct Resolve-Cores wizard step) IS verified — see SF-CORE-01/02/10. Needs a hand-seeded special-order/vendor core part (dev/data).</t>
+          <t>RETIRE-PROPOSED (spec `_4` Δ8 — invoice-gate core model removed, 2026-07-17): the 'part-sale WOs auto-resolve at receive; service WOs need manual Ok/Not OK' guardrail sentence was DELETED and Story 18 is silent on it (spec silent — flagged, not silently dropped). Kept in TestRail UNTOUCHED pending the user's / QA-lead's explicit keep-vs-retire ruling (per the Δ7 precedent of never silently dropping). | Blocked-Env (precise, reconfirmed live 2026-07-14): a SPECIAL-ORDER (vendor-sourced) core cannot be created in this build. The genuine cored catalog part P550848 (core_charge=1, catalogue_part_id 4b4753e0) carries its core attribute ONLY when added via the inventory-source catalog path (select_part forces Source=Inventory). A vendor-sourced part request for the SAME part (POST /api/work-orders/part/make-request with part_source_type='vendor' + inventory_part_id of P550848) returns 201 but the resulting part request has is_core=false and core_charge=0 — the core charge is dropped. Because a core that must be ORDERED and RECEIVED (special-order) is not seedable, the invoice-gate / receive-time core-resolution scenarios (Cores-pending flag, Resolve-at-Create-Invoice, receive-round-trip core resolution, PartRequest-only core, part-sale-vs-service auto-resolve, bulk-receive Ok/Not-OK once received, review-flow core resolution) cannot be driven. NOTE: the INVENTORY-core resolution path (line-level Ok/Not-OK, live +$ to invoice, no distinct Resolve-Cores wizard step) IS verified — see SF-CORE-01/02/10. Needs a hand-seeded special-order/vendor core part (dev/data).</t>
         </is>
       </c>
     </row>
@@ -9435,7 +10257,7 @@
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Verify cores are resolved per rules before sign-off and invoicing is blocked until both Reviewed and all cores resolved</t>
+          <t>Verify cores are decided before receiving ahead of Send to Review, and invoicing stays blocked until Reviewed and every core is decided</t>
         </is>
       </c>
       <c r="F36" s="12" t="inlineStr">
@@ -9455,7 +10277,7 @@
       </c>
       <c r="I36" s="12" t="inlineStr">
         <is>
-          <t>Aligned 2026-07-14 to design #4 un-skippable core (review flow). Blocked-Env (reconfirmed live 2026-07-14): a SPECIAL-ORDER (vendor-sourced) core cannot be created in this build — the genuine cored catalog part P550848 (core_charge=1) is stored is_core=0 and a vendor-sourced part request for it drops the core attribute, so a core that must be ORDERED and RECEIVED is not seedable. Needs a hand-seeded (dev/data) special-order core to drive the un-skippable-core completion behavior. Wording updated to the design #4 core-block behavior. design4 tooltip "Receive the core part first — its core charge must be settled before you can complete."; waiting-card "N parts waiting to receive — includes a core charge." + "Receive it to settle the core (OK / Not OK) before completing this work order." (WO Review Flow.html). Copy is per design #4 — not yet live-confirmed because a special-order (vendor-sourced) core is not seedable in this build.</t>
+          <t>REWORDED 2026-07-17 to spec `_4` (V2.6): the Story-16 core paragraph now reads 'Special-order cores (both required and optional) are pre-resolved before receiving on the resolve screen before Send to Review (no longer deferred to the invoice gate)' — the invoice-gate leg was dropped and the un-skippable/receive-first reading is replaced by gate-on-undecided (C-R4). Blocked-Env: a special-order (vendor-sourced) core is still not seedable in this build (P550848 is_core=0; a vendor-sourced part request drops the core attribute) — needs a dev-seeded special-order core. ALSO: Story 18 / SV-8353 is a new dev plan, so the pre-resolve build is likely NOT deployed on sv7301 yet — probe the completion wizard for the resolve step + the pre-resolve endpoint before any re-VIU.</t>
         </is>
       </c>
     </row>
@@ -10489,7 +11311,7 @@
           <t>SF-WOP-02 expected refinement (Bulk Receive)</t>
         </is>
       </c>
-      <c r="B10" s="21" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>PENDING — HELD FOR APPROVAL</t>
         </is>
@@ -10523,7 +11345,7 @@
           <t>Cosmetic diffs (HTML numbering / ref comma-spacing)</t>
         </is>
       </c>
-      <c r="B12" s="15" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>INTENTIONALLY LEFT</t>
         </is>

</xml_diff>

<commit_message>
Simple Flow: retire SF-CORE-05/06/09 per user ruling (deleted C29317/18/21 from TestRail, verified gone; active suite 184; deliverables regenerated)
- delete_case C29317/C29318/C29321 (3/3 HTTP 200), re-GET 400 verified gone;
  before-snapshots retained; run 325 + all other cases untouched
- case JSONs annotated Retired (bodies kept for the record)
- testrail-id-map.csv: 3 rows removed (mapping preserved in audit log + notes)
- generators exclude Retired cases; assertions 187 -> 184
- deliverables regenerated: Blockers Tracker, TestCases + Results workbooks,
  testrail-import (184 rows)
- audit log appended in spec-v4-2026-07-17/testrail-update-log.md

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_Results.xlsx
+++ b/build/simple-flow/SimpleFlow_Results.xlsx
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C4" s="2" t="n"/>
     </row>
@@ -684,7 +684,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C12" s="2" t="n"/>
     </row>
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
@@ -706,7 +706,7 @@
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>Current headline tally (2026-07-13): VIU-Verified 130 / VIU-Pending 22 / Open-Question 0 / Pending-Retest 0 = 187. Pending-Retest = the V2.4 Δ1-Δ4 cases (expected changed 2026-07-13) awaiting a live re-VIU. DEV-NOT-BUILT is 0.</t>
+          <t>Current headline tally (2026-07-13): VIU-Verified 130 / VIU-Pending 22 / Open-Question 0 / Pending-Retest 0 = 184. Pending-Retest = the V2.4 Δ1-Δ4 cases (expected changed 2026-07-13) awaiting a live re-VIU. DEV-NOT-BUILT is 0.</t>
         </is>
       </c>
       <c r="B14" s="2" t="n"/>
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C17" s="2" t="n"/>
     </row>
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
@@ -874,7 +874,7 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C28" s="2" t="n"/>
     </row>
@@ -931,7 +931,7 @@
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C35" s="2" t="n"/>
     </row>
@@ -8662,7 +8662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9250,27 +9250,27 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>C29317</t>
+          <t>C29319</t>
         </is>
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29317</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29319</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>SF-CORE-05</t>
+          <t>SF-CORE-07</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Core parts — Invoice gate</t>
+          <t>Core parts — Required invoice (Story 4)</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Verify resolving cores at the Create Invoice gate routes to receive the cored line then lets invoicing proceed</t>
+          <t>Verify the required-invoice flow asks to resolve special-order cores FIRST and then to receive them</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
@@ -9290,34 +9290,34 @@
       </c>
       <c r="I15" s="12" t="inlineStr">
         <is>
-          <t>RETIRE-PROPOSED (spec `_4` Δ8 — invoice-gate core model removed, 2026-07-17): the Create-Invoice-gate resolve module (route-to-receive, core-only partial receive at the gate) no longer exists in spec `_4` — Story 18 pre-resolves before receiving. Kept in TestRail UNTOUCHED pending the user's / QA-lead's explicit keep-vs-retire ruling (per the Δ7 precedent of never silently dropping). | Aligned 2026-07-14 to design #4 un-skippable core: the cored line must be received first (Complete Without Receiving / Skip is disabled while the core is waiting). Blocked-Env (reconfirmed live 2026-07-14): a SPECIAL-ORDER (vendor-sourced) core cannot be created in this build — the genuine cored catalog part P550848 (core_charge=1) is stored is_core=0 and a vendor-sourced part request for it drops the core attribute, so a core that must be ORDERED and RECEIVED is not seedable. Needs a hand-seeded (dev/data) special-order core to drive the un-skippable-core completion behavior. Wording updated to the design #4 core-block behavior. design4 tooltip "Receive the core part first — its core charge must be settled before you can complete."; waiting-card "N parts waiting to receive — includes a core charge." + "Receive it to settle the core (OK / Not OK) before completing this work order." (WO Review Flow.html). Copy is per design #4 — not yet live-confirmed because a special-order (vendor-sourced) core is not seedable in this build.</t>
+          <t>REWORDED 2026-07-17 to spec `_4` (V2.6) Story 18 C-R6: the required-invoice flow FLIPS from resolve-AFTER-the-receive-round-trip (old S4-C2) to resolve-FIRST-then-receive (unified with the optional flow, change-log 2026-07-16). NOTE the Resolve Cores Flow design still codes the required-flow branch as resolve-after-receive — spec (2026-07-16) wins; design flagged for cleanup. Blocked-Env: a special-order (vendor-sourced) core is still not seedable in this build (P550848 is_core=0; a vendor-sourced part request drops the core attribute) — needs a dev-seeded special-order core. ALSO: Story 18 / SV-8353 is a new dev plan, so the pre-resolve build is likely NOT deployed on sv7301 yet — probe the completion wizard for the resolve step + the pre-resolve endpoint before any re-VIU.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>C29318</t>
+          <t>C29320</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29318</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29320</t>
         </is>
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>SF-CORE-06</t>
+          <t>SF-CORE-08</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
-          <t>Core parts — Invoice gate</t>
+          <t>Core parts — Guardrail</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>Verify cancelling the invoice-gate core resolution leaves the WO completed, un-invoiced and cores-pending</t>
+          <t>Verify the completion and invoice gates detect an undecided special-order core that exists only as a requested part</t>
         </is>
       </c>
       <c r="F16" s="12" t="inlineStr">
@@ -9332,185 +9332,185 @@
       </c>
       <c r="H16" s="12" t="inlineStr">
         <is>
-          <t>BUG-10, BUG-11</t>
+          <t>BUG-10</t>
         </is>
       </c>
       <c r="I16" s="12" t="inlineStr">
         <is>
-          <t>RETIRE-PROPOSED (spec `_4` Δ8 — invoice-gate core model removed, 2026-07-17): the invoice-gate resolve module's cancel path no longer exists in spec `_4` — Story 18 pre-resolves before receiving. Kept in TestRail UNTOUCHED pending the user's / QA-lead's explicit keep-vs-retire ruling (per the Δ7 precedent of never silently dropping). | Aligned 2026-07-14 to design #4 un-skippable core. Blocked-Env (reconfirmed live 2026-07-14): a SPECIAL-ORDER (vendor-sourced) core cannot be created in this build — the genuine cored catalog part P550848 (core_charge=1) is stored is_core=0 and a vendor-sourced part request for it drops the core attribute, so a core that must be ORDERED and RECEIVED is not seedable. Needs a hand-seeded (dev/data) special-order core to drive the un-skippable-core completion behavior. Wording updated to the design #4 core-block behavior. design4 tooltip "Receive the core part first — its core charge must be settled before you can complete."; waiting-card "N parts waiting to receive — includes a core charge." + "Receive it to settle the core (OK / Not OK) before completing this work order." (WO Review Flow.html). Copy is per design #4 — not yet live-confirmed because a special-order (vendor-sourced) core is not seedable in this build.</t>
+          <t>REWORDED 2026-07-17 to spec `_4` (V2.6) Story 18 C-R2/C-R4: detection now works off the decision saved on the core work_order_part_request (core_resolution = ok | not_ok | NULL; NULL = undecided blocks) instead of the old invoice-gate PartRequest scan — no WorkOrderPart needed. Blocked-Env: a special-order (vendor-sourced) core is still not seedable in this build (P550848 is_core=0; a vendor-sourced part request drops the core attribute) — needs a dev-seeded special-order core. ALSO: Story 18 / SV-8353 is a new dev plan, so the pre-resolve build is likely NOT deployed on sv7301 yet — probe the completion wizard for the resolve step + the pre-resolve endpoint before any re-VIU.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>C29319</t>
+          <t>C29322</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29319</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29322</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>SF-CORE-07</t>
+          <t>SF-CORE-10</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Core parts — Required invoice (Story 4)</t>
+          <t>Core parts — Resolve step UI</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Verify the required-invoice flow asks to resolve special-order cores FIRST and then to receive them</t>
+          <t>Verify the core '+$ to invoice' amount is shown at the line level as a core is marked Not-OK (no Resolve-Cores wizard total)</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G17" s="12" t="inlineStr">
-        <is>
-          <t>Blocked-Env</t>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="H17" s="12" t="inlineStr">
         <is>
-          <t>BUG-10, BUG-11</t>
+          <t>BUG-10</t>
         </is>
       </c>
       <c r="I17" s="12" t="inlineStr">
         <is>
-          <t>REWORDED 2026-07-17 to spec `_4` (V2.6) Story 18 C-R6: the required-invoice flow FLIPS from resolve-AFTER-the-receive-round-trip (old S4-C2) to resolve-FIRST-then-receive (unified with the optional flow, change-log 2026-07-16). NOTE the Resolve Cores Flow design still codes the required-flow branch as resolve-after-receive — spec (2026-07-16) wins; design flagged for cleanup. Blocked-Env: a special-order (vendor-sourced) core is still not seedable in this build (P550848 is_core=0; a vendor-sourced part request drops the core attribute) — needs a dev-seeded special-order core. ALSO: Story 18 / SV-8353 is a new dev plan, so the pre-resolve build is likely NOT deployed on sv7301 yet — probe the completion wizard for the resolve step + the pre-resolve endpoint before any re-VIU.</t>
+          <t>Wording+VIU 2026-07-13: the Core sub-line shows a '+$ to invoice' amount at the line level ($0 until Not-OK); no Resolve Cores wizard total - verified prior (CORE screenshots); line-level control confirmed.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>C29320</t>
+          <t>C29331</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29320</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29331</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>SF-CORE-08</t>
+          <t>SF-VPART-01</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>Core parts — Guardrail</t>
+          <t>Vendorless / No-PN Part (Story 5)</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Verify the completion and invoice gates detect an undecided special-order core that exists only as a requested part</t>
+          <t>Verify a vendorless part can be requested with description, quantity and category (part number, cost, vendor and sell price left empty)</t>
         </is>
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G18" s="12" t="inlineStr">
-        <is>
-          <t>Blocked-Env</t>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="H18" s="12" t="inlineStr">
         <is>
-          <t>BUG-10</t>
+          <t>BUG-9</t>
         </is>
       </c>
       <c r="I18" s="12" t="inlineStr">
         <is>
-          <t>REWORDED 2026-07-17 to spec `_4` (V2.6) Story 18 C-R2/C-R4: detection now works off the decision saved on the core work_order_part_request (core_resolution = ok | not_ok | NULL; NULL = undecided blocks) instead of the old invoice-gate PartRequest scan — no WorkOrderPart needed. Blocked-Env: a special-order (vendor-sourced) core is still not seedable in this build (P550848 is_core=0; a vendor-sourced part request drops the core attribute) — needs a dev-seeded special-order core. ALSO: Story 18 / SV-8353 is a new dev plan, so the pre-resolve build is likely NOT deployed on sv7301 yet — probe the completion wizard for the resolve step + the pre-resolve endpoint before any re-VIU.</t>
+          <t>Wording+VIU 2026-07-13: receive surfaces re-confirmed live (RCV-po-list.png / RCV-bulk-receive.png) — PO list 'Purchase Orders'+'Receive'; Bulk Receive 'Receive Vendor Parts'/'Back To Purchase Orders'/vendor groups/'Apply to selected POs'/'Invoice Date'/'Tax'/'Receive All'. Behavior per prior VIU (BATCH 7 / 2026-07-10, FV screenshots). (build labels confirmed match; wording corrected where the build differs.)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>C29321</t>
+          <t>C29332</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29321</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29332</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>SF-CORE-09</t>
+          <t>SF-VPART-02</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Core parts — Guardrail</t>
+          <t>Vendorless / No-PN Part (Story 5)</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Verify part-sale work orders auto-resolve cores at receive while service work orders require manual Ok/Not OK</t>
+          <t>Verify adding a part is blocked when description, quantity or category is missing (sell price not enforced)</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G19" s="12" t="inlineStr">
-        <is>
-          <t>Blocked-Env</t>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G19" s="14" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="H19" s="12" t="inlineStr">
         <is>
-          <t>BUG-10</t>
+          <t>BUG-9</t>
         </is>
       </c>
       <c r="I19" s="12" t="inlineStr">
         <is>
-          <t>RETIRE-PROPOSED (spec `_4` Δ8 — invoice-gate core model removed, 2026-07-17): the 'part-sale WOs auto-resolve at receive; service WOs need manual Ok/Not OK' guardrail sentence was DELETED and Story 18 is silent on it (spec silent — flagged, not silently dropped). Kept in TestRail UNTOUCHED pending the user's / QA-lead's explicit keep-vs-retire ruling (per the Δ7 precedent of never silently dropping). | Blocked-Env (precise, reconfirmed live 2026-07-14): a SPECIAL-ORDER (vendor-sourced) core cannot be created in this build. The genuine cored catalog part P550848 (core_charge=1, catalogue_part_id 4b4753e0) carries its core attribute ONLY when added via the inventory-source catalog path (select_part forces Source=Inventory). A vendor-sourced part request for the SAME part (POST /api/work-orders/part/make-request with part_source_type='vendor' + inventory_part_id of P550848) returns 201 but the resulting part request has is_core=false and core_charge=0 — the core charge is dropped. Because a core that must be ORDERED and RECEIVED (special-order) is not seedable, the invoice-gate / receive-time core-resolution scenarios (Cores-pending flag, Resolve-at-Create-Invoice, receive-round-trip core resolution, PartRequest-only core, part-sale-vs-service auto-resolve, bulk-receive Ok/Not-OK once received, review-flow core resolution) cannot be driven. NOTE: the INVENTORY-core resolution path (line-level Ok/Not-OK, live +$ to invoice, no distinct Resolve-Cores wizard step) IS verified — see SF-CORE-01/02/10. Needs a hand-seeded special-order/vendor core part (dev/data).</t>
+          <t>Wording+VIU 2026-07-13: receive surfaces re-confirmed live (RCV-po-list.png / RCV-bulk-receive.png) — PO list 'Purchase Orders'+'Receive'; Bulk Receive 'Receive Vendor Parts'/'Back To Purchase Orders'/vendor groups/'Apply to selected POs'/'Invoice Date'/'Tax'/'Receive All'. Behavior per prior VIU (BATCH 7 / 2026-07-10, FV screenshots). (build labels confirmed match; wording corrected where the build differs.)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>C29322</t>
+          <t>C29337</t>
         </is>
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29322</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29337</t>
         </is>
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>SF-CORE-10</t>
+          <t>SF-VPART-07</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>Core parts — Resolve step UI</t>
+          <t>Vendorless / No-PN Part (Story 5)</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Verify the core '+$ to invoice' amount is shown at the line level as a core is marked Not-OK (no Resolve-Cores wizard total)</t>
+          <t>Verify a vendorless / no-PN part cannot be received until a part number (and vendor) is entered</t>
         </is>
       </c>
       <c r="F20" s="12" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G20" s="14" t="inlineStr">
@@ -9520,39 +9520,39 @@
       </c>
       <c r="H20" s="12" t="inlineStr">
         <is>
-          <t>BUG-10</t>
+          <t>BUG-11</t>
         </is>
       </c>
       <c r="I20" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: the Core sub-line shows a '+$ to invoice' amount at the line level ($0 until Not-OK); no Resolve Cores wizard total - verified prior (CORE screenshots); line-level control confirmed.</t>
+          <t>Wording+VIU 2026-07-13: receive surfaces re-confirmed live (RCV-po-list.png / RCV-bulk-receive.png) — PO list 'Purchase Orders'+'Receive'; Bulk Receive 'Receive Vendor Parts'/'Back To Purchase Orders'/vendor groups/'Apply to selected POs'/'Invoice Date'/'Tax'/'Receive All'. Behavior per prior VIU (BATCH 7 / 2026-07-10, FV screenshots). (build labels confirmed match; wording corrected where the build differs.)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>C29331</t>
+          <t>C29364</t>
         </is>
       </c>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29331</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29364</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>SF-VPART-01</t>
+          <t>SF-PNFIX-02</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>Vendorless / No-PN Part (Story 5)</t>
+          <t>Inline Part-Number Fix (Story 10)</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Verify a vendorless part can be requested with description, quantity and category (part number, cost, vendor and sell price left empty)</t>
+          <t>Verify a NEW part number can be entered and saved so the part can be received</t>
         </is>
       </c>
       <c r="F21" s="12" t="inlineStr">
@@ -9567,39 +9567,39 @@
       </c>
       <c r="H21" s="12" t="inlineStr">
         <is>
-          <t>BUG-9</t>
+          <t>BUG-11</t>
         </is>
       </c>
       <c r="I21" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: receive surfaces re-confirmed live (RCV-po-list.png / RCV-bulk-receive.png) — PO list 'Purchase Orders'+'Receive'; Bulk Receive 'Receive Vendor Parts'/'Back To Purchase Orders'/vendor groups/'Apply to selected POs'/'Invoice Date'/'Tax'/'Receive All'. Behavior per prior VIU (BATCH 7 / 2026-07-10, FV screenshots). (build labels confirmed match; wording corrected where the build differs.)</t>
+          <t>Rescoped 2026-07-14 for the S10-R2 deprecation (spec _3, 2026-07-14, last-update-wins ruling by QA lead): a part-number add is no longer required to create a first-class inventory/catalog part in v1. Remaining assertions VERIFIED live 2026-07-14: entering a NEW part number persists and the part becomes receivable (POST /api/orders/receive-requested-parts 200 on seeded vendor-missing PO S-15849 after entering a NEW PN + cost + sell + invoice). The previously Blocked-Env downstream inventory/catalog/Part-History creation is no longer a v1 requirement, so it is dropped from the expected result.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>C29332</t>
+          <t>C29365</t>
         </is>
       </c>
       <c r="B22" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29332</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29365</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>SF-VPART-02</t>
+          <t>SF-PNFIX-03</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>Vendorless / No-PN Part (Story 5)</t>
+          <t>Inline Part-Number Fix (Story 10)</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>Verify adding a part is blocked when description, quantity or category is missing (sell price not enforced)</t>
+          <t>Verify an EXISTING part number can be entered so the part can be received, without overwriting the item's description or category</t>
         </is>
       </c>
       <c r="F22" s="12" t="inlineStr">
@@ -9614,49 +9614,49 @@
       </c>
       <c r="H22" s="12" t="inlineStr">
         <is>
-          <t>BUG-9</t>
+          <t>BUG-11</t>
         </is>
       </c>
       <c r="I22" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: receive surfaces re-confirmed live (RCV-po-list.png / RCV-bulk-receive.png) — PO list 'Purchase Orders'+'Receive'; Bulk Receive 'Receive Vendor Parts'/'Back To Purchase Orders'/vendor groups/'Apply to selected POs'/'Invoice Date'/'Tax'/'Receive All'. Behavior per prior VIU (BATCH 7 / 2026-07-10, FV screenshots). (build labels confirmed match; wording corrected where the build differs.)</t>
+          <t>Rescoped 2026-07-14 for the S10-R2 deprecation (spec _3, last-update-wins). Verified live 2026-07-14 that entering a part number persists and the part becomes receivable (receive-requested-parts 200). The 'links to the first-class inventory item + updates stock/cost/history' assertion is deprecated (not a v1 requirement) and removed from the expected; the no-overwrite-of-description/category expectation is retained as a data-safety check.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>C29337</t>
+          <t>C29366</t>
         </is>
       </c>
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29337</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29366</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>SF-VPART-07</t>
+          <t>SF-PNFIX-04</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>Vendorless / No-PN Part (Story 5)</t>
+          <t>Inline Part-Number Fix (Story 10)</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Verify a vendorless / no-PN part cannot be received until a part number (and vendor) is entered</t>
+          <t>Verify inline part-number field-locking rules match the receive-screen rules (sell locks after invoiced/paid)</t>
         </is>
       </c>
       <c r="F23" s="12" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G23" s="14" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G23" s="12" t="inlineStr">
+        <is>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="H23" s="12" t="inlineStr">
@@ -9666,24 +9666,24 @@
       </c>
       <c r="I23" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: receive surfaces re-confirmed live (RCV-po-list.png / RCV-bulk-receive.png) — PO list 'Purchase Orders'+'Receive'; Bulk Receive 'Receive Vendor Parts'/'Back To Purchase Orders'/vendor groups/'Apply to selected POs'/'Invoice Date'/'Tax'/'Receive All'. Behavior per prior VIU (BATCH 7 / 2026-07-10, FV screenshots). (build labels confirmed match; wording corrected where the build differs.)</t>
+          <t>Blocked-Env (precise, investigated live 2026-07-14): a true invoiced/paid WO state is not drivable in this harness. On WO S-15845 (29f0c308, Complete, valid VIN set) the finance page 'Create Invoice' action and the Estimate/Invoice toggle only fire POST /api/work-orders/invoices/estimate (a recompute) — no invoice is persisted (is_invoice_created stays false, invoice_status=null, invoice_id empty); no confirm dialog renders headless. Direct invoice-create API endpoints all 404 (/api/work-orders/invoices/create, /{id}/create-invoice, /{id}/invoice, /api/work-orders/invoices). Marking the WO PAID would additionally require a payment step. So the sell-field-lock / receive-blocked-when-invoiced-or-paid behavior cannot be exercised here. Needs an invoiced+paid WO seeded by dev, or an interactive (non-headless) session that can complete the finance invoice flow.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>C29364</t>
+          <t>C29367</t>
         </is>
       </c>
       <c r="B24" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29364</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29367</t>
         </is>
       </c>
       <c r="C24" s="12" t="inlineStr">
         <is>
-          <t>SF-PNFIX-02</t>
+          <t>SF-PNFIX-05</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
@@ -9693,7 +9693,7 @@
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
-          <t>Verify a NEW part number can be entered and saved so the part can be received</t>
+          <t>Verify a part cannot be received without a part number, a vendor (for vendor-missing) and a cost / sell price, even on an invoiced/paid WO</t>
         </is>
       </c>
       <c r="F24" s="12" t="inlineStr">
@@ -9713,24 +9713,24 @@
       </c>
       <c r="I24" s="12" t="inlineStr">
         <is>
-          <t>Rescoped 2026-07-14 for the S10-R2 deprecation (spec _3, 2026-07-14, last-update-wins ruling by QA lead): a part-number add is no longer required to create a first-class inventory/catalog part in v1. Remaining assertions VERIFIED live 2026-07-14: entering a NEW part number persists and the part becomes receivable (POST /api/orders/receive-requested-parts 200 on seeded vendor-missing PO S-15849 after entering a NEW PN + cost + sell + invoice). The previously Blocked-Env downstream inventory/catalog/Part-History creation is no longer a v1 requirement, so it is dropped from the expected result.</t>
+          <t>VIU-Verified live 2026-07-14 on the Bulk Receive page (/bulk-receive) with a freshly seeded vendor-missing WO PO (S-15845, order 0ee75c5f, part 'Gear oil' no PN/no vendor/cost=sell=0). Receive gates live-confirmed: a part cannot be received without a part number, without a vendor (for a vendor-missing part), or without a cost/sell price (Receive stayed disabled until all present). The 'even on an invoiced/paid WO' clause is consistent with the field-locking behavior (SF-VAL-09: only the SELL field locks after invoiced/paid; the part-number/cost receive gates remain) — the receive gate itself is unconditional. No error surfaced (gate is a disabled affordance, not a toast).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>C29365</t>
+          <t>C29368</t>
         </is>
       </c>
       <c r="B25" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29365</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29368</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>SF-PNFIX-03</t>
+          <t>SF-PNFIX-06</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
@@ -9740,12 +9740,12 @@
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Verify an EXISTING part number can be entered so the part can be received, without overwriting the item's description or category</t>
+          <t>Verify the inline part-number save persists and enables receiving</t>
         </is>
       </c>
       <c r="F25" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G25" s="14" t="inlineStr">
@@ -9760,39 +9760,39 @@
       </c>
       <c r="I25" s="12" t="inlineStr">
         <is>
-          <t>Rescoped 2026-07-14 for the S10-R2 deprecation (spec _3, last-update-wins). Verified live 2026-07-14 that entering a part number persists and the part becomes receivable (receive-requested-parts 200). The 'links to the first-class inventory item + updates stock/cost/history' assertion is deprecated (not a v1 requirement) and removed from the expected; the no-overwrite-of-description/category expectation is retained as a data-safety check.</t>
+          <t>Rescoped 2026-07-14 for the S10-R2 deprecation (spec _3, last-update-wins). Verified live 2026-07-14 that the inline part-number save persists and the part becomes receivable (receive-requested-parts 200). The technical-guardrail assertion that the inline save must drive catalog creation + an inventory stock Part + Part History is deprecated (not a v1 requirement) and removed from the expected. NOTE: spec _3 leaves the Story-10 Acceptance-Criteria bullets and 'Technical guardrails' paragraph still describing first-class-part creation while R2 itself is struck — an internal inconsistency in the doc; flagged for spec cleanup. Applied the strike per the QA-lead last-update-wins ruling.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>C29366</t>
+          <t>C29376</t>
         </is>
       </c>
       <c r="B26" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29366</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29376</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>SF-PNFIX-04</t>
+          <t>SF-RCV-08</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>Inline Part-Number Fix (Story 10)</t>
+          <t>Accept Delivery (Story 12)</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>Verify inline part-number field-locking rules match the receive-screen rules (sell locks after invoiced/paid)</t>
+          <t>Verify each vendor group produces its own vendor bill and separate AP entry in QuickBooks</t>
         </is>
       </c>
       <c r="F26" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G26" s="12" t="inlineStr">
@@ -9807,39 +9807,39 @@
       </c>
       <c r="I26" s="12" t="inlineStr">
         <is>
-          <t>Blocked-Env (precise, investigated live 2026-07-14): a true invoiced/paid WO state is not drivable in this harness. On WO S-15845 (29f0c308, Complete, valid VIN set) the finance page 'Create Invoice' action and the Estimate/Invoice toggle only fire POST /api/work-orders/invoices/estimate (a recompute) — no invoice is persisted (is_invoice_created stays false, invoice_status=null, invoice_id empty); no confirm dialog renders headless. Direct invoice-create API endpoints all 404 (/api/work-orders/invoices/create, /{id}/create-invoice, /{id}/invoice, /api/work-orders/invoices). Marking the WO PAID would additionally require a payment step. So the sell-field-lock / receive-blocked-when-invoiced-or-paid behavior cannot be exercised here. Needs an invoiced+paid WO seeded by dev, or an interactive (non-headless) session that can complete the finance invoice flow.</t>
+          <t>Blocked-Env (precise, confirmed live 2026-07-14): QuickBooks is NOT connected on the sv7301 QA org. There is NO QuickBooks/accounting/integrations option in the Admin menu (menu = Work Orders, Schedule, Customers, Parts, Reports, Feature Flags, Settings, Staff, Locations, Departments, Taxes, Labor Rates, Canned Lines, Asset Types, Pricing, Bin Locations, Categories, IBS, Payment Methods, Contacts, Assets, Vendors, Inventory, Invoices — no QuickBooks); /administration/integrations does not exist; all QB API endpoints 404 (/api/quickbooks*, /api/integrations/quickbooks, /api/organizations/integrations); the WO finance object has invoice_shop_id=null. So QuickBooks sync/vendor-bill/AP/Journal-Entry side-effects cannot be inspected here. Needs a QB-connected company + a human in QuickBooks.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>C29367</t>
+          <t>C29388</t>
         </is>
       </c>
       <c r="B27" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29367</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29388</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>SF-PNFIX-05</t>
+          <t>SF-REV-03</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Inline Part-Number Fix (Story 10)</t>
+          <t>Review ON (Story 16)</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Verify a part cannot be received without a part number, a vendor (for vendor-missing) and a cost / sell price, even on an invoiced/paid WO</t>
+          <t>Verify the Details step collects only mileage and engine hours when review is on (VIN captured later by reviewer)</t>
         </is>
       </c>
       <c r="F27" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G27" s="14" t="inlineStr">
@@ -9849,39 +9849,39 @@
       </c>
       <c r="H27" s="12" t="inlineStr">
         <is>
-          <t>BUG-11</t>
+          <t>BUG-8</t>
         </is>
       </c>
       <c r="I27" s="12" t="inlineStr">
         <is>
-          <t>VIU-Verified live 2026-07-14 on the Bulk Receive page (/bulk-receive) with a freshly seeded vendor-missing WO PO (S-15845, order 0ee75c5f, part 'Gear oil' no PN/no vendor/cost=sell=0). Receive gates live-confirmed: a part cannot be received without a part number, without a vendor (for a vendor-missing part), or without a cost/sell price (Receive stayed disabled until all present). The 'even on an invoiced/paid WO' clause is consistent with the field-locking behavior (SF-VAL-09: only the SELL field locks after invoiced/paid; the part-number/cost receive gates remain) — the receive gate itself is unconditional. No error surfaced (gate is a disabled affordance, not a toast).</t>
+          <t>Wording+VIU 2026-07-13: the completion Details modal shows Mileage + Engine Hours and no VIN field (confirmed live on the review-off modal S2-15827; review-on captures VIN in Mark Reviewed per SF-REV-06). Upgraded from Pending - the field set is now confirmed.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>C29368</t>
+          <t>C29389</t>
         </is>
       </c>
       <c r="B28" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29368</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29389</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>SF-PNFIX-06</t>
+          <t>SF-REV-04</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>Inline Part-Number Fix (Story 10)</t>
+          <t>Review ON (Story 16)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>Verify the inline part-number save persists and enables receiving</t>
+          <t>Verify 'Receive Parts' routes to the shared receive page (no inline modal) in the review flow</t>
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr">
@@ -9901,34 +9901,34 @@
       </c>
       <c r="I28" s="12" t="inlineStr">
         <is>
-          <t>Rescoped 2026-07-14 for the S10-R2 deprecation (spec _3, last-update-wins). Verified live 2026-07-14 that the inline part-number save persists and the part becomes receivable (receive-requested-parts 200). The technical-guardrail assertion that the inline save must drive catalog creation + an inventory stock Part + Part History is deprecated (not a v1 requirement) and removed from the expected. NOTE: spec _3 leaves the Story-10 Acceptance-Criteria bullets and 'Technical guardrails' paragraph still describing first-class-part creation while R2 itself is struck — an internal inconsistency in the doc; flagged for spec cleanup. Applied the strike per the QA-lead last-update-wins ruling.</t>
+          <t>Wording+VIU 2026-07-13: 'Receive Parts' opens the shared receive page (not an inline modal) in the review flow — verified prior drive (FV-rev04-receivestep/afterreceive.png, 2026-07-10); review flow re-confirmed live this run.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>C29376</t>
+          <t>C29393</t>
         </is>
       </c>
       <c r="B29" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29376</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29393</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>SF-RCV-08</t>
+          <t>SF-REV-08</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Accept Delivery (Story 12)</t>
+          <t>Review ON (Story 16)</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>Verify each vendor group produces its own vendor bill and separate AP entry in QuickBooks</t>
+          <t>Verify Confirm Review signs off and completes the work order directly (no distinct Reviewed holding state)</t>
         </is>
       </c>
       <c r="F29" s="12" t="inlineStr">
@@ -9936,36 +9936,36 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G29" s="12" t="inlineStr">
-        <is>
-          <t>Blocked-Env</t>
+      <c r="G29" s="14" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="H29" s="12" t="inlineStr">
         <is>
-          <t>BUG-11</t>
+          <t>BUG-4</t>
         </is>
       </c>
       <c r="I29" s="12" t="inlineStr">
         <is>
-          <t>Blocked-Env (precise, confirmed live 2026-07-14): QuickBooks is NOT connected on the sv7301 QA org. There is NO QuickBooks/accounting/integrations option in the Admin menu (menu = Work Orders, Schedule, Customers, Parts, Reports, Feature Flags, Settings, Staff, Locations, Departments, Taxes, Labor Rates, Canned Lines, Asset Types, Pricing, Bin Locations, Categories, IBS, Payment Methods, Contacts, Assets, Vendors, Inventory, Invoices — no QuickBooks); /administration/integrations does not exist; all QB API endpoints 404 (/api/quickbooks*, /api/integrations/quickbooks, /api/organizations/integrations); the WO finance object has invoice_shop_id=null. So QuickBooks sync/vendor-bill/AP/Journal-Entry side-effects cannot be inspected here. Needs a QB-connected company + a human in QuickBooks.</t>
+          <t>Wording+VIU 2026-07-13 (S2-15823 live, Require Review ON): Mark Reviewed (VIN present) signs off and moves the WO directly Review -&gt; Complete; no distinct 'Reviewed' holding state and no separate final Complete click (S2-15823 went Review-&gt;Complete). | Δ5/R12 sanity clause added 2026-07-14 (review-ON last-line-resolve -&gt; Ready for Review; auto-complete trigger verified in SF-AUTO-05).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
         <is>
-          <t>C29388</t>
+          <t>C29394</t>
         </is>
       </c>
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29388</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29394</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>SF-REV-03</t>
+          <t>SF-REV-09</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -9975,12 +9975,12 @@
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>Verify the Details step collects only mileage and engine hours when review is on (VIN captured later by reviewer)</t>
+          <t>Verify Mark Reviewed is gated by the Review Work Orders permission and disabled for a role without it</t>
         </is>
       </c>
       <c r="F30" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G30" s="14" t="inlineStr">
@@ -9990,29 +9990,29 @@
       </c>
       <c r="H30" s="12" t="inlineStr">
         <is>
-          <t>BUG-8</t>
+          <t>BUG-5, BUG-7</t>
         </is>
       </c>
       <c r="I30" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: the completion Details modal shows Mileage + Engine Hours and no VIN field (confirmed live on the review-off modal S2-15827; review-on captures VIN in Mark Reviewed per SF-REV-06). Upgraded from Pending - the field set is now confirmed.</t>
+          <t>Wording+VIU 2026-07-13: Mark Reviewed gated by Review Work Orders (woReviewWorkOrders) per fresh roles matrix (roles-matrix-2026-07-13.md); role without it sees Mark Reviewed disabled + 'Awaiting review'; self-review allowed when the role holds the permission (Milos ruling). Review flow re-confirmed live.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>C29389</t>
+          <t>C29395</t>
         </is>
       </c>
       <c r="B31" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29389</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29395</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>SF-REV-04</t>
+          <t>SF-REV-10</t>
         </is>
       </c>
       <c r="D31" s="12" t="inlineStr">
@@ -10022,7 +10022,7 @@
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>Verify 'Receive Parts' routes to the shared receive page (no inline modal) in the review flow</t>
+          <t>Verify the Mark Reviewed dialog includes VIN / Serial # (required) with no review note field</t>
         </is>
       </c>
       <c r="F31" s="12" t="inlineStr">
@@ -10037,29 +10037,29 @@
       </c>
       <c r="H31" s="12" t="inlineStr">
         <is>
-          <t>BUG-11</t>
+          <t>BUG-3</t>
         </is>
       </c>
       <c r="I31" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: 'Receive Parts' opens the shared receive page (not an inline modal) in the review flow — verified prior drive (FV-rev04-receivestep/afterreceive.png, 2026-07-10); review flow re-confirmed live this run.</t>
+          <t>Wording+VIU 2026-07-13: Mark Reviewed uses VIN / Serial # only, no review note field (V2.4 Δ4 confirmed; SF-REV-06/10 were already note-free). Dialog surfaces when VIN missing (verified prior 2026-07-06); Mark Reviewed action re-confirmed live this run.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="12" t="inlineStr">
         <is>
-          <t>C29393</t>
+          <t>C29396</t>
         </is>
       </c>
       <c r="B32" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29393</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29396</t>
         </is>
       </c>
       <c r="C32" s="12" t="inlineStr">
         <is>
-          <t>SF-REV-08</t>
+          <t>SF-REV-11</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
@@ -10069,7 +10069,7 @@
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>Verify Confirm Review signs off and completes the work order directly (no distinct Reviewed holding state)</t>
+          <t>Verify sign-off completes the work order directly (no separate final Complete) and invoicing is blocked until reviewed</t>
         </is>
       </c>
       <c r="F32" s="12" t="inlineStr">
@@ -10077,9 +10077,9 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G32" s="14" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
+      <c r="G32" s="12" t="inlineStr">
+        <is>
+          <t>VIU-observed-awaiting-Milos</t>
         </is>
       </c>
       <c r="H32" s="12" t="inlineStr">
@@ -10089,24 +10089,24 @@
       </c>
       <c r="I32" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13 (S2-15823 live, Require Review ON): Mark Reviewed (VIN present) signs off and moves the WO directly Review -&gt; Complete; no distinct 'Reviewed' holding state and no separate final Complete click (S2-15823 went Review-&gt;Complete). | Δ5/R12 sanity clause added 2026-07-14 (review-ON last-line-resolve -&gt; Ready for Review; auto-complete trigger verified in SF-AUTO-05).</t>
+          <t>VIU-observed 2026-07-14 (awaiting Milos Q8). The direct-sign-off behavior is observed: Confirm Review signs off and completes the WO directly with no distinct 'Reviewed' holding state (see SF-REV-08). The 'invoicing blocked until reviewed' leg depends on the Q8 ruling about whether a separate Reviewed state should exist. No pass/fail asserted on the undecided policy. | Δ5/R12 sanity clause added 2026-07-14 (review-ON last-line-resolve -&gt; Ready for Review; auto-complete trigger verified in SF-AUTO-05).</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
         <is>
-          <t>C29394</t>
+          <t>C29399</t>
         </is>
       </c>
       <c r="B33" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29394</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29399</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
         <is>
-          <t>SF-REV-09</t>
+          <t>SF-REV-14</t>
         </is>
       </c>
       <c r="D33" s="12" t="inlineStr">
@@ -10116,54 +10116,54 @@
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
-          <t>Verify Mark Reviewed is gated by the Review Work Orders permission and disabled for a role without it</t>
+          <t>Verify cores are decided before receiving ahead of Send to Review, and invoicing stays blocked until Reviewed and every core is decided</t>
         </is>
       </c>
       <c r="F33" s="12" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G33" s="14" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G33" s="12" t="inlineStr">
+        <is>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="H33" s="12" t="inlineStr">
         <is>
-          <t>BUG-5, BUG-7</t>
+          <t>BUG-11</t>
         </is>
       </c>
       <c r="I33" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: Mark Reviewed gated by Review Work Orders (woReviewWorkOrders) per fresh roles matrix (roles-matrix-2026-07-13.md); role without it sees Mark Reviewed disabled + 'Awaiting review'; self-review allowed when the role holds the permission (Milos ruling). Review flow re-confirmed live.</t>
+          <t>REWORDED 2026-07-17 to spec `_4` (V2.6): the Story-16 core paragraph now reads 'Special-order cores (both required and optional) are pre-resolved before receiving on the resolve screen before Send to Review (no longer deferred to the invoice gate)' — the invoice-gate leg was dropped and the un-skippable/receive-first reading is replaced by gate-on-undecided (C-R4). Blocked-Env: a special-order (vendor-sourced) core is still not seedable in this build (P550848 is_core=0; a vendor-sourced part request drops the core attribute) — needs a dev-seeded special-order core. ALSO: Story 18 / SV-8353 is a new dev plan, so the pre-resolve build is likely NOT deployed on sv7301 yet — probe the completion wizard for the resolve step + the pre-resolve endpoint before any re-VIU.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="12" t="inlineStr">
         <is>
-          <t>C29395</t>
+          <t>C29406</t>
         </is>
       </c>
       <c r="B34" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29395</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29406</t>
         </is>
       </c>
       <c r="C34" s="12" t="inlineStr">
         <is>
-          <t>SF-REV-10</t>
+          <t>SF-PERM-02</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr">
         <is>
-          <t>Review ON (Story 16)</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>Verify the Mark Reviewed dialog includes VIN / Serial # (required) with no review note field</t>
+          <t>Verify which roles can complete a work order (Simple completion)</t>
         </is>
       </c>
       <c r="F34" s="12" t="inlineStr">
@@ -10178,86 +10178,86 @@
       </c>
       <c r="H34" s="12" t="inlineStr">
         <is>
-          <t>BUG-3</t>
+          <t>BUG-6</t>
         </is>
       </c>
       <c r="I34" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: Mark Reviewed uses VIN / Serial # only, no review note field (V2.4 Δ4 confirmed; SF-REV-06/10 were already note-free). Dialog surfaces when VIN missing (verified prior 2026-07-06); Mark Reviewed action re-confirmed live this run.</t>
+          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Complete-WO gate = workOrdersCreateAndEdit; roles that can complete (Admin, Service Manager, Senior SA, Service Advisor, Foreman, Parts Manager) vs cannot (Technician, Parts Tech, Office, Sales Rep, Time Clock) match the matrix. FE confirmed (Complete Work Order button hidden for Technician, prior TECH-wo-detail.png); BE does not enforce WO completion (documented gap, see SF-PERM-06).</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="12" t="inlineStr">
         <is>
-          <t>C29396</t>
+          <t>C29408</t>
         </is>
       </c>
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29396</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29408</t>
         </is>
       </c>
       <c r="C35" s="12" t="inlineStr">
         <is>
-          <t>SF-REV-11</t>
+          <t>SF-PERM-04</t>
         </is>
       </c>
       <c r="D35" s="12" t="inlineStr">
         <is>
-          <t>Review ON (Story 16)</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="E35" s="12" t="inlineStr">
         <is>
-          <t>Verify sign-off completes the work order directly (no separate final Complete) and invoicing is blocked until reviewed</t>
+          <t>Verify which roles can Mark Reviewed (sign off)</t>
         </is>
       </c>
       <c r="F35" s="12" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G35" s="12" t="inlineStr">
-        <is>
-          <t>VIU-observed-awaiting-Milos</t>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G35" s="14" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="H35" s="12" t="inlineStr">
         <is>
-          <t>BUG-4</t>
+          <t>BUG-5</t>
         </is>
       </c>
       <c r="I35" s="12" t="inlineStr">
         <is>
-          <t>VIU-observed 2026-07-14 (awaiting Milos Q8). The direct-sign-off behavior is observed: Confirm Review signs off and completes the WO directly with no distinct 'Reviewed' holding state (see SF-REV-08). The 'invoicing blocked until reviewed' leg depends on the Q8 ruling about whether a separate Reviewed state should exist. No pass/fail asserted on the undecided policy. | Δ5/R12 sanity clause added 2026-07-14 (review-ON last-line-resolve -&gt; Ready for Review; auto-complete trigger verified in SF-AUTO-05).</t>
+          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Mark Reviewed gate = woReviewWorkOrders (not open-to-all). Self-review allowed when the role holds the permission (Milos ruling 2026-07-10; no reviewer!=completer identity block). Per-role has/lacks matches the matrix.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="12" t="inlineStr">
         <is>
-          <t>C29399</t>
+          <t>C29410</t>
         </is>
       </c>
       <c r="B36" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29399</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29410</t>
         </is>
       </c>
       <c r="C36" s="12" t="inlineStr">
         <is>
-          <t>SF-REV-14</t>
+          <t>SF-PERM-06</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
         <is>
-          <t>Review ON (Story 16)</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Verify cores are decided before receiving ahead of Send to Review, and invoicing stays blocked until Reviewed and every core is decided</t>
+          <t>Verify permission gating of Simple-Flow settings and work-order actions (UI gating is the v1 pass criterion)</t>
         </is>
       </c>
       <c r="F36" s="12" t="inlineStr">
@@ -10265,36 +10265,36 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="G36" s="12" t="inlineStr">
-        <is>
-          <t>Blocked-Env</t>
+      <c r="G36" s="14" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="H36" s="12" t="inlineStr">
         <is>
-          <t>BUG-11</t>
+          <t>BUG-6</t>
         </is>
       </c>
       <c r="I36" s="12" t="inlineStr">
         <is>
-          <t>REWORDED 2026-07-17 to spec `_4` (V2.6): the Story-16 core paragraph now reads 'Special-order cores (both required and optional) are pre-resolved before receiving on the resolve screen before Send to Review (no longer deferred to the invoice gate)' — the invoice-gate leg was dropped and the un-skippable/receive-first reading is replaced by gate-on-undecided (C-R4). Blocked-Env: a special-order (vendor-sourced) core is still not seedable in this build (P550848 is_core=0; a vendor-sourced part request drops the core attribute) — needs a dev-seeded special-order core. ALSO: Story 18 / SV-8353 is a new dev plan, so the pre-resolve build is likely NOT deployed on sv7301 yet — probe the completion wizard for the resolve step + the pre-resolve endpoint before any re-VIU.</t>
+          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Live: BE enforces the distinct settings atom (Technician settings save -&gt; 403, Admin -&gt; 200) but does NOT enforce the WO-completion / review atoms (documented 'app blocks / backend allows' gap, draft TICKET 2). v1 pass = app-level restriction (Milos Round-2 ruling). Cleaned tester wording: removed backend enum names and internal 'UI pass/API fail' phrasing.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="12" t="inlineStr">
         <is>
-          <t>C29406</t>
+          <t>C29411</t>
         </is>
       </c>
       <c r="B37" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29406</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29411</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr">
         <is>
-          <t>SF-PERM-02</t>
+          <t>SF-PERM-07</t>
         </is>
       </c>
       <c r="D37" s="12" t="inlineStr">
@@ -10304,12 +10304,12 @@
       </c>
       <c r="E37" s="12" t="inlineStr">
         <is>
-          <t>Verify which roles can complete a work order (Simple completion)</t>
+          <t>Verify review sign-off is governed by the Review Work Orders custom-role permission (not open to all)</t>
         </is>
       </c>
       <c r="F37" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G37" s="14" t="inlineStr">
@@ -10319,29 +10319,29 @@
       </c>
       <c r="H37" s="12" t="inlineStr">
         <is>
-          <t>BUG-6</t>
+          <t>BUG-5, BUG-7</t>
         </is>
       </c>
       <c r="I37" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Complete-WO gate = workOrdersCreateAndEdit; roles that can complete (Admin, Service Manager, Senior SA, Service Advisor, Foreman, Parts Manager) vs cannot (Technician, Parts Tech, Office, Sales Rep, Time Clock) match the matrix. FE confirmed (Complete Work Order button hidden for Technician, prior TECH-wo-detail.png); BE does not enforce WO completion (documented gap, see SF-PERM-06).</t>
+          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Review sign-off = Review Work Orders (woReviewWorkOrders), custom-role gated, not open-to-all for v1. Self-review allowed when the role holds the permission (Milos ruling 2026-07-10).</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="12" t="inlineStr">
         <is>
-          <t>C29408</t>
+          <t>C29412</t>
         </is>
       </c>
       <c r="B38" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29408</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29412</t>
         </is>
       </c>
       <c r="C38" s="12" t="inlineStr">
         <is>
-          <t>SF-PERM-04</t>
+          <t>SF-PERM-08</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
@@ -10351,12 +10351,12 @@
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
-          <t>Verify which roles can Mark Reviewed (sign off)</t>
+          <t>Verify a user who holds the Mark Reviewed permission can Mark Reviewed a work order they completed</t>
         </is>
       </c>
       <c r="F38" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G38" s="14" t="inlineStr">
@@ -10371,39 +10371,39 @@
       </c>
       <c r="I38" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Mark Reviewed gate = woReviewWorkOrders (not open-to-all). Self-review allowed when the role holds the permission (Milos ruling 2026-07-10; no reviewer!=completer identity block). Per-role has/lacks matches the matrix.</t>
+          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Positive self-review: a role holding woReviewWorkOrders may Mark Reviewed a WO it completed (permission-gated only, no identity block). A role lacking it cannot. Matches matrix + Milos ruling.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="12" t="inlineStr">
         <is>
-          <t>C29410</t>
+          <t>C29415</t>
         </is>
       </c>
       <c r="B39" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29410</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29415</t>
         </is>
       </c>
       <c r="C39" s="12" t="inlineStr">
         <is>
-          <t>SF-PERM-06</t>
+          <t>SF-VAL-01</t>
         </is>
       </c>
       <c r="D39" s="12" t="inlineStr">
         <is>
-          <t>Permissions</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="E39" s="12" t="inlineStr">
         <is>
-          <t>Verify permission gating of Simple-Flow settings and work-order actions (UI gating is the v1 pass criterion)</t>
+          <t>Verify completion is blocked when required mileage is missing</t>
         </is>
       </c>
       <c r="F39" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G39" s="14" t="inlineStr">
@@ -10413,91 +10413,91 @@
       </c>
       <c r="H39" s="12" t="inlineStr">
         <is>
-          <t>BUG-6</t>
+          <t>BUG-8</t>
         </is>
       </c>
       <c r="I39" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Live: BE enforces the distinct settings atom (Technician settings save -&gt; 403, Admin -&gt; 200) but does NOT enforce the WO-completion / review atoms (documented 'app blocks / backend allows' gap, draft TICKET 2). v1 pass = app-level restriction (Milos Round-2 ruling). Cleaned tester wording: removed backend enum names and internal 'UI pass/API fail' phrasing.</t>
+          <t>Wording+VIU 2026-07-13 (S2-15783 live, Require Mileage ON): the completion Details modal shows a Mileage field; leaving it empty and pressing 'Complete Work Order' shows a 'required field' error and completion does not proceed. Settings restored byte-identical.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="12" t="inlineStr">
         <is>
-          <t>C29411</t>
+          <t>C29416</t>
         </is>
       </c>
       <c r="B40" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29411</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29416</t>
         </is>
       </c>
       <c r="C40" s="12" t="inlineStr">
         <is>
-          <t>SF-PERM-07</t>
+          <t>SF-VAL-02</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
         <is>
-          <t>Permissions</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Verify review sign-off is governed by the Review Work Orders custom-role permission (not open to all)</t>
+          <t>Verify completion is blocked when a required VIN is missing (non-review No-PO / Optional-invoice flow)</t>
         </is>
       </c>
       <c r="F40" s="12" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="G40" s="14" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G40" s="12" t="inlineStr">
+        <is>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="H40" s="12" t="inlineStr">
         <is>
-          <t>BUG-5, BUG-7</t>
+          <t>BUG-8</t>
         </is>
       </c>
       <c r="I40" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Review sign-off = Review Work Orders (woReviewWorkOrders), custom-role gated, not open-to-all for v1. Self-review allowed when the role holds the permission (Milos ruling 2026-07-10).</t>
+          <t>Blocked-Env (precise, investigated live 2026-07-14): a VIN-less asset cannot be seeded. Asset/vehicle creation is not exposed via API (POST /api/assets 404, POST /api/vehicles 405 GET-only, POST /api/company-vehicles 404) and the new-asset UI flow requires a VIN; all existing assets already carry a VIN. So the non-review No-PO/Optional-invoice completion cannot be driven into a VIN-missing prompt. (Also note the Story-4 completion modal no longer carries a VIN field per Delta1 — SF-COMP-16.) Needs a VIN-less asset seeded by dev/data.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="12" t="inlineStr">
         <is>
-          <t>C29412</t>
+          <t>C29417</t>
         </is>
       </c>
       <c r="B41" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29412</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29417</t>
         </is>
       </c>
       <c r="C41" s="12" t="inlineStr">
         <is>
-          <t>SF-PERM-08</t>
+          <t>SF-VAL-03</t>
         </is>
       </c>
       <c r="D41" s="12" t="inlineStr">
         <is>
-          <t>Permissions</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="E41" s="12" t="inlineStr">
         <is>
-          <t>Verify a user who holds the Mark Reviewed permission can Mark Reviewed a work order they completed</t>
+          <t>Verify completion is blocked when required engine hours are missing</t>
         </is>
       </c>
       <c r="F41" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G41" s="14" t="inlineStr">
@@ -10507,29 +10507,29 @@
       </c>
       <c r="H41" s="12" t="inlineStr">
         <is>
-          <t>BUG-5</t>
+          <t>BUG-8</t>
         </is>
       </c>
       <c r="I41" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Positive self-review: a role holding woReviewWorkOrders may Mark Reviewed a WO it completed (permission-gated only, no identity block). A role lacking it cannot. Matches matrix + Milos ruling.</t>
+          <t>Wording+VIU 2026-07-13 (S2-15783 live, Require Engine Hours ON): the completion Details modal shows an Engine Hours field; empty -&gt; 'required field' error, completion blocked. Same modal as SF-VAL-01 (Mileage + Engine Hours).</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="12" t="inlineStr">
         <is>
-          <t>C29415</t>
+          <t>C29419</t>
         </is>
       </c>
       <c r="B42" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29415</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29419</t>
         </is>
       </c>
       <c r="C42" s="12" t="inlineStr">
         <is>
-          <t>SF-VAL-01</t>
+          <t>SF-VAL-05</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
@@ -10539,7 +10539,7 @@
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Verify completion is blocked when required mileage is missing</t>
+          <t>Verify a required-invoice receive is blocked without a vendor invoice number</t>
         </is>
       </c>
       <c r="F42" s="12" t="inlineStr">
@@ -10554,29 +10554,29 @@
       </c>
       <c r="H42" s="12" t="inlineStr">
         <is>
-          <t>BUG-8</t>
+          <t>BUG-11</t>
         </is>
       </c>
       <c r="I42" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13 (S2-15783 live, Require Mileage ON): the completion Details modal shows a Mileage field; leaving it empty and pressing 'Complete Work Order' shows a 'required field' error and completion does not proceed. Settings restored byte-identical.</t>
+          <t>Wording+VIU 2026-07-13: required-invoice receive blocked without a vendor invoice number - verified prior drive (FV-val05-noinvoice/withinvoice.png, 2026-07-10). Require Vendor Invoice Number gate.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="12" t="inlineStr">
         <is>
-          <t>C29416</t>
+          <t>C29420</t>
         </is>
       </c>
       <c r="B43" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29416</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29420</t>
         </is>
       </c>
       <c r="C43" s="12" t="inlineStr">
         <is>
-          <t>SF-VAL-02</t>
+          <t>SF-VAL-06</t>
         </is>
       </c>
       <c r="D43" s="12" t="inlineStr">
@@ -10586,551 +10586,410 @@
       </c>
       <c r="E43" s="12" t="inlineStr">
         <is>
-          <t>Verify completion is blocked when a required VIN is missing (non-review No-PO / Optional-invoice flow)</t>
+          <t>Verify a vendor-missing part cannot be received without a vendor, a part number, and a cost / sell price</t>
         </is>
       </c>
       <c r="F43" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G43" s="12" t="inlineStr">
-        <is>
-          <t>Blocked-Env</t>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G43" s="14" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="H43" s="12" t="inlineStr">
         <is>
-          <t>BUG-8</t>
+          <t>BUG-11</t>
         </is>
       </c>
       <c r="I43" s="12" t="inlineStr">
         <is>
-          <t>Blocked-Env (precise, investigated live 2026-07-14): a VIN-less asset cannot be seeded. Asset/vehicle creation is not exposed via API (POST /api/assets 404, POST /api/vehicles 405 GET-only, POST /api/company-vehicles 404) and the new-asset UI flow requires a VIN; all existing assets already carry a VIN. So the non-review No-PO/Optional-invoice completion cannot be driven into a VIN-missing prompt. (Also note the Story-4 completion modal no longer carries a VIN field per Delta1 — SF-COMP-16.) Needs a VIN-less asset seeded by dev/data.</t>
+          <t>VIU-Verified live 2026-07-14 on the Bulk Receive page (/bulk-receive) with a freshly seeded vendor-missing WO PO (S-15845, order 0ee75c5f, part 'Gear oil' no PN/no vendor/cost=sell=0). Receive-button gate progression confirmed: no vendor -&gt; Receive DISABLED; vendor assigned (POST /api/orders/{id}/assign-vendor 200, auto-assigned with NO merge prompt, vendor-missing flag cleared) but no part number -&gt; DISABLED; part number entered but cost/sell still 0 -&gt; DISABLED; part number + vendor invoice number + cost + sell all present -&gt; Receive ENABLED (receivable). Confirms a vendor-missing part cannot be received without a vendor, a part number, and a cost/sell price.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="12" t="inlineStr">
         <is>
-          <t>C29417</t>
+          <t>C29427</t>
         </is>
       </c>
       <c r="B44" s="13" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29417</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29427</t>
         </is>
       </c>
       <c r="C44" s="12" t="inlineStr">
         <is>
-          <t>SF-VAL-03</t>
+          <t>SF-QB-02</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
         <is>
-          <t>Validation / Edge</t>
+          <t>QuickBooks / Inventory Integrity</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>Verify completion is blocked when required engine hours are missing</t>
+          <t>Verify Create POs OFF produces no PO, vendor bill or AP sync and no catalog/inventory sync</t>
         </is>
       </c>
       <c r="F44" s="12" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G44" s="12" t="inlineStr">
+        <is>
+          <t>VIU-observed-awaiting-Milos</t>
+        </is>
+      </c>
+      <c r="H44" s="12" t="inlineStr">
+        <is>
+          <t>BUG-1</t>
+        </is>
+      </c>
+      <c r="I44" s="12" t="inlineStr">
+        <is>
+          <t>VIU-observed 2026-07-14 (awaiting Milos Q5) AND QB-blocked. The 'Create Purchase Orders' toggle is absent (POs always-on, SF-SET-03 Deviation) so the Create-POs-OFF scenario cannot be configured; and QuickBooks is not connected on sv7301 (no QB admin/API — see bugs-log) so QB integrity cannot be inspected regardless. Milos Q5 governs whether POs-always-on is intended. No pass/fail asserted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="17" t="inlineStr">
+        <is>
+          <t>Bug / Deviation Register</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>BUG-#</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Affected cases</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="12" t="inlineStr">
+        <is>
+          <t>BUG-1</t>
+        </is>
+      </c>
+      <c r="B48" s="12" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G44" s="14" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="H44" s="12" t="inlineStr">
-        <is>
-          <t>BUG-8</t>
-        </is>
-      </c>
-      <c r="I44" s="12" t="inlineStr">
-        <is>
-          <t>Wording+VIU 2026-07-13 (S2-15783 live, Require Engine Hours ON): the completion Details modal shows an Engine Hours field; empty -&gt; 'required field' error, completion blocked. Same modal as SF-VAL-01 (Mileage + Engine Hours).</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="12" t="inlineStr">
-        <is>
-          <t>C29419</t>
-        </is>
-      </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29419</t>
-        </is>
-      </c>
-      <c r="C45" s="12" t="inlineStr">
-        <is>
-          <t>SF-VAL-05</t>
-        </is>
-      </c>
-      <c r="D45" s="12" t="inlineStr">
-        <is>
-          <t>Validation / Edge</t>
-        </is>
-      </c>
-      <c r="E45" s="12" t="inlineStr">
-        <is>
-          <t>Verify a required-invoice receive is blocked without a vendor invoice number</t>
-        </is>
-      </c>
-      <c r="F45" s="12" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G45" s="14" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="H45" s="12" t="inlineStr">
-        <is>
-          <t>BUG-11</t>
-        </is>
-      </c>
-      <c r="I45" s="12" t="inlineStr">
-        <is>
-          <t>Wording+VIU 2026-07-13: required-invoice receive blocked without a vendor invoice number - verified prior drive (FV-val05-noinvoice/withinvoice.png, 2026-07-10). Require Vendor Invoice Number gate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="12" t="inlineStr">
-        <is>
-          <t>C29420</t>
-        </is>
-      </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29420</t>
-        </is>
-      </c>
-      <c r="C46" s="12" t="inlineStr">
-        <is>
-          <t>SF-VAL-06</t>
-        </is>
-      </c>
-      <c r="D46" s="12" t="inlineStr">
-        <is>
-          <t>Validation / Edge</t>
-        </is>
-      </c>
-      <c r="E46" s="12" t="inlineStr">
-        <is>
-          <t>Verify a vendor-missing part cannot be received without a vendor, a part number, and a cost / sell price</t>
-        </is>
-      </c>
-      <c r="F46" s="12" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G46" s="14" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="H46" s="12" t="inlineStr">
-        <is>
-          <t>BUG-11</t>
-        </is>
-      </c>
-      <c r="I46" s="12" t="inlineStr">
-        <is>
-          <t>VIU-Verified live 2026-07-14 on the Bulk Receive page (/bulk-receive) with a freshly seeded vendor-missing WO PO (S-15845, order 0ee75c5f, part 'Gear oil' no PN/no vendor/cost=sell=0). Receive-button gate progression confirmed: no vendor -&gt; Receive DISABLED; vendor assigned (POST /api/orders/{id}/assign-vendor 200, auto-assigned with NO merge prompt, vendor-missing flag cleared) but no part number -&gt; DISABLED; part number entered but cost/sell still 0 -&gt; DISABLED; part number + vendor invoice number + cost + sell all present -&gt; Receive ENABLED (receivable). Confirms a vendor-missing part cannot be received without a vendor, a part number, and a cost/sell price.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="12" t="inlineStr">
-        <is>
-          <t>C29427</t>
-        </is>
-      </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29427</t>
-        </is>
-      </c>
-      <c r="C47" s="12" t="inlineStr">
-        <is>
-          <t>SF-QB-02</t>
-        </is>
-      </c>
-      <c r="D47" s="12" t="inlineStr">
-        <is>
-          <t>QuickBooks / Inventory Integrity</t>
-        </is>
-      </c>
-      <c r="E47" s="12" t="inlineStr">
-        <is>
-          <t>Verify Create POs OFF produces no PO, vendor bill or AP sync and no catalog/inventory sync</t>
-        </is>
-      </c>
-      <c r="F47" s="12" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G47" s="12" t="inlineStr">
-        <is>
-          <t>VIU-observed-awaiting-Milos</t>
-        </is>
-      </c>
-      <c r="H47" s="12" t="inlineStr">
-        <is>
-          <t>BUG-1</t>
-        </is>
-      </c>
-      <c r="I47" s="12" t="inlineStr">
-        <is>
-          <t>VIU-observed 2026-07-14 (awaiting Milos Q5) AND QB-blocked. The 'Create Purchase Orders' toggle is absent (POs always-on, SF-SET-03 Deviation) so the Create-POs-OFF scenario cannot be configured; and QuickBooks is not connected on sv7301 (no QB admin/API — see bugs-log) so QB integrity cannot be inspected regardless. Milos Q5 governs whether POs-always-on is intended. No pass/fail asserted.</t>
+      <c r="C48" s="18" t="inlineStr">
+        <is>
+          <t>OPEN (build-lag / Open Q5)</t>
+        </is>
+      </c>
+      <c r="D48" s="12" t="inlineStr">
+        <is>
+          <t>No 'Create Purchase Orders' toggle / no createPurchaseOrders field — POs always-on. V2.4 retains the No-PO path, so this is a spec-vs-build gap (build lags V2.4), not a descope.</t>
+        </is>
+      </c>
+      <c r="E48" s="12" t="inlineStr">
+        <is>
+          <t>SF-SET-03, SF-COMP-06, SF-QB-02</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="17" t="inlineStr">
-        <is>
-          <t>Bug / Deviation Register</t>
+      <c r="A49" s="12" t="inlineStr">
+        <is>
+          <t>BUG-2</t>
+        </is>
+      </c>
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C49" s="18" t="inlineStr">
+        <is>
+          <t>OPEN (Open Q6)</t>
+        </is>
+      </c>
+      <c r="D49" s="12" t="inlineStr">
+        <is>
+          <t>Save Settings button always enabled (no dirty-state gating).</t>
+        </is>
+      </c>
+      <c r="E49" s="12" t="inlineStr">
+        <is>
+          <t>SF-SET-13</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="5" t="inlineStr">
-        <is>
-          <t>BUG-#</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>Severity</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>Affected cases</t>
+      <c r="A50" s="12" t="inlineStr">
+        <is>
+          <t>BUG-3</t>
+        </is>
+      </c>
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C50" s="14" t="inlineStr">
+        <is>
+          <t>CLOSED — NOT A BUG (Milos Round-2, 2026-07-09)</t>
+        </is>
+      </c>
+      <c r="D50" s="12" t="inlineStr">
+        <is>
+          <t>Mark-Reviewed dialog has no optional review note. Milos removed the note from the design; v1 is VIN-only. SF-REV-10 expected updated to VIN-only — live now matches.</t>
+        </is>
+      </c>
+      <c r="E50" s="12" t="inlineStr">
+        <is>
+          <t>SF-REV-10</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="12" t="inlineStr">
         <is>
-          <t>BUG-1</t>
+          <t>BUG-4</t>
         </is>
       </c>
       <c r="B51" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="C51" s="18" t="inlineStr">
-        <is>
-          <t>OPEN (build-lag / Open Q5)</t>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C51" s="14" t="inlineStr">
+        <is>
+          <t>RECLASSIFIED → EXPECTED (shortcut principle, 2026-07-08)</t>
         </is>
       </c>
       <c r="D51" s="12" t="inlineStr">
         <is>
-          <t>No 'Create Purchase Orders' toggle / no createPurchaseOrders field — POs always-on. V2.4 retains the No-PO path, so this is a spec-vs-build gap (build lags V2.4), not a descope.</t>
+          <t>Review sign-off jumps Review → Complete with no distinct 'Reviewed' holding state. A skipped intermediate state reaching the same end state with no error/corruption = expected.</t>
         </is>
       </c>
       <c r="E51" s="12" t="inlineStr">
         <is>
-          <t>SF-SET-03, SF-COMP-06, SF-QB-02</t>
+          <t>SF-REV-08, SF-REV-11</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="12" t="inlineStr">
         <is>
-          <t>BUG-2</t>
+          <t>BUG-5</t>
         </is>
       </c>
       <c r="B52" s="12" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="C52" s="18" t="inlineStr">
         <is>
-          <t>OPEN (Open Q6)</t>
+          <t>OPEN (needs dev/PO ruling)</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
         <is>
-          <t>Save Settings button always enabled (no dirty-state gating).</t>
+          <t>reviewer != completer rule NOT enforced — a user can Mark-Reviewed (sign off) their own completed / sent-to-review WO. The one net-new Simple-Flow permission rule is missing.</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
         <is>
-          <t>SF-SET-13</t>
+          <t>SF-PERM-08, SF-PERM-04, SF-PERM-07, SF-REV-09</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="12" t="inlineStr">
         <is>
-          <t>BUG-3</t>
+          <t>BUG-6</t>
         </is>
       </c>
       <c r="B53" s="12" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="C53" s="14" t="inlineStr">
-        <is>
-          <t>CLOSED — NOT A BUG (Milos Round-2, 2026-07-09)</t>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C53" s="18" t="inlineStr">
+        <is>
+          <t>OPEN — API gap (v1 ruling: UI gating = PASS; API fix ticket)</t>
         </is>
       </c>
       <c r="D53" s="12" t="inlineStr">
         <is>
-          <t>Mark-Reviewed dialog has no optional review note. Milos removed the note from the design; v1 is VIN-only. SF-REV-10 expected updated to VIN-only — live now matches.</t>
+          <t>WO-completion permission is FE-only at the backend: a Technician (no workOrdersCreateAndEdit) can complete a WO via simple-complete API (201). FE hides the button; BE does not enforce (SV-7864 atom-collapse). Ruling 2026-07-09: record 'UI pass / API fail'.</t>
         </is>
       </c>
       <c r="E53" s="12" t="inlineStr">
         <is>
-          <t>SF-REV-10</t>
+          <t>SF-PERM-06, SF-PERM-02</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="12" t="inlineStr">
         <is>
-          <t>BUG-4</t>
+          <t>BUG-7</t>
         </is>
       </c>
       <c r="B54" s="12" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="C54" s="14" t="inlineStr">
-        <is>
-          <t>RECLASSIFIED → EXPECTED (shortcut principle, 2026-07-08)</t>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C54" s="18" t="inlineStr">
+        <is>
+          <t>OPEN — API gap (v1 ruling: UI gating = PASS; API fix ticket)</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr">
         <is>
-          <t>Review sign-off jumps Review → Complete with no distinct 'Reviewed' holding state. A skipped intermediate state reaching the same end state with no error/corruption = expected.</t>
+          <t>Review sign-off permission (woReviewWorkOrders) is FE-only at the backend: a Technician can drive review→complete change-status (201). Same FE-vs-BE ruling as BUG-6.</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
         <is>
-          <t>SF-REV-08, SF-REV-11</t>
+          <t>SF-PERM-07, SF-REV-09</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="12" t="inlineStr">
         <is>
-          <t>BUG-5</t>
+          <t>BUG-8</t>
         </is>
       </c>
       <c r="B55" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="C55" s="18" t="inlineStr">
         <is>
-          <t>OPEN (needs dev/PO ruling)</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="D55" s="12" t="inlineStr">
         <is>
-          <t>reviewer != completer rule NOT enforced — a user can Mark-Reviewed (sign off) their own completed / sent-to-review WO. The one net-new Simple-Flow permission rule is missing.</t>
+          <t>Mileage / VIN / engine-hours completion gates are FE-only (the simple-complete endpoint does not enforce them; only the wizard does). UI-level blocks are real; BE non-enforcement is the deviation. (Tech-story + all-lines-approved gates ARE BE-enforced.)</t>
         </is>
       </c>
       <c r="E55" s="12" t="inlineStr">
         <is>
-          <t>SF-PERM-08, SF-PERM-04, SF-PERM-07, SF-REV-09</t>
+          <t>SF-VAL-01, SF-VAL-02, SF-VAL-03, SF-COMP-05, SF-COMP-16, SF-REV-03</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="12" t="inlineStr">
         <is>
-          <t>BUG-6</t>
+          <t>BUG-9</t>
         </is>
       </c>
       <c r="B56" s="12" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="C56" s="18" t="inlineStr">
-        <is>
-          <t>OPEN — API gap (v1 ruling: UI gating = PASS; API fix ticket)</t>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C56" s="14" t="inlineStr">
+        <is>
+          <t>CLOSED — INTENDED (Milos Round-2, 2026-07-09)</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
         <is>
-          <t>WO-completion permission is FE-only at the backend: a Technician (no workOrdersCreateAndEdit) can complete a WO via simple-complete API (201). FE hides the button; BE does not enforce (SV-7864 atom-collapse). Ruling 2026-07-09: record 'UI pass / API fail'.</t>
+          <t>Vendorless 'New Part Request' requires a Category and does not enforce Sell Price. Milos ruled current behavior is expected for v1 (Category required; Sell optional). SF-VPART-01/02 expected updated accordingly.</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
         <is>
-          <t>SF-PERM-06, SF-PERM-02</t>
+          <t>SF-VPART-01, SF-VPART-02</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="12" t="inlineStr">
         <is>
-          <t>BUG-7</t>
+          <t>BUG-10</t>
         </is>
       </c>
       <c r="B57" s="12" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="C57" s="18" t="inlineStr">
-        <is>
-          <t>OPEN — API gap (v1 ruling: UI gating = PASS; API fix ticket)</t>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C57" s="14" t="inlineStr">
+        <is>
+          <t>RECLASSIFIED → EXPECTED (shortcut principle, 2026-07-08)</t>
         </is>
       </c>
       <c r="D57" s="12" t="inlineStr">
         <is>
-          <t>Review sign-off permission (woReviewWorkOrders) is FE-only at the backend: a Technician can drive review→complete change-status (201). Same FE-vs-BE ruling as BUG-6.</t>
+          <t>No distinct 'Resolve Cores' step in the completion wizard for an inventory core — resolution is a line-level Ok/Not-OK control; wizard goes Details→Success (no error/corruption). Receive-dependent special-order-core paths remain blocked by BUG-11.</t>
         </is>
       </c>
       <c r="E57" s="12" t="inlineStr">
         <is>
-          <t>SF-PERM-07, SF-REV-09</t>
+          <t>SF-CORE-01, SF-CORE-02, SF-CORE-03, SF-CORE-04, SF-CORE-05, SF-CORE-06, SF-CORE-07, SF-CORE-08, SF-CORE-09, SF-CORE-10</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="12" t="inlineStr">
         <is>
-          <t>BUG-8</t>
+          <t>BUG-11</t>
         </is>
       </c>
       <c r="B58" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High → Low</t>
         </is>
       </c>
       <c r="C58" s="18" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN — workaround exists (Bulk Receive path works)</t>
         </is>
       </c>
       <c r="D58" s="12" t="inlineStr">
         <is>
-          <t>Mileage / VIN / engine-hours completion gates are FE-only (the simple-complete endpoint does not enforce them; only the wizard does). UI-level blocks are real; BE non-enforcement is the deviation. (Tech-story + all-lines-approved gates ARE BE-enforced.)</t>
+          <t>WO-originated PO receive returns HTTP 500 on the LEGACY Accept-Delivery path (POST /api/inventory/orders/accept). The new Bulk Receive pipeline (receive-requested-parts) works (200), so the round-trip is achievable there; the legacy single-PO Accept-Delivery 500 should still be fixed.</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
         <is>
-          <t>SF-VAL-01, SF-VAL-02, SF-VAL-03, SF-COMP-05, SF-COMP-16, SF-REV-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="12" t="inlineStr">
-        <is>
-          <t>BUG-9</t>
-        </is>
-      </c>
-      <c r="B59" s="12" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="C59" s="14" t="inlineStr">
-        <is>
-          <t>CLOSED — INTENDED (Milos Round-2, 2026-07-09)</t>
-        </is>
-      </c>
-      <c r="D59" s="12" t="inlineStr">
-        <is>
-          <t>Vendorless 'New Part Request' requires a Category and does not enforce Sell Price. Milos ruled current behavior is expected for v1 (Category required; Sell optional). SF-VPART-01/02 expected updated accordingly.</t>
-        </is>
-      </c>
-      <c r="E59" s="12" t="inlineStr">
-        <is>
-          <t>SF-VPART-01, SF-VPART-02</t>
+          <t>SF-COMP-13, SF-COMP-19, SF-VAL-05, SF-VAL-06, SF-PNFIX-02, SF-PNFIX-03, SF-PNFIX-04, SF-PNFIX-05, SF-PNFIX-06, SF-RCV-08, SF-VPART-07, SF-REV-04, SF-REV-14, SF-CORE-03, SF-CORE-04, SF-CORE-05, SF-CORE-06, SF-CORE-07</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="12" t="inlineStr">
-        <is>
-          <t>BUG-10</t>
-        </is>
-      </c>
-      <c r="B60" s="12" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="C60" s="14" t="inlineStr">
-        <is>
-          <t>RECLASSIFIED → EXPECTED (shortcut principle, 2026-07-08)</t>
-        </is>
-      </c>
-      <c r="D60" s="12" t="inlineStr">
-        <is>
-          <t>No distinct 'Resolve Cores' step in the completion wizard for an inventory core — resolution is a line-level Ok/Not-OK control; wizard goes Details→Success (no error/corruption). Receive-dependent special-order-core paths remain blocked by BUG-11.</t>
-        </is>
-      </c>
-      <c r="E60" s="12" t="inlineStr">
-        <is>
-          <t>SF-CORE-01, SF-CORE-02, SF-CORE-03, SF-CORE-04, SF-CORE-05, SF-CORE-06, SF-CORE-07, SF-CORE-08, SF-CORE-09, SF-CORE-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="12" t="inlineStr">
-        <is>
-          <t>BUG-11</t>
-        </is>
-      </c>
-      <c r="B61" s="12" t="inlineStr">
-        <is>
-          <t>High → Low</t>
-        </is>
-      </c>
-      <c r="C61" s="18" t="inlineStr">
-        <is>
-          <t>OPEN — workaround exists (Bulk Receive path works)</t>
-        </is>
-      </c>
-      <c r="D61" s="12" t="inlineStr">
-        <is>
-          <t>WO-originated PO receive returns HTTP 500 on the LEGACY Accept-Delivery path (POST /api/inventory/orders/accept). The new Bulk Receive pipeline (receive-requested-parts) works (200), so the round-trip is achievable there; the legacy single-PO Accept-Delivery 500 should still be fixed.</t>
-        </is>
-      </c>
-      <c r="E61" s="12" t="inlineStr">
-        <is>
-          <t>SF-COMP-13, SF-COMP-19, SF-VAL-05, SF-VAL-06, SF-PNFIX-02, SF-PNFIX-03, SF-PNFIX-04, SF-PNFIX-05, SF-PNFIX-06, SF-RCV-08, SF-VPART-07, SF-REV-04, SF-REV-14, SF-CORE-03, SF-CORE-04, SF-CORE-05, SF-CORE-06, SF-CORE-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="19" t="inlineStr">
+      <c r="A60" s="19" t="inlineStr">
         <is>
           <t>Note: BUG-5/6/7/8/11 are OPEN (BUG-6/7 carry a v1 'UI-pass / API-fail' ruling; BUG-11 has a working Bulk-Receive path). BUG-3 and BUG-9 are CLOSED (Milos Round-2: review-note descoped; Category-required/Sell-optional intended). BUG-4 and BUG-10 are reclassified EXPECTED under the shortcut principle.</t>
         </is>
@@ -11179,9 +11038,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B42" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B43" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId44"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Simple Flow: SV-8183 optional regression edits — SF-PERM-06 (accept per-role enforcement) + SF-PERM-12 (Rule-24 API-flag notes)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_Results.xlsx
+++ b/build/simple-flow/SimpleFlow_Results.xlsx
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C17" s="2" t="n"/>
     </row>
@@ -743,12 +743,12 @@
           <t>Cases with NO TestRail ID (blank)</t>
         </is>
       </c>
-      <c r="B18" s="9" t="n">
-        <v>2</v>
+      <c r="B18" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Blank: SF-PERM-11, SF-PERM-12 — add after the next TestRail sync (IDs not guessed).</t>
+          <t>All authored cases have a TestRail ID (C&lt;id&gt;) + view link.</t>
         </is>
       </c>
     </row>
@@ -7329,7 +7329,7 @@
       </c>
       <c r="I133" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Live: BE enforces the distinct settings atom (Technician settings save -&gt; 403, Admin -&gt; 200) but does NOT enforce the WO-completion / review atoms (documented 'app blocks / backend allows' gap, draft TICKET 2). v1 pass = app-level restriction (Milos Round-2 ruling). Cleaned tester wording: removed backend enum names and internal 'UI pass/API fail' phrasing.</t>
+          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Live: BE enforces the distinct settings atom (Technician settings save -&gt; 403, Admin -&gt; 200) but does NOT enforce the WO-completion / review atoms (documented 'app blocks / backend allows' gap, draft TICKET 2). v1 pass = app-level restriction (Milos Round-2 ruling). Cleaned tester wording: removed backend enum names and internal 'UI pass/API fail' phrasing. | OPTIONAL REGRESSION EDIT 2026-07-24 (user-authorized): added the per-role Bulk Receive 'accept' backend-enforcement matrix (step 5 + expected 5) — POST /api/inventory/orders/accept returns 403 for the 4 No roles (Office, Sales Rep, Technician, Time Clock) and is allowed for the 7 Yes roles (Admin, Service Manager, Senior SA, Service Advisor, Foreman, Parts Manager, Parts Tech), matching §9.2 exactly (source: rerun2-2026-07-24 be-matrix-11roles.json; recommendation Finding 5). This is the single feature endpoint that genuinely BE-enforces per role — pure regression insurance, no status change.</t>
         </is>
       </c>
     </row>
@@ -7522,8 +7522,16 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="12" t="inlineStr"/>
-      <c r="B138" s="12" t="inlineStr"/>
+      <c r="A138" s="12" t="inlineStr">
+        <is>
+          <t>C30647</t>
+        </is>
+      </c>
+      <c r="B138" s="13" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30647</t>
+        </is>
+      </c>
       <c r="C138" s="12" t="inlineStr">
         <is>
           <t>SF-PERM-12</t>
@@ -7556,7 +7564,7 @@
       </c>
       <c r="I138" s="12" t="inlineStr">
         <is>
-          <t>[No TestRail ID in map — add after next TestRail sync] Authored 2026-07-24 as a corrective case for the SV-8516 coverage gap (no per-role part edit/cancel/return negative existed). LIVE re-verify 2026-07-24 on a CLEAN Time Clock template role (drift ruled out, Rule 26; role e35b0211 = 3/3 == template scheduleView/timesheetsView/workOrdersView, before &amp; after; impersonated via switch-user on henry.hess, restored to Technician after): the Time Clock part-row ⋮ menu shows ONLY 'Return' — no Edit / Cancel / Change Vendor items (sv8516-tc-menus.json: MENU=['Return']; Cancel/Change Vendor keywords = false). The original over-grant's Edit/Cancel/Change-Vendor controls have been removed from the Time Clock UI, so the front-end gating holds and this case PASSES. FLAG (Standing Rule 24): the same edit can still succeed through the API (POST /api/work-orders/part/change-request {id,line,work_order,description,quantity,part_source_type,part_category_id,cost} -&gt; HTTP 200 and the change persisted, confirmed live on Time Clock at 3 perms); per the product ruling 2026-07-24 this front-end-only gating is ACCEPTED for now and is NOT a defect. Editing an already-received part is blocked by state ('Part requests can't be modified once received') for Admin and Time Clock alike, not by permission. Deviation from spec wording noted only as a flag (not a bug): requirements §9.2 'Time Clock = No across every column' and §9.4 atom-collapse (the FE gate is a convenience, not a BE-enforceable boundary — so the residual API-possibility is spec-anticipated). Evidence: build/simple-flow/sv8183/ayesha-issues/reverify-2026-07-24/ (sv8516-tc-wo-lines.png, sv8516-tc-menus.json, LOG-SV-8516.md).</t>
+          <t>Authored 2026-07-24 as a corrective case for the SV-8516 coverage gap (no per-role part edit/cancel/return negative existed). LIVE re-verify 2026-07-24 on a CLEAN Time Clock template role (drift ruled out, Rule 26; role e35b0211 = 3/3 == template scheduleView/timesheetsView/workOrdersView, before &amp; after; impersonated via switch-user on henry.hess, restored to Technician after): the Time Clock part-row ⋮ menu shows ONLY 'Return' — no Edit / Cancel / Change Vendor items (sv8516-tc-menus.json: MENU=['Return']; Cancel/Change Vendor keywords = false). The original over-grant's Edit/Cancel/Change-Vendor controls have been removed from the Time Clock UI, so the front-end gating holds and this case PASSES. PASS per Rule 24 (FE gating is the pass criterion; API-possible accepted): the same edit can still succeed through the API (POST /api/work-orders/part/change-request {id,line,work_order,description,quantity,part_source_type,part_category_id,cost} -&gt; HTTP 200 and the change persisted, confirmed live on Time Clock at 3 perms); per the strengthened Standing Rule 24 (user ruling 2026-07-24) FE-blocks + BE/API-allows = a PASSED test case, so this front-end-only gating is ACCEPTED and is NOT a defect. Editing an already-received part is blocked by state ('Part requests can't be modified once received') for Admin and Time Clock alike, not by permission. Deviation from spec wording noted only as a flag (not a bug): requirements §9.2 'Time Clock = No across every column' and §9.4 atom-collapse (the FE gate is a convenience, not a BE-enforceable boundary — so the residual API-possibility is spec-anticipated). Evidence: build/simple-flow/sv8183/ayesha-issues/reverify-2026-07-24/ (sv8516-tc-wo-lines.png, sv8516-tc-menus.json, LOG-SV-8516.md). | OPTIONAL TRACEABILITY EDIT 2026-07-24 (user-authorized): appended a plain QA note to Expected recording the two accepted Rule-24 API behaviors — NEW-1 (a no-access role can still change a part's vendor via the API even though the control is FE-hidden; BE applies the See-Financial-Data gate rather than Vendor &amp; Order Mgmt: Create &amp; Edit per §9.1, a spec-conformance flag not a defect) and NEW-2 (part add/delete via POST /api/work-orders/part/make-request and /parts/delete is not BE-enforced for ANY role, §9.4 / SV-7864 atom-collapse). Both are FE-blocks + BE/API-allows = PASS per the strengthened Standing Rule 24; no status change (source: rerun-2026-07-24 / rerun2-2026-07-24 FINDINGS + recommendation Findings 1 &amp; 2).</t>
         </is>
       </c>
     </row>
@@ -8403,21 +8411,22 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B135" r:id="rId134"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B136" r:id="rId135"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B137" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B139" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B140" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B141" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B142" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B143" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B144" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B145" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B146" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B147" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B148" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B149" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B150" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B151" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B152" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B153" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B138" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B139" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B140" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B141" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B142" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B143" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B144" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B145" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B146" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B147" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B148" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B149" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B150" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B151" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B152" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B153" r:id="rId152"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10460,7 +10469,7 @@
       </c>
       <c r="I36" s="12" t="inlineStr">
         <is>
-          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Live: BE enforces the distinct settings atom (Technician settings save -&gt; 403, Admin -&gt; 200) but does NOT enforce the WO-completion / review atoms (documented 'app blocks / backend allows' gap, draft TICKET 2). v1 pass = app-level restriction (Milos Round-2 ruling). Cleaned tester wording: removed backend enum names and internal 'UI pass/API fail' phrasing.</t>
+          <t>Wording+VIU 2026-07-13: role expectation re-verified against the fresh live roles matrix (roles-matrix-2026-07-13.md; GET /api/roles/{id} + /api/auth/me/fe-permissions, no system-role drift). Live: BE enforces the distinct settings atom (Technician settings save -&gt; 403, Admin -&gt; 200) but does NOT enforce the WO-completion / review atoms (documented 'app blocks / backend allows' gap, draft TICKET 2). v1 pass = app-level restriction (Milos Round-2 ruling). Cleaned tester wording: removed backend enum names and internal 'UI pass/API fail' phrasing. | OPTIONAL REGRESSION EDIT 2026-07-24 (user-authorized): added the per-role Bulk Receive 'accept' backend-enforcement matrix (step 5 + expected 5) — POST /api/inventory/orders/accept returns 403 for the 4 No roles (Office, Sales Rep, Technician, Time Clock) and is allowed for the 7 Yes roles (Admin, Service Manager, Senior SA, Service Advisor, Foreman, Parts Manager, Parts Tech), matching §9.2 exactly (source: rerun2-2026-07-24 be-matrix-11roles.json; recommendation Finding 5). This is the single feature endpoint that genuinely BE-enforces per role — pure regression insurance, no status change.</t>
         </is>
       </c>
     </row>

</xml_diff>